<commit_message>
Tableau récap Halle : food cost retenu à 45 % (point mort, résultat, matière), la mesure du panel gardée en colonne et en hypothèse
generer.py prend --food 45 (défaut) ou --food mesure. Dans l'Excel, le food cost est une seule case (Récap!B31) reprise par tous les mois ; le tableau des hypothèses compare 45 %, 45 % avec les frais généraux d'octobre, le food cost ticket par ticket et celui du panel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfhpzegTMHxDopBcc2QwLH
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
+++ b/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
@@ -114,12 +114,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="142">
   <si>
     <t xml:space="preserve">Atelier by – Halle · tableau récap</t>
   </si>
   <si>
-    <t xml:space="preserve">Mars → septembre 2026 (7 mois pleins), lu le 13 octobre 2026. Hors TVA. En vert : liens vers « Mois par mois » ; en bleu : chiffres lus ; fond jaune : hypothèses à modifier ; en noir : calculs.</t>
+    <t xml:space="preserve">Mars → septembre 2026 (7 mois pleins), lu le 13 octobre 2026. Hors TVA. Food cost retenu : 45 % (case B31, appliquée à tous les mois). En vert : liens vers « Mois par mois » ; en bleu : chiffres lus ; fond jaune : hypothèses à modifier ; en noir : calculs.</t>
   </si>
   <si>
     <t xml:space="preserve">Ventes et clients</t>
@@ -206,7 +206,7 @@
     <t xml:space="preserve">Matière (food cost)</t>
   </si>
   <si>
-    <t xml:space="preserve">seuil réseau 32 % ; modèle du franchiseur 36 % + 2 % d’emballage</t>
+    <t xml:space="preserve">food cost retenu 45 % (case B31) ; mesuré 37,4 % au panel ; seuil réseau 32 %</t>
   </si>
   <si>
     <t xml:space="preserve">Main-d’œuvre encodée</t>
@@ -257,57 +257,60 @@
     <t xml:space="preserve">absentes du panel : à renseigner avec le franchisé</t>
   </si>
   <si>
+    <t xml:space="preserve">Food cost (hypothèse, s’applique à tous les mois)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hypothèse demandée ; mesuré 36,5 % par le panel (juillet → septembre), 43,9 % ticket par ticket (août-septembre)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charges fixes par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taux de marge brute (1 − food cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point mort, CA par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">charges fixes ÷ taux de marge brute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point mort, CA par jour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point mort, clients par jour au panier actuel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marge de sécurité (baisse de CA possible avant le point mort)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">face au CA moyen mars → septembre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultat encodé au CA actuel (par mois)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avec ces hypothèses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultat encodé à l’objectif (par mois)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point mort en plus pour 1 000 € de charges fixes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultat en plus pour 1 000 € de CA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le point mort selon les hypothèses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charges fixes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Food cost</t>
   </si>
   <si>
-    <t xml:space="preserve">mesure du panel ; recomposé ticket par ticket par le cockpit : 43,9 % (août-septembre)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charges fixes par mois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taux de marge brute (1 − food cost)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Point mort, CA par mois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">charges fixes ÷ taux de marge brute</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Point mort, CA par jour</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Point mort, clients par jour au panier actuel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marge de sécurité (baisse de CA possible avant le point mort)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">face au CA moyen mars → septembre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Résultat encodé au CA actuel (par mois)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avec ces hypothèses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Résultat encodé à l’objectif (par mois)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Point mort en plus pour 1 000 € de charges fixes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Résultat en plus pour 1 000 € de CA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le point mort selon les hypothèses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charges fixes</t>
-  </si>
-  <si>
     <t xml:space="preserve">Point mort / mois</t>
   </si>
   <si>
@@ -317,16 +320,16 @@
     <t xml:space="preserve">Marge de sécurité</t>
   </si>
   <si>
-    <t xml:space="preserve">Coûts encodés au panel (juillet → septembre)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frais généraux encodés en octobre (par jour × 31)</t>
+    <t xml:space="preserve">Food cost retenu, charges juillet → septembre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le même, avec les frais généraux d’octobre (par jour × 31)</t>
   </si>
   <si>
     <t xml:space="preserve">Food cost recomposé ticket par ticket (août-septembre)</t>
   </si>
   <si>
-    <t xml:space="preserve">Les deux à la fois</t>
+    <t xml:space="preserve">Food cost mesuré par le panel (juillet → septembre)</t>
   </si>
   <si>
     <t xml:space="preserve">À savoir</t>
@@ -371,7 +374,7 @@
     <t xml:space="preserve">CA par jour (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">Food cost (% CA)</t>
+    <t xml:space="preserve">Food cost retenu (% CA)</t>
   </si>
   <si>
     <t xml:space="preserve">Matière (€)</t>
@@ -399,6 +402,9 @@
   </si>
   <si>
     <t xml:space="preserve">Résultat (% CA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Food cost mesuré par le panel (% CA)</t>
   </si>
   <si>
     <t xml:space="preserve">Mars</t>
@@ -835,7 +841,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1409,19 +1415,19 @@
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">'Mois par mois'!K13</f>
-        <v>19309.8761742857</v>
+        <v>23221.5145714286</v>
       </c>
       <c r="C21" s="18" t="n">
         <f aca="false">IF('Mois par mois'!C13&gt;0,B21/'Mois par mois'!C13,0)</f>
-        <v>0.374197998657673</v>
+        <v>0.45</v>
       </c>
       <c r="D21" s="7" t="n">
         <f aca="false">'Mois par mois'!K14</f>
-        <v>18159.4685666667</v>
+        <v>22415.5875</v>
       </c>
       <c r="E21" s="18" t="n">
         <f aca="false">IF('Mois par mois'!C14&gt;0,D21/'Mois par mois'!C14,0)</f>
-        <v>0.364557067933196</v>
+        <v>0.45</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>30</v>
@@ -1481,19 +1487,19 @@
       </c>
       <c r="B24" s="20" t="n">
         <f aca="false">SUM(B21:B23)</f>
-        <v>40022.4047457143</v>
+        <v>43934.0431428571</v>
       </c>
       <c r="C24" s="21" t="n">
         <f aca="false">IF('Mois par mois'!C13&gt;0,B24/'Mois par mois'!C13,0)</f>
-        <v>0.775577410343888</v>
+        <v>0.851379411686214</v>
       </c>
       <c r="D24" s="20" t="n">
         <f aca="false">SUM(D21:D23)</f>
-        <v>39787.4885666667</v>
+        <v>44043.6075</v>
       </c>
       <c r="E24" s="21" t="n">
         <f aca="false">IF('Mois par mois'!C14&gt;0,D24/'Mois par mois'!C14,0)</f>
-        <v>0.798746401583273</v>
+        <v>0.884189333650077</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1502,19 +1508,19 @@
       </c>
       <c r="B25" s="23" t="n">
         <f aca="false">'Mois par mois'!C13-B24</f>
-        <v>11580.9609685714</v>
+        <v>7669.32257142857</v>
       </c>
       <c r="C25" s="24" t="n">
         <f aca="false">IF('Mois par mois'!C13&gt;0,B25/'Mois par mois'!C13,0)</f>
-        <v>0.224422589656112</v>
+        <v>0.148620588313786</v>
       </c>
       <c r="D25" s="23" t="n">
         <f aca="false">'Mois par mois'!C14-D24</f>
-        <v>10024.9281</v>
+        <v>5768.80916666667</v>
       </c>
       <c r="E25" s="24" t="n">
         <f aca="false">IF('Mois par mois'!C14&gt;0,D25/'Mois par mois'!C14,0)</f>
-        <v>0.201253598416727</v>
+        <v>0.115810666349923</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>37</v>
@@ -1574,8 +1580,7 @@
         <v>47</v>
       </c>
       <c r="B31" s="26" t="n">
-        <f aca="false">'Mois par mois'!J14</f>
-        <v>0.364557067933196</v>
+        <v>0.45</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>48</v>
@@ -1597,7 +1602,7 @@
       </c>
       <c r="B33" s="18" t="n">
         <f aca="false">1-B31</f>
-        <v>0.635442932066804</v>
+        <v>0.55</v>
       </c>
       <c r="F33" s="2"/>
     </row>
@@ -1607,7 +1612,7 @@
       </c>
       <c r="B34" s="28" t="n">
         <f aca="false">IF(B33&gt;0,B32/B33,0)</f>
-        <v>34036.1327643601</v>
+        <v>39323.6727272727</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>52</v>
@@ -1619,7 +1624,7 @@
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">B34/B13</f>
-        <v>1118.99614567759</v>
+        <v>1292.83307596513</v>
       </c>
       <c r="F35" s="2"/>
     </row>
@@ -1629,7 +1634,7 @@
       </c>
       <c r="B36" s="10" t="n">
         <f aca="false">IF(B9&gt;0,B35/B9,0)</f>
-        <v>91.846491749306</v>
+        <v>106.114916394961</v>
       </c>
       <c r="F36" s="2"/>
     </row>
@@ -1639,7 +1644,7 @@
       </c>
       <c r="B37" s="29" t="n">
         <f aca="false">IF(B5&gt;0,1-B34/B5,0)</f>
-        <v>0.34042804586024</v>
+        <v>0.237963024640727</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>56</v>
@@ -1651,7 +1656,7 @@
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">B5*B33-B32</f>
-        <v>11162.9740140013</v>
+        <v>6753.83114285714</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>58</v>
@@ -1663,7 +1668,7 @@
       </c>
       <c r="B39" s="8" t="n">
         <f aca="false">B12*B33-B32</f>
-        <v>17133.998856075</v>
+        <v>11921.98</v>
       </c>
       <c r="F39" s="2"/>
     </row>
@@ -1673,7 +1678,7 @@
       </c>
       <c r="B40" s="8" t="n">
         <f aca="false">IF(B33&gt;0,1000/B33,0)</f>
-        <v>1573.70544156886</v>
+        <v>1818.18181818182</v>
       </c>
       <c r="F40" s="2"/>
     </row>
@@ -1683,7 +1688,7 @@
       </c>
       <c r="B41" s="8" t="n">
         <f aca="false">1000*B33</f>
-        <v>635.442932066804</v>
+        <v>550</v>
       </c>
       <c r="F41" s="2"/>
     </row>
@@ -1695,21 +1700,21 @@
         <v>63</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B44" s="8" t="n">
         <f aca="false">'Mois par mois'!L14+'Mois par mois'!P14</f>
@@ -1717,24 +1722,24 @@
       </c>
       <c r="C44" s="30" t="n">
         <f aca="false">'Mois par mois'!J14</f>
-        <v>0.364557067933196</v>
+        <v>0.45</v>
       </c>
       <c r="D44" s="31" t="n">
         <f aca="false">IF(C44&lt;1,B44/(1-C44),0)</f>
-        <v>34036.1327643601</v>
+        <v>39323.6727272727</v>
       </c>
       <c r="E44" s="8" t="n">
         <f aca="false">D44/$B$13</f>
-        <v>1118.99614567759</v>
+        <v>1292.83307596513</v>
       </c>
       <c r="F44" s="32" t="n">
         <f aca="false">IF($B$5&gt;0,1-D44/$B$5,0)</f>
-        <v>0.34042804586024</v>
+        <v>0.237963024640727</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B45" s="8" t="n">
         <f aca="false">'Mois par mois'!L14+'Mois par mois'!P16*31</f>
@@ -1742,24 +1747,24 @@
       </c>
       <c r="C45" s="30" t="n">
         <f aca="false">'Mois par mois'!J14</f>
-        <v>0.364557067933196</v>
+        <v>0.45</v>
       </c>
       <c r="D45" s="31" t="n">
         <f aca="false">IF(C45&lt;1,B45/(1-C45),0)</f>
-        <v>37238.7702171273</v>
+        <v>43023.8424242424</v>
       </c>
       <c r="E45" s="8" t="n">
         <f aca="false">D45/$B$13</f>
-        <v>1224.28833590555</v>
+        <v>1414.48249066002</v>
       </c>
       <c r="F45" s="32" t="n">
         <f aca="false">IF($B$5&gt;0,1-D45/$B$5,0)</f>
-        <v>0.278365476715054</v>
+        <v>0.166258986623971</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B46" s="8" t="n">
         <f aca="false">B44</f>
@@ -1783,37 +1788,37 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B47" s="8" t="n">
-        <f aca="false">B45</f>
-        <v>23663.1133333333</v>
-      </c>
-      <c r="C47" s="18" t="n">
-        <f aca="false">C46</f>
-        <v>0.4386</v>
+        <f aca="false">B44</f>
+        <v>21628.02</v>
+      </c>
+      <c r="C47" s="30" t="n">
+        <f aca="false">'Mois par mois'!T14</f>
+        <v>0.364557067933196</v>
       </c>
       <c r="D47" s="31" t="n">
         <f aca="false">IF(C47&lt;1,B47/(1-C47),0)</f>
-        <v>42150.1840636504</v>
+        <v>34036.1327643601</v>
       </c>
       <c r="E47" s="8" t="n">
         <f aca="false">D47/$B$13</f>
-        <v>1385.75947606522</v>
+        <v>1118.99614567759</v>
       </c>
       <c r="F47" s="32" t="n">
         <f aca="false">IF($B$5&gt;0,1-D47/$B$5,0)</f>
-        <v>0.183189245890958</v>
+        <v>0.34042804586024</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="34" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B50" s="34"/>
       <c r="C50" s="34"/>
@@ -1823,7 +1828,7 @@
     </row>
     <row r="51" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="34" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B51" s="34"/>
       <c r="C51" s="34"/>
@@ -1833,7 +1838,7 @@
     </row>
     <row r="52" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="34" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B52" s="34"/>
       <c r="C52" s="34"/>
@@ -1863,85 +1868,88 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="2" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="R4" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="S4" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
+      </c>
+      <c r="T4" s="4" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B5" s="35" t="n">
         <v>31</v>
@@ -1971,12 +1979,13 @@
         <f aca="false">IF(B5&gt;0,F5/B5,0)</f>
         <v>140.032258064516</v>
       </c>
-      <c r="J5" s="33" t="n">
-        <v>0.398</v>
+      <c r="J5" s="30" t="n">
+        <f aca="false">Récap!$B$31</f>
+        <v>0.45</v>
       </c>
       <c r="K5" s="8" t="n">
         <f aca="false">C5*J5</f>
-        <v>19409.40132</v>
+        <v>21945.303</v>
       </c>
       <c r="L5" s="17" t="n">
         <v>6334</v>
@@ -2001,16 +2010,19 @@
       </c>
       <c r="R5" s="8" t="n">
         <f aca="false">C5-K5-L5-P5</f>
-        <v>13664.41868</v>
+        <v>11128.517</v>
       </c>
       <c r="S5" s="18" t="n">
         <f aca="false">IF(C5&gt;0,R5/C5,0)</f>
-        <v>0.280196104195964</v>
+        <v>0.228196104195964</v>
+      </c>
+      <c r="T5" s="33" t="n">
+        <v>0.398</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B6" s="35" t="n">
         <v>30</v>
@@ -2040,12 +2052,13 @@
         <f aca="false">IF(B6&gt;0,F6/B6,0)</f>
         <v>149.533333333333</v>
       </c>
-      <c r="J6" s="33" t="n">
-        <v>0.391</v>
+      <c r="J6" s="30" t="n">
+        <f aca="false">Récap!$B$31</f>
+        <v>0.45</v>
       </c>
       <c r="K6" s="8" t="n">
         <f aca="false">C6*J6</f>
-        <v>21830.14387</v>
+        <v>25124.2065</v>
       </c>
       <c r="L6" s="17" t="n">
         <v>5814.5</v>
@@ -2070,16 +2083,19 @@
       </c>
       <c r="R6" s="8" t="n">
         <f aca="false">C6-K6-L6-P6</f>
-        <v>18578.22613</v>
+        <v>15284.1635</v>
       </c>
       <c r="S6" s="18" t="n">
         <f aca="false">IF(C6&gt;0,R6/C6,0)</f>
-        <v>0.332754857690729</v>
+        <v>0.273754857690729</v>
+      </c>
+      <c r="T6" s="33" t="n">
+        <v>0.391</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B7" s="35" t="n">
         <v>31</v>
@@ -2109,12 +2125,13 @@
         <f aca="false">IF(B7&gt;0,F7/B7,0)</f>
         <v>153.41935483871</v>
       </c>
-      <c r="J7" s="33" t="n">
-        <v>0.372</v>
+      <c r="J7" s="30" t="n">
+        <f aca="false">Récap!$B$31</f>
+        <v>0.45</v>
       </c>
       <c r="K7" s="8" t="n">
         <f aca="false">C7*J7</f>
-        <v>22409.12004</v>
+        <v>27107.8065</v>
       </c>
       <c r="L7" s="17" t="n">
         <v>10080.5</v>
@@ -2139,16 +2156,19 @@
       </c>
       <c r="R7" s="8" t="n">
         <f aca="false">C7-K7-L7-P7</f>
-        <v>8216.22996</v>
+        <v>3517.5435</v>
       </c>
       <c r="S7" s="18" t="n">
         <f aca="false">IF(C7&gt;0,R7/C7,0)</f>
-        <v>0.136392573187358</v>
+        <v>0.0583925731873584</v>
+      </c>
+      <c r="T7" s="33" t="n">
+        <v>0.372</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B8" s="35" t="n">
         <v>30</v>
@@ -2178,12 +2198,13 @@
         <f aca="false">IF(B8&gt;0,F8/B8,0)</f>
         <v>127.033333333333</v>
       </c>
-      <c r="J8" s="33" t="n">
-        <v>0.363</v>
+      <c r="J8" s="30" t="n">
+        <f aca="false">Récap!$B$31</f>
+        <v>0.45</v>
       </c>
       <c r="K8" s="8" t="n">
         <f aca="false">C8*J8</f>
-        <v>17042.06229</v>
+        <v>21126.5235</v>
       </c>
       <c r="L8" s="17" t="n">
         <v>8714</v>
@@ -2208,16 +2229,19 @@
       </c>
       <c r="R8" s="8" t="n">
         <f aca="false">C8-K8-L8-P8</f>
-        <v>10533.06771</v>
+        <v>6448.6065</v>
       </c>
       <c r="S8" s="18" t="n">
         <f aca="false">IF(C8&gt;0,R8/C8,0)</f>
-        <v>0.224356859731323</v>
+        <v>0.137356859731323</v>
+      </c>
+      <c r="T8" s="33" t="n">
+        <v>0.363</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B9" s="35" t="n">
         <v>30</v>
@@ -2247,12 +2271,13 @@
         <f aca="false">IF(B9&gt;0,F9/B9,0)</f>
         <v>125.866666666667</v>
       </c>
-      <c r="J9" s="33" t="n">
-        <v>0.368</v>
+      <c r="J9" s="30" t="n">
+        <f aca="false">Récap!$B$31</f>
+        <v>0.45</v>
       </c>
       <c r="K9" s="8" t="n">
         <f aca="false">C9*J9</f>
-        <v>17015.0504</v>
+        <v>20806.4475</v>
       </c>
       <c r="L9" s="17" t="n">
         <v>8110.75</v>
@@ -2277,16 +2302,19 @@
       </c>
       <c r="R9" s="8" t="n">
         <f aca="false">C9-K9-L9-P9</f>
-        <v>8068.1196</v>
+        <v>4276.7225</v>
       </c>
       <c r="S9" s="18" t="n">
         <f aca="false">IF(C9&gt;0,R9/C9,0)</f>
-        <v>0.174496574679556</v>
+        <v>0.0924965746795555</v>
+      </c>
+      <c r="T9" s="33" t="n">
+        <v>0.368</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B10" s="35" t="n">
         <v>31</v>
@@ -2316,12 +2344,13 @@
         <f aca="false">IF(B10&gt;0,F10/B10,0)</f>
         <v>139.451612903226</v>
       </c>
-      <c r="J10" s="33" t="n">
-        <v>0.364</v>
+      <c r="J10" s="30" t="n">
+        <f aca="false">Récap!$B$31</f>
+        <v>0.45</v>
       </c>
       <c r="K10" s="8" t="n">
         <f aca="false">C10*J10</f>
-        <v>19055.7458</v>
+        <v>23557.9275</v>
       </c>
       <c r="L10" s="17" t="n">
         <v>8167.75</v>
@@ -2346,16 +2375,19 @@
       </c>
       <c r="R10" s="8" t="n">
         <f aca="false">C10-K10-L10-P10</f>
-        <v>12084.8242</v>
+        <v>7582.6425</v>
       </c>
       <c r="S10" s="18" t="n">
         <f aca="false">IF(C10&gt;0,R10/C10,0)</f>
-        <v>0.230842500470383</v>
+        <v>0.144842500470383</v>
+      </c>
+      <c r="T10" s="33" t="n">
+        <v>0.364</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B11" s="35" t="n">
         <v>30</v>
@@ -2385,12 +2417,13 @@
         <f aca="false">IF(B11&gt;0,F11/B11,0)</f>
         <v>138.533333333333</v>
       </c>
-      <c r="J11" s="33" t="n">
-        <v>0.362</v>
+      <c r="J11" s="30" t="n">
+        <f aca="false">Récap!$B$31</f>
+        <v>0.45</v>
       </c>
       <c r="K11" s="8" t="n">
         <f aca="false">C11*J11</f>
-        <v>18407.6095</v>
+        <v>22882.3875</v>
       </c>
       <c r="L11" s="17" t="n">
         <v>9477.5</v>
@@ -2415,16 +2448,19 @@
       </c>
       <c r="R11" s="8" t="n">
         <f aca="false">C11-K11-L11-P11</f>
-        <v>9921.8405</v>
+        <v>5447.0625</v>
       </c>
       <c r="S11" s="18" t="n">
         <f aca="false">IF(C11&gt;0,R11/C11,0)</f>
-        <v>0.195120733140281</v>
+        <v>0.107120733140281</v>
+      </c>
+      <c r="T11" s="33" t="n">
+        <v>0.362</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="37" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B12" s="38" t="n">
         <f aca="false">SUM(B5:B11)</f>
@@ -2460,11 +2496,11 @@
       </c>
       <c r="J12" s="42" t="n">
         <f aca="false">IF(C12&gt;0,K12/C12,0)</f>
-        <v>0.374197998657673</v>
+        <v>0.45</v>
       </c>
       <c r="K12" s="39" t="n">
         <f aca="false">SUM(K5:K11)</f>
-        <v>135169.13322</v>
+        <v>162550.602</v>
       </c>
       <c r="L12" s="39" t="n">
         <f aca="false">SUM(L5:L11)</f>
@@ -2492,16 +2528,20 @@
       </c>
       <c r="R12" s="39" t="n">
         <f aca="false">SUM(R5:R11)</f>
-        <v>81066.72678</v>
+        <v>53685.258</v>
       </c>
       <c r="S12" s="42" t="n">
         <f aca="false">IF(C12&gt;0,R12/C12,0)</f>
-        <v>0.224422589656112</v>
+        <v>0.148620588313786</v>
+      </c>
+      <c r="T12" s="42" t="n">
+        <f aca="false">IF(SUM(C5:C11)&gt;0,SUMPRODUCT(C5:C11,T5:T11)/SUM(C5:C11),0)</f>
+        <v>0.374197998657673</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="37" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B13" s="43" t="n">
         <f aca="false">AVERAGE(B5:B11)</f>
@@ -2537,11 +2577,11 @@
       </c>
       <c r="J13" s="42" t="n">
         <f aca="false">IF(C13&gt;0,K13/C13,0)</f>
-        <v>0.374197998657673</v>
+        <v>0.45</v>
       </c>
       <c r="K13" s="39" t="n">
         <f aca="false">AVERAGE(K5:K11)</f>
-        <v>19309.8761742857</v>
+        <v>23221.5145714286</v>
       </c>
       <c r="L13" s="39" t="n">
         <f aca="false">AVERAGE(L5:L11)</f>
@@ -2569,16 +2609,20 @@
       </c>
       <c r="R13" s="39" t="n">
         <f aca="false">AVERAGE(R5:R11)</f>
-        <v>11580.9609685714</v>
+        <v>7669.32257142857</v>
       </c>
       <c r="S13" s="42" t="n">
         <f aca="false">IF(C13&gt;0,R13/C13,0)</f>
-        <v>0.224422589656112</v>
+        <v>0.148620588313786</v>
+      </c>
+      <c r="T13" s="42" t="n">
+        <f aca="false">IF(SUM(C5:C11)&gt;0,SUMPRODUCT(C5:C11,T5:T11)/SUM(C5:C11),0)</f>
+        <v>0.374197998657673</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="37" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B14" s="43" t="n">
         <f aca="false">AVERAGE(B9:B11)</f>
@@ -2614,11 +2658,11 @@
       </c>
       <c r="J14" s="42" t="n">
         <f aca="false">IF(C14&gt;0,K14/C14,0)</f>
-        <v>0.364557067933196</v>
+        <v>0.45</v>
       </c>
       <c r="K14" s="39" t="n">
         <f aca="false">AVERAGE(K9:K11)</f>
-        <v>18159.4685666667</v>
+        <v>22415.5875</v>
       </c>
       <c r="L14" s="39" t="n">
         <f aca="false">AVERAGE(L9:L11)</f>
@@ -2646,16 +2690,20 @@
       </c>
       <c r="R14" s="39" t="n">
         <f aca="false">AVERAGE(R9:R11)</f>
-        <v>10024.9281</v>
+        <v>5768.80916666667</v>
       </c>
       <c r="S14" s="42" t="n">
         <f aca="false">IF(C14&gt;0,R14/C14,0)</f>
-        <v>0.201253598416727</v>
+        <v>0.115810666349923</v>
+      </c>
+      <c r="T14" s="42" t="n">
+        <f aca="false">IF(SUM(C9:C11)&gt;0,SUMPRODUCT(C9:C11,T9:T11)/SUM(C9:C11),0)</f>
+        <v>0.364557067933196</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="44" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B16" s="35" t="n">
         <v>12</v>
@@ -2689,7 +2737,7 @@
         <v>486.38</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2721,17 +2769,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C3" s="7" t="n">
         <f aca="false">'Mois par mois'!C13</f>
@@ -2740,30 +2788,30 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="45" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B5" s="45" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C5" s="45" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D5" s="45" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E5" s="45" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F5" s="45" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C6" s="33" t="n">
         <v>0</v>
@@ -2779,10 +2827,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C7" s="33" t="n">
         <v>0</v>
@@ -2798,10 +2846,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C8" s="33" t="n">
         <v>0.07</v>
@@ -2814,15 +2862,15 @@
         <v>3612.2356</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C9" s="33" t="n">
         <v>0.05</v>
@@ -2835,15 +2883,15 @@
         <v>2580.16828571429</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C10" s="33" t="n">
         <v>0.01</v>
@@ -2856,15 +2904,15 @@
         <v>516.033657142857</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C11" s="33" t="n">
         <v>0.01</v>
@@ -2877,15 +2925,15 @@
         <v>516.033657142857</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C12" s="33" t="n">
         <v>0.02</v>
@@ -2898,15 +2946,15 @@
         <v>1032.06731428571</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C13" s="33" t="n">
         <v>0.015</v>
@@ -2919,15 +2967,15 @@
         <v>774.050485714286</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C14" s="33" t="n">
         <v>0.015</v>
@@ -2940,15 +2988,15 @@
         <v>774.050485714286</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C15" s="33" t="n">
         <v>0.05</v>
@@ -2961,15 +3009,15 @@
         <v>2580.16828571429</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C16" s="33" t="n">
         <v>0.015</v>
@@ -2982,12 +3030,12 @@
         <v>774.050485714286</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="19" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C17" s="21" t="n">
         <f aca="false">SUM(C6:C16)</f>
@@ -3000,7 +3048,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E19" s="7" t="n">
         <f aca="false">'Mois par mois'!P14</f>
@@ -3009,7 +3057,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tableau récap Halle : main-d'œuvre retenue à 2 650 € par semaine (point mort, résultat, mois par mois), la main-d'œuvre encodée au panel gardée en colonne
generer.py prend --mo 2650 (défaut) ou --mo encodee ; la semaine est comptée au prorata des jours du mois. Dans l'Excel, la main-d'œuvre par semaine est une seule case (Récap!C28), reprise par tous les mois et par le point mort.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfhpzegTMHxDopBcc2QwLH
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
+++ b/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
@@ -63,6 +63,18 @@
         </r>
       </text>
     </comment>
+    <comment ref="C28" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Main-d’œuvre par semaine, montant communiqué le 13 octobre 2026 ; remplace la main-d’œuvre encodée au panel, dans tous les mois (feuille « Mois par mois », colonne L) et dans le point mort.</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="C46" authorId="0">
       <text>
         <r>
@@ -97,6 +109,18 @@
         </r>
       </text>
     </comment>
+    <comment ref="L5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Main-d’œuvre par semaine (Récap!C28) × jours du mois ÷ 7.</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="P16" authorId="0">
       <text>
         <r>
@@ -114,7 +138,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="144">
   <si>
     <t xml:space="preserve">Atelier by – Halle · tableau récap</t>
   </si>
@@ -209,10 +233,10 @@
     <t xml:space="preserve">food cost retenu 45 % (case B31) ; mesuré 37,4 % au panel ; seuil réseau 32 %</t>
   </si>
   <si>
-    <t xml:space="preserve">Main-d’œuvre encodée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">seuil réseau 33 % ; le franchisé est à 0 €/h au panel</t>
+    <t xml:space="preserve">Main-d’œuvre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 650 € par semaine (case C28) ; encodée au panel : 8 100 € par mois ; seuil réseau 33 %</t>
   </si>
   <si>
     <t xml:space="preserve">Frais généraux encodés</t>
@@ -224,10 +248,10 @@
     <t xml:space="preserve">Total des coûts</t>
   </si>
   <si>
-    <t xml:space="preserve">Résultat opérationnel encodé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avant rémunération du gérant, charges financières et impôts</t>
+    <t xml:space="preserve">Résultat opérationnel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avant charges financières et impôts</t>
   </si>
   <si>
     <t xml:space="preserve">Le point mort (structure de coûts juillet → septembre)</t>
@@ -236,13 +260,16 @@
     <t xml:space="preserve">Valeur</t>
   </si>
   <si>
+    <t xml:space="preserve">€ par semaine</t>
+  </si>
+  <si>
     <t xml:space="preserve">Comment</t>
   </si>
   <si>
-    <t xml:space="preserve">Main-d’œuvre par mois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hypothèse : remplacer pour tester</t>
+    <t xml:space="preserve">Main-d’œuvre par mois (la semaine en C, × 365/12 ÷ 7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hypothèse : 2 650 € par semaine (case C28) ; encodée au panel : 8 585 € par mois en juillet → septembre</t>
   </si>
   <si>
     <t xml:space="preserve">Frais généraux par mois</t>
@@ -287,13 +314,13 @@
     <t xml:space="preserve">face au CA moyen mars → septembre</t>
   </si>
   <si>
-    <t xml:space="preserve">Résultat encodé au CA actuel (par mois)</t>
+    <t xml:space="preserve">Résultat au CA actuel (par mois)</t>
   </si>
   <si>
     <t xml:space="preserve">avec ces hypothèses</t>
   </si>
   <si>
-    <t xml:space="preserve">Résultat encodé à l’objectif (par mois)</t>
+    <t xml:space="preserve">Résultat à l’objectif (par mois)</t>
   </si>
   <si>
     <t xml:space="preserve">Point mort en plus pour 1 000 € de charges fixes</t>
@@ -335,7 +362,7 @@
     <t xml:space="preserve">À savoir</t>
   </si>
   <si>
-    <t xml:space="preserve">Main-d’œuvre encodée = heures planifiées × taux horaire du panel (8 à 16 €/h selon les mois) : le franchisé y compte pour 0 €/h et les charges sociales n’y sont vraisemblablement pas toutes. Résultat et point mort sont donc avant la rémunération du gérant : l’ajouter en « Autres charges fixes ».</t>
+    <t xml:space="preserve">Main-d’œuvre retenue : 2 650 € par semaine (case C28), au prorata des jours de chaque mois. Elle remplace la main-d’œuvre encodée au panel (8 100 € par mois en moyenne, colonne U de « Mois par mois »). Si la rémunération du gérant n’y est pas, l’ajouter en « Autres charges fixes ».</t>
   </si>
   <si>
     <t xml:space="preserve">Les frais généraux encodés sont un montant mensuel saisi au panel, sans détail ; la feuille « Modèle de charges » donne le contenu attendu par le franchiseur (loyer, énergie, redevances, amortissements…).</t>
@@ -380,7 +407,7 @@
     <t xml:space="preserve">Matière (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">Main-d’œuvre encodée (€)</t>
+    <t xml:space="preserve">Main-d’œuvre retenue (€)</t>
   </si>
   <si>
     <t xml:space="preserve">Main-d’œuvre (% CA)</t>
@@ -389,7 +416,7 @@
     <t xml:space="preserve">Heures planifiées</t>
   </si>
   <si>
-    <t xml:space="preserve">Coût horaire encodé (€/h)</t>
+    <t xml:space="preserve">Coût horaire retenu (€/h)</t>
   </si>
   <si>
     <t xml:space="preserve">Frais généraux encodés (€)</t>
@@ -405,6 +432,9 @@
   </si>
   <si>
     <t xml:space="preserve">Food cost mesuré par le panel (% CA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main-d’œuvre encodée au panel (€)</t>
   </si>
   <si>
     <t xml:space="preserve">Mars</t>
@@ -736,7 +766,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -835,6 +865,10 @@
     </xf>
     <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -1439,19 +1473,19 @@
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">'Mois par mois'!L13</f>
-        <v>8099.85714285714</v>
+        <v>11573.4693877551</v>
       </c>
       <c r="C22" s="18" t="n">
         <f aca="false">IF('Mois par mois'!C13&gt;0,B22/'Mois par mois'!C13,0)</f>
-        <v>0.156963737359767</v>
+        <v>0.224277413450789</v>
       </c>
       <c r="D22" s="7" t="n">
         <f aca="false">'Mois par mois'!L14</f>
-        <v>8585.33333333333</v>
+        <v>11609.5238095238</v>
       </c>
       <c r="E22" s="18" t="n">
         <f aca="false">IF('Mois par mois'!C14&gt;0,D22/'Mois par mois'!C14,0)</f>
-        <v>0.172353278717321</v>
+        <v>0.233064857848839</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>32</v>
@@ -1487,19 +1521,19 @@
       </c>
       <c r="B24" s="20" t="n">
         <f aca="false">SUM(B21:B23)</f>
-        <v>43934.0431428571</v>
+        <v>47407.6553877551</v>
       </c>
       <c r="C24" s="21" t="n">
         <f aca="false">IF('Mois par mois'!C13&gt;0,B24/'Mois par mois'!C13,0)</f>
-        <v>0.851379411686214</v>
+        <v>0.918693087777236</v>
       </c>
       <c r="D24" s="20" t="n">
         <f aca="false">SUM(D21:D23)</f>
-        <v>44043.6075</v>
+        <v>47067.7979761905</v>
       </c>
       <c r="E24" s="21" t="n">
         <f aca="false">IF('Mois par mois'!C14&gt;0,D24/'Mois par mois'!C14,0)</f>
-        <v>0.884189333650077</v>
+        <v>0.944900912781595</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1508,19 +1542,19 @@
       </c>
       <c r="B25" s="23" t="n">
         <f aca="false">'Mois par mois'!C13-B24</f>
-        <v>7669.32257142857</v>
+        <v>4195.71032653061</v>
       </c>
       <c r="C25" s="24" t="n">
         <f aca="false">IF('Mois par mois'!C13&gt;0,B25/'Mois par mois'!C13,0)</f>
-        <v>0.148620588313786</v>
+        <v>0.0813069122227639</v>
       </c>
       <c r="D25" s="23" t="n">
         <f aca="false">'Mois par mois'!C14-D24</f>
-        <v>5768.80916666667</v>
+        <v>2744.61869047619</v>
       </c>
       <c r="E25" s="24" t="n">
         <f aca="false">IF('Mois par mois'!C14&gt;0,D25/'Mois par mois'!C14,0)</f>
-        <v>0.115810666349923</v>
+        <v>0.0550990872184048</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>37</v>
@@ -1533,72 +1567,77 @@
       <c r="B27" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="4"/>
+      <c r="C27" s="25" t="s">
+        <v>40</v>
+      </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
       <c r="F27" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B28" s="25" t="n">
-        <f aca="false">'Mois par mois'!L14</f>
-        <v>8585.33333333333</v>
+        <v>42</v>
+      </c>
+      <c r="B28" s="8" t="n">
+        <f aca="false">C28*B13/7</f>
+        <v>11514.880952381</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>2650</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B29" s="25" t="n">
+        <v>44</v>
+      </c>
+      <c r="B29" s="26" t="n">
         <f aca="false">'Mois par mois'!P14</f>
         <v>13042.6866666667</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B30" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B31" s="26" t="n">
+        <v>48</v>
+      </c>
+      <c r="B31" s="27" t="n">
         <v>0.45</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B32" s="20" t="n">
         <f aca="false">SUM(B28:B30)</f>
-        <v>21628.02</v>
+        <v>24557.5676190476</v>
       </c>
       <c r="F32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B33" s="18" t="n">
         <f aca="false">1-B31</f>
@@ -1607,74 +1646,74 @@
       <c r="F33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="B34" s="28" t="n">
+      <c r="A34" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="29" t="n">
         <f aca="false">IF(B33&gt;0,B32/B33,0)</f>
-        <v>39323.6727272727</v>
+        <v>44650.1229437229</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">B34/B13</f>
-        <v>1292.83307596513</v>
+        <v>1467.94924746486</v>
       </c>
       <c r="F35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B36" s="10" t="n">
         <f aca="false">IF(B9&gt;0,B35/B9,0)</f>
-        <v>106.114916394961</v>
+        <v>120.48834034548</v>
       </c>
       <c r="F36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B37" s="29" t="n">
+        <v>56</v>
+      </c>
+      <c r="B37" s="30" t="n">
         <f aca="false">IF(B5&gt;0,1-B34/B5,0)</f>
-        <v>0.237963024640727</v>
+        <v>0.134743977923088</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">B5*B33-B32</f>
-        <v>6753.83114285714</v>
+        <v>3824.28352380953</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B39" s="8" t="n">
         <f aca="false">B12*B33-B32</f>
-        <v>11921.98</v>
+        <v>8992.43238095238</v>
       </c>
       <c r="F39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B40" s="8" t="n">
         <f aca="false">IF(B33&gt;0,1000/B33,0)</f>
@@ -1684,7 +1723,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B41" s="8" t="n">
         <f aca="false">1000*B33</f>
@@ -1694,157 +1733,157 @@
     </row>
     <row r="43" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B44" s="8" t="n">
-        <f aca="false">'Mois par mois'!L14+'Mois par mois'!P14</f>
-        <v>21628.02</v>
-      </c>
-      <c r="C44" s="30" t="n">
+        <f aca="false">$B$28+'Mois par mois'!P14</f>
+        <v>24557.5676190476</v>
+      </c>
+      <c r="C44" s="31" t="n">
         <f aca="false">'Mois par mois'!J14</f>
         <v>0.45</v>
       </c>
-      <c r="D44" s="31" t="n">
+      <c r="D44" s="32" t="n">
         <f aca="false">IF(C44&lt;1,B44/(1-C44),0)</f>
-        <v>39323.6727272727</v>
+        <v>44650.1229437229</v>
       </c>
       <c r="E44" s="8" t="n">
         <f aca="false">D44/$B$13</f>
-        <v>1292.83307596513</v>
-      </c>
-      <c r="F44" s="32" t="n">
+        <v>1467.94924746486</v>
+      </c>
+      <c r="F44" s="33" t="n">
         <f aca="false">IF($B$5&gt;0,1-D44/$B$5,0)</f>
-        <v>0.237963024640727</v>
+        <v>0.134743977923088</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B45" s="8" t="n">
-        <f aca="false">'Mois par mois'!L14+'Mois par mois'!P16*31</f>
-        <v>23663.1133333333</v>
-      </c>
-      <c r="C45" s="30" t="n">
+        <f aca="false">$B$28+'Mois par mois'!P16*31</f>
+        <v>26592.660952381</v>
+      </c>
+      <c r="C45" s="31" t="n">
         <f aca="false">'Mois par mois'!J14</f>
         <v>0.45</v>
       </c>
-      <c r="D45" s="31" t="n">
+      <c r="D45" s="32" t="n">
         <f aca="false">IF(C45&lt;1,B45/(1-C45),0)</f>
-        <v>43023.8424242424</v>
+        <v>48350.2926406926</v>
       </c>
       <c r="E45" s="8" t="n">
         <f aca="false">D45/$B$13</f>
-        <v>1414.48249066002</v>
-      </c>
-      <c r="F45" s="32" t="n">
+        <v>1589.59866215976</v>
+      </c>
+      <c r="F45" s="33" t="n">
         <f aca="false">IF($B$5&gt;0,1-D45/$B$5,0)</f>
-        <v>0.166258986623971</v>
+        <v>0.0630399399063326</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B46" s="8" t="n">
         <f aca="false">B44</f>
-        <v>21628.02</v>
-      </c>
-      <c r="C46" s="33" t="n">
+        <v>24557.5676190476</v>
+      </c>
+      <c r="C46" s="34" t="n">
         <v>0.4386</v>
       </c>
-      <c r="D46" s="31" t="n">
+      <c r="D46" s="32" t="n">
         <f aca="false">IF(C46&lt;1,B46/(1-C46),0)</f>
-        <v>38525.1514071963</v>
+        <v>43743.4407179331</v>
       </c>
       <c r="E46" s="8" t="n">
         <f aca="false">D46/$B$13</f>
-        <v>1266.58032023659</v>
-      </c>
-      <c r="F46" s="32" t="n">
+        <v>1438.14051675396</v>
+      </c>
+      <c r="F46" s="33" t="n">
         <f aca="false">IF($B$5&gt;0,1-D46/$B$5,0)</f>
-        <v>0.253437234685428</v>
+        <v>0.152314192835231</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B47" s="8" t="n">
         <f aca="false">B44</f>
-        <v>21628.02</v>
-      </c>
-      <c r="C47" s="30" t="n">
+        <v>24557.5676190476</v>
+      </c>
+      <c r="C47" s="31" t="n">
         <f aca="false">'Mois par mois'!T14</f>
         <v>0.364557067933196</v>
       </c>
-      <c r="D47" s="31" t="n">
+      <c r="D47" s="32" t="n">
         <f aca="false">IF(C47&lt;1,B47/(1-C47),0)</f>
-        <v>34036.1327643601</v>
+        <v>38646.3777937904</v>
       </c>
       <c r="E47" s="8" t="n">
         <f aca="false">D47/$B$13</f>
-        <v>1118.99614567759</v>
-      </c>
-      <c r="F47" s="32" t="n">
+        <v>1270.5658452753</v>
+      </c>
+      <c r="F47" s="33" t="n">
         <f aca="false">IF($B$5&gt;0,1-D47/$B$5,0)</f>
-        <v>0.34042804586024</v>
+        <v>0.251088039339037</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="B50" s="34"/>
-      <c r="C50" s="34"/>
-      <c r="D50" s="34"/>
-      <c r="E50" s="34"/>
-      <c r="F50" s="34"/>
+      <c r="A50" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="B50" s="35"/>
+      <c r="C50" s="35"/>
+      <c r="D50" s="35"/>
+      <c r="E50" s="35"/>
+      <c r="F50" s="35"/>
     </row>
     <row r="51" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="34" t="s">
-        <v>74</v>
-      </c>
-      <c r="B51" s="34"/>
-      <c r="C51" s="34"/>
-      <c r="D51" s="34"/>
-      <c r="E51" s="34"/>
-      <c r="F51" s="34"/>
+      <c r="A51" s="35" t="s">
+        <v>75</v>
+      </c>
+      <c r="B51" s="35"/>
+      <c r="C51" s="35"/>
+      <c r="D51" s="35"/>
+      <c r="E51" s="35"/>
+      <c r="F51" s="35"/>
     </row>
     <row r="52" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="34" t="s">
-        <v>75</v>
-      </c>
-      <c r="B52" s="34"/>
-      <c r="C52" s="34"/>
-      <c r="D52" s="34"/>
-      <c r="E52" s="34"/>
-      <c r="F52" s="34"/>
+      <c r="A52" s="35" t="s">
+        <v>76</v>
+      </c>
+      <c r="B52" s="35"/>
+      <c r="C52" s="35"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="35"/>
+      <c r="F52" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1868,90 +1907,93 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="2" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="R4" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S4" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
+      </c>
+      <c r="U4" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="B5" s="35" t="n">
+        <v>99</v>
+      </c>
+      <c r="B5" s="36" t="n">
         <v>31</v>
       </c>
       <c r="C5" s="17" t="n">
@@ -1960,11 +2002,11 @@
       <c r="D5" s="17" t="n">
         <v>62000</v>
       </c>
-      <c r="E5" s="29" t="n">
+      <c r="E5" s="30" t="n">
         <f aca="false">IF(D5&gt;0,C5/D5,0)</f>
         <v>0.78657</v>
       </c>
-      <c r="F5" s="35" t="n">
+      <c r="F5" s="36" t="n">
         <v>4341</v>
       </c>
       <c r="G5" s="12" t="n">
@@ -1979,7 +2021,7 @@
         <f aca="false">IF(B5&gt;0,F5/B5,0)</f>
         <v>140.032258064516</v>
       </c>
-      <c r="J5" s="30" t="n">
+      <c r="J5" s="31" t="n">
         <f aca="false">Récap!$B$31</f>
         <v>0.45</v>
       </c>
@@ -1987,19 +2029,20 @@
         <f aca="false">C5*J5</f>
         <v>21945.303</v>
       </c>
-      <c r="L5" s="17" t="n">
-        <v>6334</v>
+      <c r="L5" s="7" t="n">
+        <f aca="false">Récap!$C$28*31/7</f>
+        <v>11735.7142857143</v>
       </c>
       <c r="M5" s="18" t="n">
         <f aca="false">IF(C5&gt;0,L5/C5,0)</f>
-        <v>0.129882007097373</v>
-      </c>
-      <c r="N5" s="36" t="n">
+        <v>0.240647004444251</v>
+      </c>
+      <c r="N5" s="37" t="n">
         <v>801.5</v>
       </c>
       <c r="O5" s="12" t="n">
         <f aca="false">IF(N5&gt;0,L5/N5,0)</f>
-        <v>7.90268247036806</v>
+        <v>14.6421887532306</v>
       </c>
       <c r="P5" s="17" t="n">
         <v>9359.52</v>
@@ -2010,21 +2053,24 @@
       </c>
       <c r="R5" s="8" t="n">
         <f aca="false">C5-K5-L5-P5</f>
-        <v>11128.517</v>
+        <v>5726.80271428571</v>
       </c>
       <c r="S5" s="18" t="n">
         <f aca="false">IF(C5&gt;0,R5/C5,0)</f>
-        <v>0.228196104195964</v>
-      </c>
-      <c r="T5" s="33" t="n">
+        <v>0.117431106849086</v>
+      </c>
+      <c r="T5" s="34" t="n">
         <v>0.398</v>
+      </c>
+      <c r="U5" s="17" t="n">
+        <v>6334</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B6" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="B6" s="36" t="n">
         <v>30</v>
       </c>
       <c r="C6" s="17" t="n">
@@ -2033,11 +2079,11 @@
       <c r="D6" s="17" t="n">
         <v>62000</v>
       </c>
-      <c r="E6" s="29" t="n">
+      <c r="E6" s="30" t="n">
         <f aca="false">IF(D6&gt;0,C6/D6,0)</f>
         <v>0.900509193548387</v>
       </c>
-      <c r="F6" s="35" t="n">
+      <c r="F6" s="36" t="n">
         <v>4486</v>
       </c>
       <c r="G6" s="12" t="n">
@@ -2052,7 +2098,7 @@
         <f aca="false">IF(B6&gt;0,F6/B6,0)</f>
         <v>149.533333333333</v>
       </c>
-      <c r="J6" s="30" t="n">
+      <c r="J6" s="31" t="n">
         <f aca="false">Récap!$B$31</f>
         <v>0.45</v>
       </c>
@@ -2060,19 +2106,20 @@
         <f aca="false">C6*J6</f>
         <v>25124.2065</v>
       </c>
-      <c r="L6" s="17" t="n">
-        <v>5814.5</v>
+      <c r="L6" s="7" t="n">
+        <f aca="false">Récap!$C$28*30/7</f>
+        <v>11357.1428571429</v>
       </c>
       <c r="M6" s="18" t="n">
         <f aca="false">IF(C6&gt;0,L6/C6,0)</f>
-        <v>0.104143587579572</v>
-      </c>
-      <c r="N6" s="36" t="n">
+        <v>0.203417938222817</v>
+      </c>
+      <c r="N6" s="37" t="n">
         <v>758</v>
       </c>
       <c r="O6" s="12" t="n">
         <f aca="false">IF(N6&gt;0,L6/N6,0)</f>
-        <v>7.67084432717678</v>
+        <v>14.9830380701093</v>
       </c>
       <c r="P6" s="17" t="n">
         <v>9608.7</v>
@@ -2083,21 +2130,24 @@
       </c>
       <c r="R6" s="8" t="n">
         <f aca="false">C6-K6-L6-P6</f>
-        <v>15284.1635</v>
+        <v>9741.52064285714</v>
       </c>
       <c r="S6" s="18" t="n">
         <f aca="false">IF(C6&gt;0,R6/C6,0)</f>
-        <v>0.273754857690729</v>
-      </c>
-      <c r="T6" s="33" t="n">
+        <v>0.174480507047485</v>
+      </c>
+      <c r="T6" s="34" t="n">
         <v>0.391</v>
+      </c>
+      <c r="U6" s="17" t="n">
+        <v>5814.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B7" s="35" t="n">
+        <v>101</v>
+      </c>
+      <c r="B7" s="36" t="n">
         <v>31</v>
       </c>
       <c r="C7" s="17" t="n">
@@ -2106,11 +2156,11 @@
       <c r="D7" s="17" t="n">
         <v>62000</v>
       </c>
-      <c r="E7" s="29" t="n">
+      <c r="E7" s="30" t="n">
         <f aca="false">IF(D7&gt;0,C7/D7,0)</f>
         <v>0.971605967741936</v>
       </c>
-      <c r="F7" s="35" t="n">
+      <c r="F7" s="36" t="n">
         <v>4756</v>
       </c>
       <c r="G7" s="12" t="n">
@@ -2125,7 +2175,7 @@
         <f aca="false">IF(B7&gt;0,F7/B7,0)</f>
         <v>153.41935483871</v>
       </c>
-      <c r="J7" s="30" t="n">
+      <c r="J7" s="31" t="n">
         <f aca="false">Récap!$B$31</f>
         <v>0.45</v>
       </c>
@@ -2133,19 +2183,20 @@
         <f aca="false">C7*J7</f>
         <v>27107.8065</v>
       </c>
-      <c r="L7" s="17" t="n">
-        <v>10080.5</v>
+      <c r="L7" s="7" t="n">
+        <f aca="false">Récap!$C$28*31/7</f>
+        <v>11735.7142857143</v>
       </c>
       <c r="M7" s="18" t="n">
         <f aca="false">IF(C7&gt;0,L7/C7,0)</f>
-        <v>0.167340171916898</v>
-      </c>
-      <c r="N7" s="36" t="n">
+        <v>0.194817364827045</v>
+      </c>
+      <c r="N7" s="37" t="n">
         <v>628</v>
       </c>
       <c r="O7" s="12" t="n">
         <f aca="false">IF(N7&gt;0,L7/N7,0)</f>
-        <v>16.0517515923567</v>
+        <v>18.6874431301183</v>
       </c>
       <c r="P7" s="17" t="n">
         <v>19533.72</v>
@@ -2156,21 +2207,24 @@
       </c>
       <c r="R7" s="8" t="n">
         <f aca="false">C7-K7-L7-P7</f>
-        <v>3517.5435</v>
+        <v>1862.32921428571</v>
       </c>
       <c r="S7" s="18" t="n">
         <f aca="false">IF(C7&gt;0,R7/C7,0)</f>
-        <v>0.0583925731873584</v>
-      </c>
-      <c r="T7" s="33" t="n">
+        <v>0.0309153802772117</v>
+      </c>
+      <c r="T7" s="34" t="n">
         <v>0.372</v>
+      </c>
+      <c r="U7" s="17" t="n">
+        <v>10080.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B8" s="35" t="n">
+        <v>102</v>
+      </c>
+      <c r="B8" s="36" t="n">
         <v>30</v>
       </c>
       <c r="C8" s="17" t="n">
@@ -2179,11 +2233,11 @@
       <c r="D8" s="17" t="n">
         <v>62000</v>
       </c>
-      <c r="E8" s="29" t="n">
+      <c r="E8" s="30" t="n">
         <f aca="false">IF(D8&gt;0,C8/D8,0)</f>
         <v>0.757223064516129</v>
       </c>
-      <c r="F8" s="35" t="n">
+      <c r="F8" s="36" t="n">
         <v>3811</v>
       </c>
       <c r="G8" s="12" t="n">
@@ -2198,7 +2252,7 @@
         <f aca="false">IF(B8&gt;0,F8/B8,0)</f>
         <v>127.033333333333</v>
       </c>
-      <c r="J8" s="30" t="n">
+      <c r="J8" s="31" t="n">
         <f aca="false">Récap!$B$31</f>
         <v>0.45</v>
       </c>
@@ -2206,19 +2260,20 @@
         <f aca="false">C8*J8</f>
         <v>21126.5235</v>
       </c>
-      <c r="L8" s="17" t="n">
-        <v>8714</v>
+      <c r="L8" s="7" t="n">
+        <f aca="false">Récap!$C$28*30/7</f>
+        <v>11357.1428571429</v>
       </c>
       <c r="M8" s="18" t="n">
         <f aca="false">IF(C8&gt;0,L8/C8,0)</f>
-        <v>0.185610282732983</v>
-      </c>
-      <c r="N8" s="36" t="n">
+        <v>0.241909857327652</v>
+      </c>
+      <c r="N8" s="37" t="n">
         <v>617.5</v>
       </c>
       <c r="O8" s="12" t="n">
         <f aca="false">IF(N8&gt;0,L8/N8,0)</f>
-        <v>14.1117408906883</v>
+        <v>18.3921341816079</v>
       </c>
       <c r="P8" s="17" t="n">
         <v>10658.7</v>
@@ -2229,21 +2284,24 @@
       </c>
       <c r="R8" s="8" t="n">
         <f aca="false">C8-K8-L8-P8</f>
-        <v>6448.6065</v>
+        <v>3805.46364285714</v>
       </c>
       <c r="S8" s="18" t="n">
         <f aca="false">IF(C8&gt;0,R8/C8,0)</f>
-        <v>0.137356859731323</v>
-      </c>
-      <c r="T8" s="33" t="n">
+        <v>0.0810572851366536</v>
+      </c>
+      <c r="T8" s="34" t="n">
         <v>0.363</v>
+      </c>
+      <c r="U8" s="17" t="n">
+        <v>8714</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B9" s="35" t="n">
+        <v>103</v>
+      </c>
+      <c r="B9" s="36" t="n">
         <v>30</v>
       </c>
       <c r="C9" s="17" t="n">
@@ -2252,11 +2310,11 @@
       <c r="D9" s="17" t="n">
         <v>62000</v>
       </c>
-      <c r="E9" s="29" t="n">
+      <c r="E9" s="30" t="n">
         <f aca="false">IF(D9&gt;0,C9/D9,0)</f>
         <v>0.745750806451613</v>
       </c>
-      <c r="F9" s="35" t="n">
+      <c r="F9" s="36" t="n">
         <v>3776</v>
       </c>
       <c r="G9" s="12" t="n">
@@ -2271,7 +2329,7 @@
         <f aca="false">IF(B9&gt;0,F9/B9,0)</f>
         <v>125.866666666667</v>
       </c>
-      <c r="J9" s="30" t="n">
+      <c r="J9" s="31" t="n">
         <f aca="false">Récap!$B$31</f>
         <v>0.45</v>
       </c>
@@ -2279,19 +2337,20 @@
         <f aca="false">C9*J9</f>
         <v>20806.4475</v>
       </c>
-      <c r="L9" s="17" t="n">
-        <v>8110.75</v>
+      <c r="L9" s="7" t="n">
+        <f aca="false">Récap!$C$28*31/7</f>
+        <v>11735.7142857143</v>
       </c>
       <c r="M9" s="18" t="n">
         <f aca="false">IF(C9&gt;0,L9/C9,0)</f>
-        <v>0.175418581187394</v>
-      </c>
-      <c r="N9" s="36" t="n">
+        <v>0.253818987050597</v>
+      </c>
+      <c r="N9" s="37" t="n">
         <v>675.5</v>
       </c>
       <c r="O9" s="12" t="n">
         <f aca="false">IF(N9&gt;0,L9/N9,0)</f>
-        <v>12.0070318282754</v>
+        <v>17.3733742201544</v>
       </c>
       <c r="P9" s="17" t="n">
         <v>13042.63</v>
@@ -2302,21 +2361,24 @@
       </c>
       <c r="R9" s="8" t="n">
         <f aca="false">C9-K9-L9-P9</f>
-        <v>4276.7225</v>
+        <v>651.758214285715</v>
       </c>
       <c r="S9" s="18" t="n">
         <f aca="false">IF(C9&gt;0,R9/C9,0)</f>
-        <v>0.0924965746795555</v>
-      </c>
-      <c r="T9" s="33" t="n">
+        <v>0.0140961688163523</v>
+      </c>
+      <c r="T9" s="34" t="n">
         <v>0.368</v>
+      </c>
+      <c r="U9" s="17" t="n">
+        <v>8110.75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B10" s="35" t="n">
+        <v>104</v>
+      </c>
+      <c r="B10" s="36" t="n">
         <v>31</v>
       </c>
       <c r="C10" s="17" t="n">
@@ -2325,11 +2387,11 @@
       <c r="D10" s="17" t="n">
         <v>61000</v>
       </c>
-      <c r="E10" s="29" t="n">
+      <c r="E10" s="30" t="n">
         <f aca="false">IF(D10&gt;0,C10/D10,0)</f>
         <v>0.858212295081967</v>
       </c>
-      <c r="F10" s="35" t="n">
+      <c r="F10" s="36" t="n">
         <v>4323</v>
       </c>
       <c r="G10" s="12" t="n">
@@ -2344,7 +2406,7 @@
         <f aca="false">IF(B10&gt;0,F10/B10,0)</f>
         <v>139.451612903226</v>
       </c>
-      <c r="J10" s="30" t="n">
+      <c r="J10" s="31" t="n">
         <f aca="false">Récap!$B$31</f>
         <v>0.45</v>
       </c>
@@ -2352,19 +2414,20 @@
         <f aca="false">C10*J10</f>
         <v>23557.9275</v>
       </c>
-      <c r="L10" s="17" t="n">
-        <v>8167.75</v>
+      <c r="L10" s="7" t="n">
+        <f aca="false">Récap!$C$28*31/7</f>
+        <v>11735.7142857143</v>
       </c>
       <c r="M10" s="18" t="n">
         <f aca="false">IF(C10&gt;0,L10/C10,0)</f>
-        <v>0.15601913623344</v>
-      </c>
-      <c r="N10" s="36" t="n">
+        <v>0.22417385521589</v>
+      </c>
+      <c r="N10" s="37" t="n">
         <v>792</v>
       </c>
       <c r="O10" s="12" t="n">
         <f aca="false">IF(N10&gt;0,L10/N10,0)</f>
-        <v>10.3128156565657</v>
+        <v>14.8178210678211</v>
       </c>
       <c r="P10" s="17" t="n">
         <v>13042.63</v>
@@ -2375,21 +2438,24 @@
       </c>
       <c r="R10" s="8" t="n">
         <f aca="false">C10-K10-L10-P10</f>
-        <v>7582.6425</v>
+        <v>4014.67821428571</v>
       </c>
       <c r="S10" s="18" t="n">
         <f aca="false">IF(C10&gt;0,R10/C10,0)</f>
-        <v>0.144842500470383</v>
-      </c>
-      <c r="T10" s="33" t="n">
+        <v>0.0766877814879332</v>
+      </c>
+      <c r="T10" s="34" t="n">
         <v>0.364</v>
+      </c>
+      <c r="U10" s="17" t="n">
+        <v>8167.75</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B11" s="35" t="n">
+        <v>105</v>
+      </c>
+      <c r="B11" s="36" t="n">
         <v>30</v>
       </c>
       <c r="C11" s="17" t="n">
@@ -2398,11 +2464,11 @@
       <c r="D11" s="17" t="n">
         <v>61000</v>
       </c>
-      <c r="E11" s="29" t="n">
+      <c r="E11" s="30" t="n">
         <f aca="false">IF(D11&gt;0,C11/D11,0)</f>
         <v>0.833602459016393</v>
       </c>
-      <c r="F11" s="35" t="n">
+      <c r="F11" s="36" t="n">
         <v>4156</v>
       </c>
       <c r="G11" s="12" t="n">
@@ -2417,7 +2483,7 @@
         <f aca="false">IF(B11&gt;0,F11/B11,0)</f>
         <v>138.533333333333</v>
       </c>
-      <c r="J11" s="30" t="n">
+      <c r="J11" s="31" t="n">
         <f aca="false">Récap!$B$31</f>
         <v>0.45</v>
       </c>
@@ -2425,19 +2491,20 @@
         <f aca="false">C11*J11</f>
         <v>22882.3875</v>
       </c>
-      <c r="L11" s="17" t="n">
-        <v>9477.5</v>
+      <c r="L11" s="7" t="n">
+        <f aca="false">Récap!$C$28*30/7</f>
+        <v>11357.1428571429</v>
       </c>
       <c r="M11" s="18" t="n">
         <f aca="false">IF(C11&gt;0,L11/C11,0)</f>
-        <v>0.186382430592087</v>
-      </c>
-      <c r="N11" s="36" t="n">
+        <v>0.223347073626574</v>
+      </c>
+      <c r="N11" s="37" t="n">
         <v>782</v>
       </c>
       <c r="O11" s="12" t="n">
         <f aca="false">IF(N11&gt;0,L11/N11,0)</f>
-        <v>12.1195652173913</v>
+        <v>14.5232005845817</v>
       </c>
       <c r="P11" s="17" t="n">
         <v>13042.8</v>
@@ -2448,264 +2515,279 @@
       </c>
       <c r="R11" s="8" t="n">
         <f aca="false">C11-K11-L11-P11</f>
-        <v>5447.0625</v>
+        <v>3567.41964285714</v>
       </c>
       <c r="S11" s="18" t="n">
         <f aca="false">IF(C11&gt;0,R11/C11,0)</f>
-        <v>0.107120733140281</v>
-      </c>
-      <c r="T11" s="33" t="n">
+        <v>0.0701560901057949</v>
+      </c>
+      <c r="T11" s="34" t="n">
         <v>0.362</v>
       </c>
+      <c r="U11" s="17" t="n">
+        <v>9477.5</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37" t="s">
-        <v>104</v>
-      </c>
-      <c r="B12" s="38" t="n">
+      <c r="A12" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" s="39" t="n">
         <f aca="false">SUM(B5:B11)</f>
         <v>213</v>
       </c>
-      <c r="C12" s="39" t="n">
+      <c r="C12" s="40" t="n">
         <f aca="false">SUM(C5:C11)</f>
         <v>361223.56</v>
       </c>
-      <c r="D12" s="39" t="n">
+      <c r="D12" s="40" t="n">
         <f aca="false">SUM(D5:D11)</f>
         <v>432000</v>
       </c>
-      <c r="E12" s="40" t="n">
+      <c r="E12" s="41" t="n">
         <f aca="false">IF(D12&gt;0,C12/D12,0)</f>
         <v>0.836165648148148</v>
       </c>
-      <c r="F12" s="38" t="n">
+      <c r="F12" s="39" t="n">
         <f aca="false">SUM(F5:F11)</f>
         <v>29649</v>
       </c>
-      <c r="G12" s="41" t="n">
+      <c r="G12" s="42" t="n">
         <f aca="false">IF(F12&gt;0,C12/F12,0)</f>
         <v>12.1833302978178</v>
       </c>
-      <c r="H12" s="39" t="n">
+      <c r="H12" s="40" t="n">
         <f aca="false">IF(B12&gt;0,C12/B12,0)</f>
         <v>1695.88525821596</v>
       </c>
-      <c r="I12" s="38" t="n">
+      <c r="I12" s="39" t="n">
         <f aca="false">IF(B12&gt;0,F12/B12,0)</f>
         <v>139.197183098592</v>
       </c>
-      <c r="J12" s="42" t="n">
+      <c r="J12" s="43" t="n">
         <f aca="false">IF(C12&gt;0,K12/C12,0)</f>
         <v>0.45</v>
       </c>
-      <c r="K12" s="39" t="n">
+      <c r="K12" s="40" t="n">
         <f aca="false">SUM(K5:K11)</f>
         <v>162550.602</v>
       </c>
-      <c r="L12" s="39" t="n">
+      <c r="L12" s="40" t="n">
         <f aca="false">SUM(L5:L11)</f>
-        <v>56699</v>
-      </c>
-      <c r="M12" s="42" t="n">
+        <v>81014.2857142857</v>
+      </c>
+      <c r="M12" s="43" t="n">
         <f aca="false">IF(C12&gt;0,L12/C12,0)</f>
-        <v>0.156963737359767</v>
-      </c>
-      <c r="N12" s="43" t="n">
+        <v>0.224277413450789</v>
+      </c>
+      <c r="N12" s="44" t="n">
         <f aca="false">SUM(N5:N11)</f>
         <v>5054.5</v>
       </c>
-      <c r="O12" s="41" t="n">
+      <c r="O12" s="42" t="n">
         <f aca="false">IF(N12&gt;0,L12/N12,0)</f>
-        <v>11.2175289346127</v>
-      </c>
-      <c r="P12" s="39" t="n">
+        <v>16.0281503045377</v>
+      </c>
+      <c r="P12" s="40" t="n">
         <f aca="false">SUM(P5:P11)</f>
         <v>88288.7</v>
       </c>
-      <c r="Q12" s="42" t="n">
+      <c r="Q12" s="43" t="n">
         <f aca="false">IF(C12&gt;0,P12/C12,0)</f>
         <v>0.244415674326448</v>
       </c>
-      <c r="R12" s="39" t="n">
+      <c r="R12" s="40" t="n">
         <f aca="false">SUM(R5:R11)</f>
-        <v>53685.258</v>
-      </c>
-      <c r="S12" s="42" t="n">
+        <v>29369.9722857143</v>
+      </c>
+      <c r="S12" s="43" t="n">
         <f aca="false">IF(C12&gt;0,R12/C12,0)</f>
-        <v>0.148620588313786</v>
-      </c>
-      <c r="T12" s="42" t="n">
+        <v>0.0813069122227639</v>
+      </c>
+      <c r="T12" s="43" t="n">
         <f aca="false">IF(SUM(C5:C11)&gt;0,SUMPRODUCT(C5:C11,T5:T11)/SUM(C5:C11),0)</f>
         <v>0.374197998657673</v>
       </c>
+      <c r="U12" s="40" t="n">
+        <f aca="false">SUM(U5:U11)</f>
+        <v>56699</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37" t="s">
-        <v>105</v>
-      </c>
-      <c r="B13" s="43" t="n">
+      <c r="A13" s="38" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="44" t="n">
         <f aca="false">AVERAGE(B5:B11)</f>
         <v>30.4285714285714</v>
       </c>
-      <c r="C13" s="39" t="n">
+      <c r="C13" s="40" t="n">
         <f aca="false">AVERAGE(C5:C11)</f>
         <v>51603.3657142857</v>
       </c>
-      <c r="D13" s="39" t="n">
+      <c r="D13" s="40" t="n">
         <f aca="false">AVERAGE(D5:D11)</f>
         <v>61714.2857142857</v>
       </c>
-      <c r="E13" s="40" t="n">
+      <c r="E13" s="41" t="n">
         <f aca="false">IF(D13&gt;0,C13/D13,0)</f>
         <v>0.836165648148148</v>
       </c>
-      <c r="F13" s="38" t="n">
+      <c r="F13" s="39" t="n">
         <f aca="false">AVERAGE(F5:F11)</f>
         <v>4235.57142857143</v>
       </c>
-      <c r="G13" s="41" t="n">
+      <c r="G13" s="42" t="n">
         <f aca="false">IF(F13&gt;0,C13/F13,0)</f>
         <v>12.1833302978178</v>
       </c>
-      <c r="H13" s="39" t="n">
+      <c r="H13" s="40" t="n">
         <f aca="false">IF(B13&gt;0,C13/B13,0)</f>
         <v>1695.88525821596</v>
       </c>
-      <c r="I13" s="38" t="n">
+      <c r="I13" s="39" t="n">
         <f aca="false">IF(B13&gt;0,F13/B13,0)</f>
         <v>139.197183098592</v>
       </c>
-      <c r="J13" s="42" t="n">
+      <c r="J13" s="43" t="n">
         <f aca="false">IF(C13&gt;0,K13/C13,0)</f>
         <v>0.45</v>
       </c>
-      <c r="K13" s="39" t="n">
+      <c r="K13" s="40" t="n">
         <f aca="false">AVERAGE(K5:K11)</f>
         <v>23221.5145714286</v>
       </c>
-      <c r="L13" s="39" t="n">
+      <c r="L13" s="40" t="n">
         <f aca="false">AVERAGE(L5:L11)</f>
-        <v>8099.85714285714</v>
-      </c>
-      <c r="M13" s="42" t="n">
+        <v>11573.4693877551</v>
+      </c>
+      <c r="M13" s="43" t="n">
         <f aca="false">IF(C13&gt;0,L13/C13,0)</f>
-        <v>0.156963737359767</v>
-      </c>
-      <c r="N13" s="43" t="n">
+        <v>0.224277413450789</v>
+      </c>
+      <c r="N13" s="44" t="n">
         <f aca="false">AVERAGE(N5:N11)</f>
         <v>722.071428571429</v>
       </c>
-      <c r="O13" s="41" t="n">
+      <c r="O13" s="42" t="n">
         <f aca="false">IF(N13&gt;0,L13/N13,0)</f>
-        <v>11.2175289346127</v>
-      </c>
-      <c r="P13" s="39" t="n">
+        <v>16.0281503045377</v>
+      </c>
+      <c r="P13" s="40" t="n">
         <f aca="false">AVERAGE(P5:P11)</f>
         <v>12612.6714285714</v>
       </c>
-      <c r="Q13" s="42" t="n">
+      <c r="Q13" s="43" t="n">
         <f aca="false">IF(C13&gt;0,P13/C13,0)</f>
         <v>0.244415674326448</v>
       </c>
-      <c r="R13" s="39" t="n">
+      <c r="R13" s="40" t="n">
         <f aca="false">AVERAGE(R5:R11)</f>
-        <v>7669.32257142857</v>
-      </c>
-      <c r="S13" s="42" t="n">
+        <v>4195.71032653061</v>
+      </c>
+      <c r="S13" s="43" t="n">
         <f aca="false">IF(C13&gt;0,R13/C13,0)</f>
-        <v>0.148620588313786</v>
-      </c>
-      <c r="T13" s="42" t="n">
+        <v>0.0813069122227639</v>
+      </c>
+      <c r="T13" s="43" t="n">
         <f aca="false">IF(SUM(C5:C11)&gt;0,SUMPRODUCT(C5:C11,T5:T11)/SUM(C5:C11),0)</f>
         <v>0.374197998657673</v>
       </c>
+      <c r="U13" s="40" t="n">
+        <f aca="false">AVERAGE(U5:U11)</f>
+        <v>8099.85714285714</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="37" t="s">
-        <v>106</v>
-      </c>
-      <c r="B14" s="43" t="n">
+      <c r="A14" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="44" t="n">
         <f aca="false">AVERAGE(B9:B11)</f>
         <v>30.3333333333333</v>
       </c>
-      <c r="C14" s="39" t="n">
+      <c r="C14" s="40" t="n">
         <f aca="false">AVERAGE(C9:C11)</f>
         <v>49812.4166666667</v>
       </c>
-      <c r="D14" s="39" t="n">
+      <c r="D14" s="40" t="n">
         <f aca="false">AVERAGE(D9:D11)</f>
         <v>61333.3333333333</v>
       </c>
-      <c r="E14" s="40" t="n">
+      <c r="E14" s="41" t="n">
         <f aca="false">IF(D14&gt;0,C14/D14,0)</f>
         <v>0.812158967391304</v>
       </c>
-      <c r="F14" s="38" t="n">
+      <c r="F14" s="39" t="n">
         <f aca="false">AVERAGE(F9:F11)</f>
         <v>4085</v>
       </c>
-      <c r="G14" s="41" t="n">
+      <c r="G14" s="42" t="n">
         <f aca="false">IF(F14&gt;0,C14/F14,0)</f>
         <v>12.1939820481436</v>
       </c>
-      <c r="H14" s="39" t="n">
+      <c r="H14" s="40" t="n">
         <f aca="false">IF(B14&gt;0,C14/B14,0)</f>
         <v>1642.16758241758</v>
       </c>
-      <c r="I14" s="38" t="n">
+      <c r="I14" s="39" t="n">
         <f aca="false">IF(B14&gt;0,F14/B14,0)</f>
         <v>134.67032967033</v>
       </c>
-      <c r="J14" s="42" t="n">
+      <c r="J14" s="43" t="n">
         <f aca="false">IF(C14&gt;0,K14/C14,0)</f>
         <v>0.45</v>
       </c>
-      <c r="K14" s="39" t="n">
+      <c r="K14" s="40" t="n">
         <f aca="false">AVERAGE(K9:K11)</f>
         <v>22415.5875</v>
       </c>
-      <c r="L14" s="39" t="n">
+      <c r="L14" s="40" t="n">
         <f aca="false">AVERAGE(L9:L11)</f>
-        <v>8585.33333333333</v>
-      </c>
-      <c r="M14" s="42" t="n">
+        <v>11609.5238095238</v>
+      </c>
+      <c r="M14" s="43" t="n">
         <f aca="false">IF(C14&gt;0,L14/C14,0)</f>
-        <v>0.172353278717321</v>
-      </c>
-      <c r="N14" s="43" t="n">
+        <v>0.233064857848839</v>
+      </c>
+      <c r="N14" s="44" t="n">
         <f aca="false">AVERAGE(N9:N11)</f>
         <v>749.833333333333</v>
       </c>
-      <c r="O14" s="41" t="n">
+      <c r="O14" s="42" t="n">
         <f aca="false">IF(N14&gt;0,L14/N14,0)</f>
-        <v>11.4496554789953</v>
-      </c>
-      <c r="P14" s="39" t="n">
+        <v>15.4828057028546</v>
+      </c>
+      <c r="P14" s="40" t="n">
         <f aca="false">AVERAGE(P9:P11)</f>
         <v>13042.6866666667</v>
       </c>
-      <c r="Q14" s="42" t="n">
+      <c r="Q14" s="43" t="n">
         <f aca="false">IF(C14&gt;0,P14/C14,0)</f>
         <v>0.261836054932756</v>
       </c>
-      <c r="R14" s="39" t="n">
+      <c r="R14" s="40" t="n">
         <f aca="false">AVERAGE(R9:R11)</f>
-        <v>5768.80916666667</v>
-      </c>
-      <c r="S14" s="42" t="n">
+        <v>2744.61869047619</v>
+      </c>
+      <c r="S14" s="43" t="n">
         <f aca="false">IF(C14&gt;0,R14/C14,0)</f>
-        <v>0.115810666349923</v>
-      </c>
-      <c r="T14" s="42" t="n">
+        <v>0.0550990872184049</v>
+      </c>
+      <c r="T14" s="43" t="n">
         <f aca="false">IF(SUM(C9:C11)&gt;0,SUMPRODUCT(C9:C11,T9:T11)/SUM(C9:C11),0)</f>
         <v>0.364557067933196</v>
       </c>
+      <c r="U14" s="40" t="n">
+        <f aca="false">AVERAGE(U9:U11)</f>
+        <v>8585.33333333333</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="44" t="s">
-        <v>107</v>
-      </c>
-      <c r="B16" s="35" t="n">
+      <c r="A16" s="45" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="36" t="n">
         <v>12</v>
       </c>
       <c r="C16" s="17" t="n">
@@ -2714,11 +2796,11 @@
       <c r="D16" s="17" t="n">
         <v>23834.15</v>
       </c>
-      <c r="E16" s="29" t="n">
+      <c r="E16" s="30" t="n">
         <f aca="false">IF(D16&gt;0,C16/D16,0)</f>
         <v>0.981857964307517</v>
       </c>
-      <c r="F16" s="35" t="n">
+      <c r="F16" s="36" t="n">
         <v>1835</v>
       </c>
       <c r="G16" s="12" t="n">
@@ -2737,7 +2819,7 @@
         <v>486.38</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2769,17 +2851,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C3" s="7" t="n">
         <f aca="false">'Mois par mois'!C13</f>
@@ -2787,36 +2869,36 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="45" t="s">
-        <v>112</v>
-      </c>
-      <c r="B5" s="45" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5" s="45" t="s">
+      <c r="A5" s="46" t="s">
         <v>114</v>
       </c>
-      <c r="D5" s="45" t="s">
+      <c r="B5" s="46" t="s">
         <v>115</v>
       </c>
-      <c r="E5" s="45" t="s">
+      <c r="C5" s="46" t="s">
         <v>116</v>
       </c>
-      <c r="F5" s="45" t="s">
+      <c r="D5" s="46" t="s">
         <v>117</v>
+      </c>
+      <c r="E5" s="46" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5" s="46" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="C6" s="33" t="n">
+        <v>121</v>
+      </c>
+      <c r="C6" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="33" t="n">
+      <c r="D6" s="34" t="n">
         <v>0.36</v>
       </c>
       <c r="E6" s="8" t="n">
@@ -2827,15 +2909,15 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C7" s="33" t="n">
+        <v>122</v>
+      </c>
+      <c r="C7" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="33" t="n">
+      <c r="D7" s="34" t="n">
         <v>0.02</v>
       </c>
       <c r="E7" s="8" t="n">
@@ -2846,15 +2928,15 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="C8" s="33" t="n">
+        <v>124</v>
+      </c>
+      <c r="C8" s="34" t="n">
         <v>0.07</v>
       </c>
-      <c r="D8" s="33" t="n">
+      <c r="D8" s="34" t="n">
         <v>0.07</v>
       </c>
       <c r="E8" s="8" t="n">
@@ -2862,20 +2944,20 @@
         <v>3612.2356</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="C9" s="33" t="n">
+        <v>126</v>
+      </c>
+      <c r="C9" s="34" t="n">
         <v>0.05</v>
       </c>
-      <c r="D9" s="33" t="n">
+      <c r="D9" s="34" t="n">
         <v>0.05</v>
       </c>
       <c r="E9" s="8" t="n">
@@ -2883,20 +2965,20 @@
         <v>2580.16828571429</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="C10" s="33" t="n">
+        <v>128</v>
+      </c>
+      <c r="C10" s="34" t="n">
         <v>0.01</v>
       </c>
-      <c r="D10" s="33" t="n">
+      <c r="D10" s="34" t="n">
         <v>0.005</v>
       </c>
       <c r="E10" s="8" t="n">
@@ -2904,20 +2986,20 @@
         <v>516.033657142857</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="C11" s="33" t="n">
+        <v>130</v>
+      </c>
+      <c r="C11" s="34" t="n">
         <v>0.01</v>
       </c>
-      <c r="D11" s="33" t="n">
+      <c r="D11" s="34" t="n">
         <v>0.01</v>
       </c>
       <c r="E11" s="8" t="n">
@@ -2925,20 +3007,20 @@
         <v>516.033657142857</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="C12" s="33" t="n">
+        <v>133</v>
+      </c>
+      <c r="C12" s="34" t="n">
         <v>0.02</v>
       </c>
-      <c r="D12" s="33" t="n">
+      <c r="D12" s="34" t="n">
         <v>0.02</v>
       </c>
       <c r="E12" s="8" t="n">
@@ -2946,20 +3028,20 @@
         <v>1032.06731428571</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="C13" s="33" t="n">
+        <v>134</v>
+      </c>
+      <c r="C13" s="34" t="n">
         <v>0.015</v>
       </c>
-      <c r="D13" s="33" t="n">
+      <c r="D13" s="34" t="n">
         <v>0.015</v>
       </c>
       <c r="E13" s="8" t="n">
@@ -2967,20 +3049,20 @@
         <v>774.050485714286</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="C14" s="33" t="n">
+        <v>135</v>
+      </c>
+      <c r="C14" s="34" t="n">
         <v>0.015</v>
       </c>
-      <c r="D14" s="33" t="n">
+      <c r="D14" s="34" t="n">
         <v>0.015</v>
       </c>
       <c r="E14" s="8" t="n">
@@ -2988,20 +3070,20 @@
         <v>774.050485714286</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="C15" s="33" t="n">
+        <v>137</v>
+      </c>
+      <c r="C15" s="34" t="n">
         <v>0.05</v>
       </c>
-      <c r="D15" s="33" t="n">
+      <c r="D15" s="34" t="n">
         <v>0.07</v>
       </c>
       <c r="E15" s="8" t="n">
@@ -3009,20 +3091,20 @@
         <v>2580.16828571429</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="C16" s="33" t="n">
+        <v>139</v>
+      </c>
+      <c r="C16" s="34" t="n">
         <v>0.015</v>
       </c>
-      <c r="D16" s="33" t="n">
+      <c r="D16" s="34" t="n">
         <v>0.015</v>
       </c>
       <c r="E16" s="8" t="n">
@@ -3030,12 +3112,12 @@
         <v>774.050485714286</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="19" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C17" s="21" t="n">
         <f aca="false">SUM(C6:C16)</f>
@@ -3048,7 +3130,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E19" s="7" t="n">
         <f aca="false">'Mois par mois'!P14</f>
@@ -3057,7 +3139,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tableau récap Halle : page 3, le compte d'exploitation de la fiduciaire (à valider, rapproché de la caisse) ; page 4, le plan d'action (dix actions commerciales, plan matière à 40 %)
compta.json porte l'analyse comptable transmise le 13/10 (avril → septembre lissé sur 6 mois) ; la page 3 signale l'ouverture au 20 février et l'écart de 12 % entre CA comptable et caisse. plan.json porte les actions. L'Excel gagne la feuille « Compte d'exploitation » : actuel, plan matière (+ 5 % de prix, − 4 600 € d'achats) et + 15 % de CA avec matière à 40 %, points morts compris.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfhpzegTMHxDopBcc2QwLH
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
+++ b/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Récap" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Mois par mois" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Modèle de charges" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Compte d’exploitation" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -137,8 +138,30 @@
 </comments>
 </file>
 
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="B44" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Mars → septembre (feuille Mois par mois) + février, du 20 au 28 : 6 507 €.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="211">
   <si>
     <t xml:space="preserve">Atelier by – Halle · tableau récap</t>
   </si>
@@ -570,6 +593,207 @@
   </si>
   <si>
     <t xml:space="preserve">La matière (36 %) et l’emballage (2 %) ne sont qu’en théorique dans ce modèle : le food cost mesuré en tient lieu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le compte d’exploitation comptable, avril → septembre 2026 (à valider)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyse transmise le 13 octobre 2026, à partir de la situation comptable au 30/09/2026 de la fiduciaire (Pardoen). Période supposée par l'analyse : avril → septembre 2026, lissée sur 6 mois ; loyer, charges locatives, assurance bâtiment et fiduciaire ramenés à leur coût mensuel. À valider. En bleu : montants de l’analyse ; fond jaune : paramètres ; en noir : calculs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paramètres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausse de prix moyenne (plan B1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">baguette et tradition inchangées, + 8 à 10 % sur viennoiserie, pâtisserie, traiteur ; volumes supposés inchangés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baisse des achats du plan (B2 + B3 + B4), € par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 300 € (commandes sur ventes réelles) + 1 150 € (sorties tracées) + 1 150 € (audit fournitures)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hausse de CA du scénario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">les + 15 % visés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière du scénario (% du CA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la cible du plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rémunération de Nathan, € par semaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">absente des comptes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remboursements crédits et leasing, € par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≈ 211 k€ sur 10 ans et 38 k€ sur 5 ans, selon l’analyse (le capital seul fait ≈ 2 390 €)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semaines par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poste (€ par mois)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actuel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% CA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan matière (B1 → B4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ 15 % de CA, matière 40 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chiffre d’affaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Achats matière (marchandises + fournitures + boissons)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emballages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marge brute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnel (sans rémunération de Nathan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loyer + charges locatives + assurance incendie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Énergie, eau, location panneaux PV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autres charges diverses (probablement les redevances)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Honoraires (fiduciaire, secrétariat social, Indeed…)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Location containers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voiture (location, carburant, assurance)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entretien, hygiène, extincteurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin, IT, téléphone, poste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Publicité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Petit matériel, entretien machines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caisse, terminal, assurances diverses, intérim, taxes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA d’exploitation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rémunération de Nathan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA, Nathan payé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remboursements crédits et leasing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Après Nathan et la banque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point mort, Nathan payé (CA par mois)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point mort avec les remboursements (CA par mois)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point mort : charges fixes (Nathan et remboursements compris) ÷ (1 − achats et emballages en % du CA). « Autres charges diverses » (probablement les redevances) comptées en fixe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le rapprochement avec la caisse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA comptable de la période (€ par mois × 6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le magasin a ouvert le 20 février 2026, pas en avril : à rapprocher avec la fiduciaire (période couverte, TVA, factures hors caisse).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA de caisse HT, avril → septembre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écart comptable − caisse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA de caisse HT, du 20 février au 30 septembre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D’où vient la perte de la situation au 30/09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pré-ouverture 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charges courues d'octobre à mars sans CA (≈ 5,3 k€ par mois)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avec une ouverture au 20 février, « charges courues » et « exploitation réelle » sont à refaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erreur de stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exploitation réelle d'avril à septembre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amortissements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frais financiers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Somme des lignes (arrondies)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perte de la situation au 30/09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À faire corriger par Pardoen avant de signer la situation et le PV d’AG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stock négatif (− 6 173 €) : impossible. Chaque millier d'euros de vrai stock en fin de période, c'est un millier d'euros de résultat en plus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">« Formation pré et post ouverture » à − 31 000 € en actif : une immobilisation négative n'a pas de sens, probablement une note de crédit mal imputée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobilier en leasing (60,9 k€) jamais amorti : il manque environ 1 000 € d'amortissement par mois, le résultat réel est donc plus mauvais que celui affiché.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rémunération dirigeant à − 2 000 € (solde débiteur) : à expliquer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lignes à justifier une par une : « autres charges diverses » à 9 k€ (si ce sont bien les redevances, à 2,6 % du CA, les reclasser), containers 7,8 k€, secrétariat social 5,8 k€ (probablement Liantis de Nathan dedans), voiture 6,6 k€.</t>
   </si>
 </sst>
 </file>
@@ -3151,4 +3375,967 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G61"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="27" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>4600</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B8" s="27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B11" s="15" t="n">
+        <f aca="false">52/12</f>
+        <v>4.33333333333333</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="B14" s="17" t="n">
+        <v>58216</v>
+      </c>
+      <c r="C14" s="24" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B14/B$14,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D14" s="23" t="n">
+        <f aca="false">B14*(1+$B$5)</f>
+        <v>61126.8</v>
+      </c>
+      <c r="E14" s="24" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D14/D$14,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F14" s="23" t="n">
+        <f aca="false">B14*(1+$B$7)</f>
+        <v>66948.4</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F14/F$14,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>28144</v>
+      </c>
+      <c r="C15" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B15/B$14,0)</f>
+        <v>0.483440978425175</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <f aca="false">B15-$B$6</f>
+        <v>23544</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D15/D$14,0)</f>
+        <v>0.385166571781935</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <f aca="false">F14*$B$8</f>
+        <v>26779.36</v>
+      </c>
+      <c r="G15" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F15/F$14,0)</f>
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B16" s="17" t="n">
+        <v>914</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B16/B$14,0)</f>
+        <v>0.0157001511611928</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <f aca="false">B16</f>
+        <v>914</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D16/D$14,0)</f>
+        <v>0.0149525249154217</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <f aca="false">IF(B14&gt;0,B16/B14*F14,0)</f>
+        <v>1051.1</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F16/F$14,0)</f>
+        <v>0.0157001511611928</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="B17" s="20" t="n">
+        <f aca="false">B14-B15-B16</f>
+        <v>29158</v>
+      </c>
+      <c r="C17" s="24" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B17/B$14,0)</f>
+        <v>0.500858870413632</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <f aca="false">D14-D15-D16</f>
+        <v>36668.8</v>
+      </c>
+      <c r="E17" s="24" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D17/D$14,0)</f>
+        <v>0.599880903302643</v>
+      </c>
+      <c r="F17" s="20" t="n">
+        <f aca="false">F14-F15-F16</f>
+        <v>39117.94</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F17/F$14,0)</f>
+        <v>0.584299848838807</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B18" s="17" t="n">
+        <v>9364</v>
+      </c>
+      <c r="C18" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B18/B$14,0)</f>
+        <v>0.160849251064999</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <f aca="false">B18</f>
+        <v>9364</v>
+      </c>
+      <c r="E18" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D18/D$14,0)</f>
+        <v>0.153189762919047</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <f aca="false">B18</f>
+        <v>9364</v>
+      </c>
+      <c r="G18" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F18/F$14,0)</f>
+        <v>0.139868913969565</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B19" s="17" t="n">
+        <v>4862</v>
+      </c>
+      <c r="C19" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B19/B$14,0)</f>
+        <v>0.0835165590215748</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <f aca="false">B19</f>
+        <v>4862</v>
+      </c>
+      <c r="E19" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D19/D$14,0)</f>
+        <v>0.0795395800205475</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <f aca="false">B19</f>
+        <v>4862</v>
+      </c>
+      <c r="G19" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F19/F$14,0)</f>
+        <v>0.0726230948013694</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B20" s="17" t="n">
+        <v>1514</v>
+      </c>
+      <c r="C20" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B20/B$14,0)</f>
+        <v>0.0260065961247767</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <f aca="false">B20</f>
+        <v>1514</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D20/D$14,0)</f>
+        <v>0.0247681867855016</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <f aca="false">B20</f>
+        <v>1514</v>
+      </c>
+      <c r="G20" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F20/F$14,0)</f>
+        <v>0.0226144314128493</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B21" s="17" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C21" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B21/B$14,0)</f>
+        <v>0.0259378864916861</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <f aca="false">B21</f>
+        <v>1510</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D21/D$14,0)</f>
+        <v>0.0247027490397011</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <f aca="false">B21</f>
+        <v>1510</v>
+      </c>
+      <c r="G21" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F21/F$14,0)</f>
+        <v>0.022554683905814</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B22" s="17" t="n">
+        <v>1493</v>
+      </c>
+      <c r="C22" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B22/B$14,0)</f>
+        <v>0.0256458705510513</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <f aca="false">B22</f>
+        <v>1493</v>
+      </c>
+      <c r="E22" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D22/D$14,0)</f>
+        <v>0.0244246386200488</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <f aca="false">B22</f>
+        <v>1493</v>
+      </c>
+      <c r="G22" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F22/F$14,0)</f>
+        <v>0.0223007570009141</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B23" s="17" t="n">
+        <v>1295</v>
+      </c>
+      <c r="C23" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B23/B$14,0)</f>
+        <v>0.0222447437130686</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <f aca="false">B23</f>
+        <v>1295</v>
+      </c>
+      <c r="E23" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D23/D$14,0)</f>
+        <v>0.0211854702029224</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <f aca="false">B23</f>
+        <v>1295</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F23/F$14,0)</f>
+        <v>0.0193432554026683</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B24" s="17" t="n">
+        <v>1104</v>
+      </c>
+      <c r="C24" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B24/B$14,0)</f>
+        <v>0.0189638587329944</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <f aca="false">B24</f>
+        <v>1104</v>
+      </c>
+      <c r="E24" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D24/D$14,0)</f>
+        <v>0.018060817840947</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <f aca="false">B24</f>
+        <v>1104</v>
+      </c>
+      <c r="G24" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F24/F$14,0)</f>
+        <v>0.0164903119417342</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="B25" s="17" t="n">
+        <v>1011</v>
+      </c>
+      <c r="C25" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B25/B$14,0)</f>
+        <v>0.0173663597636389</v>
+      </c>
+      <c r="D25" s="8" t="n">
+        <f aca="false">B25</f>
+        <v>1011</v>
+      </c>
+      <c r="E25" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D25/D$14,0)</f>
+        <v>0.0165393902510846</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <f aca="false">B25</f>
+        <v>1011</v>
+      </c>
+      <c r="G25" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F25/F$14,0)</f>
+        <v>0.0151011824031642</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="B26" s="17" t="n">
+        <v>778</v>
+      </c>
+      <c r="C26" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B26/B$14,0)</f>
+        <v>0.0133640236361138</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <f aca="false">B26</f>
+        <v>778</v>
+      </c>
+      <c r="E26" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D26/D$14,0)</f>
+        <v>0.0127276415582036</v>
+      </c>
+      <c r="F26" s="8" t="n">
+        <f aca="false">B26</f>
+        <v>778</v>
+      </c>
+      <c r="G26" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F26/F$14,0)</f>
+        <v>0.0116208901183598</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="B27" s="17" t="n">
+        <v>738</v>
+      </c>
+      <c r="C27" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B27/B$14,0)</f>
+        <v>0.0126769273052082</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <f aca="false">B27</f>
+        <v>738</v>
+      </c>
+      <c r="E27" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D27/D$14,0)</f>
+        <v>0.0120732641001983</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <f aca="false">B27</f>
+        <v>738</v>
+      </c>
+      <c r="G27" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F27/F$14,0)</f>
+        <v>0.0110234150480071</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="B28" s="17" t="n">
+        <v>685</v>
+      </c>
+      <c r="C28" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B28/B$14,0)</f>
+        <v>0.0117665246667583</v>
+      </c>
+      <c r="D28" s="8" t="n">
+        <f aca="false">B28</f>
+        <v>685</v>
+      </c>
+      <c r="E28" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D28/D$14,0)</f>
+        <v>0.0112062139683412</v>
+      </c>
+      <c r="F28" s="8" t="n">
+        <f aca="false">B28</f>
+        <v>685</v>
+      </c>
+      <c r="G28" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F28/F$14,0)</f>
+        <v>0.0102317605797898</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="B29" s="17" t="n">
+        <v>512</v>
+      </c>
+      <c r="C29" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B29/B$14,0)</f>
+        <v>0.00879483303559159</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <f aca="false">B29</f>
+        <v>512</v>
+      </c>
+      <c r="E29" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D29/D$14,0)</f>
+        <v>0.00837603146246818</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <f aca="false">B29</f>
+        <v>512</v>
+      </c>
+      <c r="G29" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F29/F$14,0)</f>
+        <v>0.00764768090051443</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="B30" s="20" t="n">
+        <f aca="false">B17-SUM(B18:B29)</f>
+        <v>4292</v>
+      </c>
+      <c r="C30" s="24" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B30/B$14,0)</f>
+        <v>0.0737254363061701</v>
+      </c>
+      <c r="D30" s="20" t="n">
+        <f aca="false">D17-SUM(D18:D29)</f>
+        <v>11802.8</v>
+      </c>
+      <c r="E30" s="24" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D30/D$14,0)</f>
+        <v>0.193087156533632</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <f aca="false">F17-SUM(F18:F29)</f>
+        <v>14251.94</v>
+      </c>
+      <c r="G30" s="24" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F30/F$14,0)</f>
+        <v>0.212879471354058</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="B31" s="8" t="n">
+        <f aca="false">-$B$9*$B$11</f>
+        <v>-2166.66666666667</v>
+      </c>
+      <c r="C31" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B31/B$14,0)</f>
+        <v>-0.037217717924053</v>
+      </c>
+      <c r="D31" s="8" t="n">
+        <f aca="false">-$B$9*$B$11</f>
+        <v>-2166.66666666667</v>
+      </c>
+      <c r="E31" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D31/D$14,0)</f>
+        <v>-0.0354454456419552</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <f aca="false">-$B$9*$B$11</f>
+        <v>-2166.66666666667</v>
+      </c>
+      <c r="G31" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F31/F$14,0)</f>
+        <v>-0.0323632329774374</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="B32" s="23" t="n">
+        <f aca="false">B30+B31</f>
+        <v>2125.33333333333</v>
+      </c>
+      <c r="C32" s="24" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B32/B$14,0)</f>
+        <v>0.0365077183821172</v>
+      </c>
+      <c r="D32" s="23" t="n">
+        <f aca="false">D30+D31</f>
+        <v>9636.13333333334</v>
+      </c>
+      <c r="E32" s="24" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D32/D$14,0)</f>
+        <v>0.157641710891677</v>
+      </c>
+      <c r="F32" s="23" t="n">
+        <f aca="false">F30+F31</f>
+        <v>12085.2733333333</v>
+      </c>
+      <c r="G32" s="24" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F32/F$14,0)</f>
+        <v>0.18051623837662</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="B33" s="8" t="n">
+        <f aca="false">-$B$10</f>
+        <v>-2900</v>
+      </c>
+      <c r="C33" s="18" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B33/B$14,0)</f>
+        <v>-0.0498144839906555</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <f aca="false">-$B$10</f>
+        <v>-2900</v>
+      </c>
+      <c r="E33" s="18" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D33/D$14,0)</f>
+        <v>-0.0474423657053862</v>
+      </c>
+      <c r="F33" s="8" t="n">
+        <f aca="false">-$B$10</f>
+        <v>-2900</v>
+      </c>
+      <c r="G33" s="18" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F33/F$14,0)</f>
+        <v>-0.04331694260057</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="B34" s="20" t="n">
+        <f aca="false">B32+B33</f>
+        <v>-774.666666666667</v>
+      </c>
+      <c r="C34" s="24" t="n">
+        <f aca="false">IF(B$14&lt;&gt;0,B34/B$14,0)</f>
+        <v>-0.0133067656085383</v>
+      </c>
+      <c r="D34" s="20" t="n">
+        <f aca="false">D32+D33</f>
+        <v>6736.13333333334</v>
+      </c>
+      <c r="E34" s="24" t="n">
+        <f aca="false">IF(D$14&lt;&gt;0,D34/D$14,0)</f>
+        <v>0.11019934518629</v>
+      </c>
+      <c r="F34" s="20" t="n">
+        <f aca="false">F32+F33</f>
+        <v>9185.27333333333</v>
+      </c>
+      <c r="G34" s="24" t="n">
+        <f aca="false">IF(F$14&lt;&gt;0,F34/F$14,0)</f>
+        <v>0.13719929577605</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="28" t="s">
+        <v>186</v>
+      </c>
+      <c r="B36" s="32" t="n">
+        <f aca="false">IF(B14&gt;0,(SUM(B18:B29)-B31)/(1-(B15+B16)/B14),0)</f>
+        <v>53972.6223563573</v>
+      </c>
+      <c r="D36" s="32" t="n">
+        <f aca="false">IF(D14&gt;0,(SUM(D18:D29)-D31)/(1-(D15+D16)/D14),0)</f>
+        <v>45063.3892791692</v>
+      </c>
+      <c r="F36" s="32" t="n">
+        <f aca="false">IF(F14&gt;0,(SUM(F18:F29)-F31)/(1-(F15+F16)/F14),0)</f>
+        <v>46265.0584633717</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="28" t="s">
+        <v>187</v>
+      </c>
+      <c r="B37" s="32" t="n">
+        <f aca="false">IF(B14&gt;0,(SUM(B18:B29)-B31-B33)/(1-(B15+B16)/B14),0)</f>
+        <v>59762.6765438873</v>
+      </c>
+      <c r="D37" s="32" t="n">
+        <f aca="false">IF(D14&gt;0,(SUM(D18:D29)-D31-D33)/(1-(D15+D16)/D14),0)</f>
+        <v>49897.682193036</v>
+      </c>
+      <c r="F37" s="32" t="n">
+        <f aca="false">IF(F14&gt;0,(SUM(F18:F29)-F31-F33)/(1-(F15+F16)/F14),0)</f>
+        <v>51228.2635810236</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="B41" s="8" t="n">
+        <f aca="false">B14*6</f>
+        <v>349296</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B42" s="7" t="n">
+        <f aca="false">SUM('Mois par mois'!C6:C11)</f>
+        <v>312456.22</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B43" s="8" t="n">
+        <f aca="false">B41-B42</f>
+        <v>36839.78</v>
+      </c>
+      <c r="C43" s="18" t="n">
+        <f aca="false">IF(B42&gt;0,B43/B42,0)</f>
+        <v>0.117903813852706</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="B44" s="7" t="n">
+        <f aca="false">SUM('Mois par mois'!C5:C11)+6506.85</f>
+        <v>367730.41</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="B47" s="17" t="n">
+        <v>-22600</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="B48" s="17" t="n">
+        <v>-31800</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="B49" s="17" t="n">
+        <v>-6200</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B50" s="17" t="n">
+        <v>25800</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="B51" s="17" t="n">
+        <v>-13400</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B52" s="17" t="n">
+        <v>-11900</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="B53" s="20" t="n">
+        <f aca="false">SUM(B47:B52)</f>
+        <v>-60100</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="B54" s="17" t="n">
+        <v>-59900</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="35" t="s">
+        <v>206</v>
+      </c>
+      <c r="B57" s="35"/>
+      <c r="C57" s="35"/>
+      <c r="D57" s="35"/>
+      <c r="E57" s="35"/>
+      <c r="F57" s="35"/>
+      <c r="G57" s="35"/>
+    </row>
+    <row r="58" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="35" t="s">
+        <v>207</v>
+      </c>
+      <c r="B58" s="35"/>
+      <c r="C58" s="35"/>
+      <c r="D58" s="35"/>
+      <c r="E58" s="35"/>
+      <c r="F58" s="35"/>
+      <c r="G58" s="35"/>
+    </row>
+    <row r="59" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="35" t="s">
+        <v>208</v>
+      </c>
+      <c r="B59" s="35"/>
+      <c r="C59" s="35"/>
+      <c r="D59" s="35"/>
+      <c r="E59" s="35"/>
+      <c r="F59" s="35"/>
+      <c r="G59" s="35"/>
+    </row>
+    <row r="60" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="35" t="s">
+        <v>209</v>
+      </c>
+      <c r="B60" s="35"/>
+      <c r="C60" s="35"/>
+      <c r="D60" s="35"/>
+      <c r="E60" s="35"/>
+      <c r="F60" s="35"/>
+      <c r="G60" s="35"/>
+    </row>
+    <row r="61" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="B61" s="35"/>
+      <c r="C61" s="35"/>
+      <c r="D61" s="35"/>
+      <c r="E61" s="35"/>
+      <c r="F61" s="35"/>
+      <c r="G61" s="35"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A58:G58"/>
+    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A60:G60"/>
+    <mergeCell ref="A61:G61"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Tableau récap Halle : page 5, l'application et le bilan côte à côte (avril → septembre) avec la cascade du résultat à l'EBITDA ; plan commercial réduit à cinq actions, mi-octobre → fin novembre
L'Excel gagne la feuille « Application ou bilan », reliée par formules à « Mois par mois » et à « Compte d'exploitation ».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfhpzegTMHxDopBcc2QwLH
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
+++ b/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Mois par mois" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Modèle de charges" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Compte d’exploitation" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Application ou bilan" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -161,7 +162,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="236">
   <si>
     <t xml:space="preserve">Atelier by – Halle · tableau récap</t>
   </si>
@@ -794,6 +795,81 @@
   </si>
   <si>
     <t xml:space="preserve">Lignes à justifier une par une : « autres charges diverses » à 9 k€ (si ce sont bien les redevances, à 2,6 % du CA, les reclasser), containers 7,8 k€, secrétariat social 5,8 k€ (probablement Liantis de Nathan dedans), voiture 6,6 k€.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L’application ou le bilan : avril → septembre 2026, en € par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Application : la caisse et le P&amp;L du panel (feuille « Mois par mois », main-d’œuvre encodée, food cost mesuré par le panel). Bilan : la situation au 30/09 de la fiduciaire, lissée sur 6 mois (feuille « Compte d’exploitation », à valider). En vert : liens ; en noir : calculs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Application</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écart (bilan − application)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ce qui change d’une source à l’autre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">caisse HT ; à rapprocher (période, TVA, factures hors caisse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matière</t>
+  </si>
+  <si>
+    <t xml:space="preserve">application : coût de recette des ventes (panel) ; bilan : achats + emballages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heures planifiées × taux du panel, contre salaires ; Nathan absent des deux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">montant saisi au panel, contre factures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultat · EBITDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avant Nathan, amortissements, charges financières</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point mort (CA par mois)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">charges fixes ÷ (1 − matière en % du CA), Nathan non payé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients par mois (application)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panier moyen (application)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Du résultat de l’application à l’EBITDA du bilan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultat de l’application</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ CA du bilan en plus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− matière achetée en plus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− personnel en plus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− frais généraux en plus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA du bilan (somme des lignes)</t>
   </si>
 </sst>
 </file>
@@ -4338,4 +4414,324 @@
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="70"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <f aca="false">AVERAGE('Mois par mois'!C6:C11)</f>
+        <v>52076.0366666667</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <f aca="false">'Compte d’exploitation'!B14</f>
+        <v>58216</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <f aca="false">D5-B5</f>
+        <v>6139.96333333334</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <f aca="false">SUMPRODUCT('Mois par mois'!C6:C11,'Mois par mois'!T6:T11)/6</f>
+        <v>19293.28865</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <f aca="false">IF(B$5&gt;0,B6/B$5,0)</f>
+        <v>0.370483045272711</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <f aca="false">'Compte d’exploitation'!B15+'Compte d’exploitation'!B16</f>
+        <v>29058</v>
+      </c>
+      <c r="E6" s="18" t="n">
+        <f aca="false">IF(D$5&gt;0,D6/D$5,0)</f>
+        <v>0.499141129586368</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <f aca="false">D6-B6</f>
+        <v>9764.71135</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <f aca="false">B5-B6</f>
+        <v>32782.7480166667</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <f aca="false">IF(B$5&gt;0,B7/B$5,0)</f>
+        <v>0.62951695472729</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <f aca="false">D5-D6</f>
+        <v>29158</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <f aca="false">IF(D$5&gt;0,D7/D$5,0)</f>
+        <v>0.500858870413632</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <f aca="false">D7-B7</f>
+        <v>-3624.74801666666</v>
+      </c>
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <f aca="false">AVERAGE('Mois par mois'!U6:U11)</f>
+        <v>8394.16666666667</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <f aca="false">IF(B$5&gt;0,B8/B$5,0)</f>
+        <v>0.161190582155798</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <f aca="false">'Compte d’exploitation'!B18</f>
+        <v>9364</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <f aca="false">IF(D$5&gt;0,D8/D$5,0)</f>
+        <v>0.160849251064999</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <f aca="false">D8-B8</f>
+        <v>969.833333333334</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <f aca="false">AVERAGE('Mois par mois'!P6:P11)</f>
+        <v>13154.8633333333</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <f aca="false">IF(B$5&gt;0,B9/B$5,0)</f>
+        <v>0.252608765477608</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <f aca="false">SUM('Compte d’exploitation'!B19:B29)</f>
+        <v>15502</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <f aca="false">IF(D$5&gt;0,D9/D$5,0)</f>
+        <v>0.266284183042463</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <f aca="false">D9-B9</f>
+        <v>2347.13666666667</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="22" t="s">
+        <v>223</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <f aca="false">B7-B8-B9</f>
+        <v>11233.7180166667</v>
+      </c>
+      <c r="C10" s="18" t="n">
+        <f aca="false">IF(B$5&gt;0,B10/B$5,0)</f>
+        <v>0.215717607093883</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <f aca="false">D7-D8-D9</f>
+        <v>4292</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <f aca="false">IF(D$5&gt;0,D10/D$5,0)</f>
+        <v>0.0737254363061701</v>
+      </c>
+      <c r="F10" s="23" t="n">
+        <f aca="false">D10-B10</f>
+        <v>-6941.71801666667</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <f aca="false">IF(B5&gt;0,(B8+B9)/(1-B6/B5),0)</f>
+        <v>34231.0557931441</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <f aca="false">IF(D5&gt;0,(D8+D9)/(1-D6/D5),0)</f>
+        <v>49646.7198024556</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <f aca="false">D11-B11</f>
+        <v>15415.6640093115</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="B12" s="9" t="n">
+        <f aca="false">AVERAGE('Mois par mois'!F6:F11)</f>
+        <v>4218</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <f aca="false">IF(B12&gt;0,B5/B12,0)</f>
+        <v>12.3461443021969</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="B16" s="8" t="n">
+        <f aca="false">B10</f>
+        <v>11233.7180166667</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="B17" s="8" t="n">
+        <f aca="false">D5-B5</f>
+        <v>6139.96333333334</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="B18" s="8" t="n">
+        <f aca="false">-(D6-B6)</f>
+        <v>-9764.71135</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="B19" s="8" t="n">
+        <f aca="false">-(D8-B8)</f>
+        <v>-969.833333333334</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="B20" s="8" t="n">
+        <f aca="false">-(D9-B9)</f>
+        <v>-2347.13666666667</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="B21" s="20" t="n">
+        <f aca="false">SUM(B16:B20)</f>
+        <v>4292.00000000001</v>
+      </c>
+      <c r="C21" s="2" t="str">
+        <f aca="false">IF(ABS(B21-D10)&lt;1,"= bilan","écart")</f>
+        <v>= bilan</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Tableau récap Halle : les actions commerciales cèdent la place à la grille + 50 → + 250 € par jour (CA, marge directe, résultat récap et bilan, à personnel égal)
Page 4 : la grille, puis le plan matière (inchangé). L'Excel gagne la feuille « Euros par jour », reliée par formules à « Récap » et « Compte d'exploitation ».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfhpzegTMHxDopBcc2QwLH
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
+++ b/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Modèle de charges" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Compte d’exploitation" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Application ou bilan" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Euros par jour" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -162,7 +163,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="255">
   <si>
     <t xml:space="preserve">Atelier by – Halle · tableau récap</t>
   </si>
@@ -870,6 +871,63 @@
   </si>
   <si>
     <t xml:space="preserve">EBITDA du bilan (somme des lignes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ce que rapportent quelques euros de plus par jour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À personnel et frais généraux égaux, un euro vendu en plus ne coûte que sa matière. Paliers en bleu (modifiables) ; liens en vert vers « Récap » et « Compte d’exploitation ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jours par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taux de marge, bilan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA Nathan payé, bilan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Après remboursements, bilan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taux de marge, récap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultat actuel, récap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€ par jour en plus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA en plus par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA en plus par an</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients par jour en plus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ou panier en plus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marge directe par mois (récap)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résultat par mois (récap)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marge directe par mois (bilan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA Nathan payé (bilan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Après remboursements (bilan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ligne 0 : aujourd’hui. Récap : moyenne de mars à septembre ; bilan : avril → septembre. Une vente faite avec une remise rapporte moins que la marge directe.</t>
   </si>
 </sst>
 </file>
@@ -1066,7 +1124,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1253,6 +1311,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -4734,4 +4796,389 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="6" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="B4" s="47" t="n">
+        <f aca="false">Récap!B13</f>
+        <v>30.4166666666667</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="F4" s="31" t="n">
+        <f aca="false">1-('Compte d’exploitation'!B15+'Compte d’exploitation'!B16)/'Compte d’exploitation'!B14</f>
+        <v>0.500858870413632</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="11" t="n">
+        <f aca="false">Récap!B9</f>
+        <v>12.1833302978178</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <f aca="false">'Compte d’exploitation'!B32</f>
+        <v>2125.33333333333</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="9" t="n">
+        <f aca="false">Récap!B8</f>
+        <v>139.197183098592</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <f aca="false">'Compte d’exploitation'!B34</f>
+        <v>-774.666666666667</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="B7" s="31" t="n">
+        <f aca="false">1-Récap!B31</f>
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <f aca="false">Récap!B25</f>
+        <v>4195.71032653061</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <f aca="false">A11*$B$4</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <f aca="false">A11*365</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <f aca="false">IF($B$5&gt;0,A11/$B$5,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <f aca="false">IF($B$6&gt;0,A11/$B$6,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <f aca="false">B11*$B$7</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="23" t="n">
+        <f aca="false">$B$8+F11</f>
+        <v>4195.71032653061</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <f aca="false">B11*$F$4</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="23" t="n">
+        <f aca="false">$F$5+H11</f>
+        <v>2125.33333333333</v>
+      </c>
+      <c r="J11" s="23" t="n">
+        <f aca="false">$F$6+H11</f>
+        <v>-774.666666666667</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <f aca="false">A12*$B$4</f>
+        <v>1520.83333333333</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <f aca="false">A12*365</f>
+        <v>18250</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <f aca="false">IF($B$5&gt;0,A12/$B$5,0)</f>
+        <v>4.10396819077914</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <f aca="false">IF($B$6&gt;0,A12/$B$6,0)</f>
+        <v>0.359202671253668</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <f aca="false">B12*$B$7</f>
+        <v>836.458333333334</v>
+      </c>
+      <c r="G12" s="23" t="n">
+        <f aca="false">$B$8+F12</f>
+        <v>5032.16865986395</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <f aca="false">B12*$F$4</f>
+        <v>761.722865420732</v>
+      </c>
+      <c r="I12" s="23" t="n">
+        <f aca="false">$F$5+H12</f>
+        <v>2887.05619875407</v>
+      </c>
+      <c r="J12" s="23" t="n">
+        <f aca="false">$F$6+H12</f>
+        <v>-12.9438012459344</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="n">
+        <v>100</v>
+      </c>
+      <c r="B13" s="8" t="n">
+        <f aca="false">A13*$B$4</f>
+        <v>3041.66666666667</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <f aca="false">A13*365</f>
+        <v>36500</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <f aca="false">IF($B$5&gt;0,A13/$B$5,0)</f>
+        <v>8.20793638155828</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <f aca="false">IF($B$6&gt;0,A13/$B$6,0)</f>
+        <v>0.718405342507336</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <f aca="false">B13*$B$7</f>
+        <v>1672.91666666667</v>
+      </c>
+      <c r="G13" s="23" t="n">
+        <f aca="false">$B$8+F13</f>
+        <v>5868.62699319728</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <f aca="false">B13*$F$4</f>
+        <v>1523.44573084146</v>
+      </c>
+      <c r="I13" s="23" t="n">
+        <f aca="false">$F$5+H13</f>
+        <v>3648.7790641748</v>
+      </c>
+      <c r="J13" s="23" t="n">
+        <f aca="false">$F$6+H13</f>
+        <v>748.779064174798</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="n">
+        <v>150</v>
+      </c>
+      <c r="B14" s="8" t="n">
+        <f aca="false">A14*$B$4</f>
+        <v>4562.5</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <f aca="false">A14*365</f>
+        <v>54750</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <f aca="false">IF($B$5&gt;0,A14/$B$5,0)</f>
+        <v>12.3119045723374</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <f aca="false">IF($B$6&gt;0,A14/$B$6,0)</f>
+        <v>1.077608013761</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <f aca="false">B14*$B$7</f>
+        <v>2509.375</v>
+      </c>
+      <c r="G14" s="23" t="n">
+        <f aca="false">$B$8+F14</f>
+        <v>6705.08532653061</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <f aca="false">B14*$F$4</f>
+        <v>2285.1685962622</v>
+      </c>
+      <c r="I14" s="23" t="n">
+        <f aca="false">$F$5+H14</f>
+        <v>4410.50192959553</v>
+      </c>
+      <c r="J14" s="23" t="n">
+        <f aca="false">$F$6+H14</f>
+        <v>1510.50192959553</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <f aca="false">A15*$B$4</f>
+        <v>6083.33333333333</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <f aca="false">A15*365</f>
+        <v>73000</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <f aca="false">IF($B$5&gt;0,A15/$B$5,0)</f>
+        <v>16.4158727631166</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <f aca="false">IF($B$6&gt;0,A15/$B$6,0)</f>
+        <v>1.43681068501467</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <f aca="false">B15*$B$7</f>
+        <v>3345.83333333333</v>
+      </c>
+      <c r="G15" s="23" t="n">
+        <f aca="false">$B$8+F15</f>
+        <v>7541.54365986395</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <f aca="false">B15*$F$4</f>
+        <v>3046.89146168293</v>
+      </c>
+      <c r="I15" s="23" t="n">
+        <f aca="false">$F$5+H15</f>
+        <v>5172.22479501626</v>
+      </c>
+      <c r="J15" s="23" t="n">
+        <f aca="false">$F$6+H15</f>
+        <v>2272.22479501626</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17" t="n">
+        <v>250</v>
+      </c>
+      <c r="B16" s="8" t="n">
+        <f aca="false">A16*$B$4</f>
+        <v>7604.16666666667</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <f aca="false">A16*365</f>
+        <v>91250</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <f aca="false">IF($B$5&gt;0,A16/$B$5,0)</f>
+        <v>20.5198409538957</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <f aca="false">IF($B$6&gt;0,A16/$B$6,0)</f>
+        <v>1.79601335626834</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <f aca="false">B16*$B$7</f>
+        <v>4182.29166666667</v>
+      </c>
+      <c r="G16" s="23" t="n">
+        <f aca="false">$B$8+F16</f>
+        <v>8378.00199319728</v>
+      </c>
+      <c r="H16" s="8" t="n">
+        <f aca="false">B16*$F$4</f>
+        <v>3808.61432710366</v>
+      </c>
+      <c r="I16" s="23" t="n">
+        <f aca="false">$F$5+H16</f>
+        <v>5933.94766043699</v>
+      </c>
+      <c r="J16" s="23" t="n">
+        <f aca="false">$F$6+H16</f>
+        <v>3033.94766043699</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Tableau récap Halle : ouverture en mars — le compte de la fiduciaire recalculé sur sept mois (le CA comptable colle à la caisse de mars à septembre), page 4 et page 5 sur la même période, plan matière recalculé
compta.json porte la période réelle (7 mois) et les lignes déjà mensuelles (loyer, honoraires), qui ne se recalculent pas. La page 3 montre l'analyse (÷ 6) et le recalcul (÷ 7) côte à côte, perte comprise. L'Excel prend le nombre de mois en paramètre (feuille « Compte d'exploitation ») ; « Application ou bilan » et « Euros par jour » lisent la colonne recalculée.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfhpzegTMHxDopBcc2QwLH
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
+++ b/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
@@ -140,30 +140,8 @@
 </comments>
 </file>
 
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <authors>
-    <author>Unknown Author</author>
-  </authors>
-  <commentList>
-    <comment ref="B44" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Mars → septembre (feuille Mois par mois) + février, du 20 au 28 : 6 507 €.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="267">
   <si>
     <t xml:space="preserve">Atelier by – Halle · tableau récap</t>
   </si>
@@ -393,7 +371,7 @@
     <t xml:space="preserve">Les frais généraux encodés sont un montant mensuel saisi au panel, sans détail ; la feuille « Modèle de charges » donne le contenu attendu par le franchiseur (loyer, énergie, redevances, amortissements…).</t>
   </si>
   <si>
-    <t xml:space="preserve">Février (ouverture le 20) et octobre, partiels, restent hors des moyennes. Juin et juillet : travaux sur le viaduc de Halle, effet estimé − 20 %.</t>
+    <t xml:space="preserve">Ouverture en mars ; les ventes de février (du 20 au 28) et octobre, partiels, restent hors des moyennes. Juin et juillet : travaux sur le viaduc de Halle, effet estimé − 20 %.</t>
   </si>
   <si>
     <t xml:space="preserve">Atelier by – Halle · les mois pleins, mars → septembre 2026</t>
@@ -597,25 +575,46 @@
     <t xml:space="preserve">La matière (36 %) et l’emballage (2 %) ne sont qu’en théorique dans ce modèle : le food cost mesuré en tient lieu.</t>
   </si>
   <si>
-    <t xml:space="preserve">Le compte d’exploitation comptable, avril → septembre 2026 (à valider)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyse transmise le 13 octobre 2026, à partir de la situation comptable au 30/09/2026 de la fiduciaire (Pardoen). Période supposée par l'analyse : avril → septembre 2026, lissée sur 6 mois ; loyer, charges locatives, assurance bâtiment et fiduciaire ramenés à leur coût mensuel. À valider. En bleu : montants de l’analyse ; fond jaune : paramètres ; en noir : calculs.</t>
+    <t xml:space="preserve">Le compte d’exploitation comptable, mars → septembre 2026 (à valider)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyse transmise le 13 octobre 2026, à partir de la situation comptable au 30/09/2026 de la fiduciaire (Pardoen), lissée sur 6 mois (ouverture supposée en avril). Recalcul du 13 octobre : le magasin a ouvert en mars, les totaux de la période se divisent par 7 ; loyer, charges locatives, assurance et honoraires, déjà ramenés à leur coût mensuel par l'analyse, restent tels quels. À valider avec la fiduciaire. En bleu : montants de l’analyse ; fond jaune : paramètres ; en noir : calculs.</t>
   </si>
   <si>
     <t xml:space="preserve">Paramètres</t>
   </si>
   <si>
+    <t xml:space="preserve">Mois de l’analyse (ouverture supposée en avril)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la division faite par l’analyse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mois d’exploitation réels (ouverture en mars)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chaque ligne × mois de l’analyse ÷ mois réels, sauf les coûts déjà mensuels</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hausse de prix moyenne (plan B1)</t>
   </si>
   <si>
-    <t xml:space="preserve">baguette et tradition inchangées, + 8 à 10 % sur viennoiserie, pâtisserie, traiteur ; volumes supposés inchangés</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baisse des achats du plan (B2 + B3 + B4), € par mois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 300 € (commandes sur ventes réelles) + 1 150 € (sorties tracées) + 1 150 € (audit fournitures)</t>
+    <t xml:space="preserve">baguette et tradition inchangées ; volumes supposés inchangés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commandes sur ventes réelles (B2), % des achats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sorties tracées (B3), % des achats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Achats fournitures sur la période</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total de la période, selon l’analyse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audit fournitures (B4), % de la ligne</t>
   </si>
   <si>
     <t xml:space="preserve">Hausse de CA du scénario</t>
@@ -639,7 +638,7 @@
     <t xml:space="preserve">Remboursements crédits et leasing, € par mois</t>
   </si>
   <si>
-    <t xml:space="preserve">≈ 211 k€ sur 10 ans et 38 k€ sur 5 ans, selon l’analyse (le capital seul fait ≈ 2 390 €)</t>
+    <t xml:space="preserve">≈ 211 k€ sur 10 ans et 38 k€ sur 5 ans, selon l’analyse</t>
   </si>
   <si>
     <t xml:space="preserve">Semaines par mois</t>
@@ -648,7 +647,10 @@
     <t xml:space="preserve">Poste (€ par mois)</t>
   </si>
   <si>
-    <t xml:space="preserve">Actuel</t>
+    <t xml:space="preserve">Analyse (÷ 6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recalcul (mois réels)</t>
   </si>
   <si>
     <t xml:space="preserve">% CA</t>
@@ -675,7 +677,7 @@
     <t xml:space="preserve">Personnel (sans rémunération de Nathan)</t>
   </si>
   <si>
-    <t xml:space="preserve">Loyer + charges locatives + assurance incendie</t>
+    <t xml:space="preserve">Loyer + charges locatives + assurance incendie (coût mensuel, inchangé)</t>
   </si>
   <si>
     <t xml:space="preserve">Énergie, eau, location panneaux PV</t>
@@ -684,7 +686,7 @@
     <t xml:space="preserve">Autres charges diverses (probablement les redevances)</t>
   </si>
   <si>
-    <t xml:space="preserve">Honoraires (fiduciaire, secrétariat social, Indeed…)</t>
+    <t xml:space="preserve">Honoraires (fiduciaire, secrétariat social, Indeed…) (coût mensuel, inchangé)</t>
   </si>
   <si>
     <t xml:space="preserve">Location containers</t>
@@ -729,43 +731,55 @@
     <t xml:space="preserve">Point mort avec les remboursements (CA par mois)</t>
   </si>
   <si>
-    <t xml:space="preserve">Point mort : charges fixes (Nathan et remboursements compris) ÷ (1 − achats et emballages en % du CA). « Autres charges diverses » (probablement les redevances) comptées en fixe.</t>
+    <t xml:space="preserve">Point mort : charges fixes (Nathan et remboursements compris) ÷ (1 − achats et emballages en % du CA). « Autres charges diverses » (probablement les redevances) comptées en fixe. Plan matière et scénario partent du recalcul.</t>
   </si>
   <si>
     <t xml:space="preserve">Le rapprochement avec la caisse</t>
   </si>
   <si>
-    <t xml:space="preserve">CA comptable de la période (€ par mois × 6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le magasin a ouvert le 20 février 2026, pas en avril : à rapprocher avec la fiduciaire (période couverte, TVA, factures hors caisse).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CA de caisse HT, avril → septembre</t>
+    <t xml:space="preserve">CA comptable de la période (analyse × mois de l’analyse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le CA comptable colle à la caisse de mars à septembre, pas à celle d’avril à septembre : les comptes couvrent sept mois.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA de caisse HT, mars → septembre</t>
   </si>
   <si>
     <t xml:space="preserve">Écart comptable − caisse</t>
   </si>
   <si>
-    <t xml:space="preserve">CA de caisse HT, du 20 février au 30 septembre</t>
+    <t xml:space="preserve">CA de caisse HT, avril → septembre (l’hypothèse de l’analyse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écart comptable − caisse d’avril à septembre</t>
   </si>
   <si>
     <t xml:space="preserve">D’où vient la perte de la situation au 30/09</t>
   </si>
   <si>
+    <t xml:space="preserve">Analyse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recalcul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charges courues par mois sans CA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pré-ouverture 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">Charges courues d'octobre à mars sans CA (≈ 5,3 k€ par mois)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">avec une ouverture au 20 février, « charges courues » et « exploitation réelle » sont à refaire</t>
+    <t xml:space="preserve">Mois sans CA (octobre → février)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charges courues sans CA (analyse : octobre → mars ; recalcul : octobre → février)</t>
   </si>
   <si>
     <t xml:space="preserve">Erreur de stock</t>
   </si>
   <si>
-    <t xml:space="preserve">Exploitation réelle d'avril à septembre</t>
+    <t xml:space="preserve">Exploitation réelle (analyse : avril → septembre ; recalcul : mars → septembre)</t>
   </si>
   <si>
     <t xml:space="preserve">Amortissements</t>
@@ -774,7 +788,7 @@
     <t xml:space="preserve">Frais financiers</t>
   </si>
   <si>
-    <t xml:space="preserve">Somme des lignes (arrondies)</t>
+    <t xml:space="preserve">Somme des lignes</t>
   </si>
   <si>
     <t xml:space="preserve">Perte de la situation au 30/09</t>
@@ -798,10 +812,10 @@
     <t xml:space="preserve">Lignes à justifier une par une : « autres charges diverses » à 9 k€ (si ce sont bien les redevances, à 2,6 % du CA, les reclasser), containers 7,8 k€, secrétariat social 5,8 k€ (probablement Liantis de Nathan dedans), voiture 6,6 k€.</t>
   </si>
   <si>
-    <t xml:space="preserve">L’application ou le bilan : avril → septembre 2026, en € par mois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Application : la caisse et le P&amp;L du panel (feuille « Mois par mois », main-d’œuvre encodée, food cost mesuré par le panel). Bilan : la situation au 30/09 de la fiduciaire, lissée sur 6 mois (feuille « Compte d’exploitation », à valider). En vert : liens ; en noir : calculs.</t>
+    <t xml:space="preserve">L’application ou le bilan : mars → septembre 2026, en € par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Application : la caisse et le P&amp;L du panel (feuille « Mois par mois », main-d’œuvre encodée, food cost mesuré par le panel). Bilan : la situation au 30/09 de la fiduciaire, recalculée sur les mois réels (feuille « Compte d’exploitation », colonne Recalcul, à valider). En vert : liens ; en noir : calculs.</t>
   </si>
   <si>
     <t xml:space="preserve">Application</t>
@@ -816,7 +830,7 @@
     <t xml:space="preserve">Ce qui change d’une source à l’autre</t>
   </si>
   <si>
-    <t xml:space="preserve">caisse HT ; à rapprocher (période, TVA, factures hors caisse)</t>
+    <t xml:space="preserve">caisse HT, contre CA comptable recalculé</t>
   </si>
   <si>
     <t xml:space="preserve">Matière</t>
@@ -858,16 +872,16 @@
     <t xml:space="preserve">Résultat de l’application</t>
   </si>
   <si>
-    <t xml:space="preserve">+ CA du bilan en plus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">− matière achetée en plus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">− personnel en plus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">− frais généraux en plus</t>
+    <t xml:space="preserve">Écart de CA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écart de matière</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écart de personnel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écart de frais généraux</t>
   </si>
   <si>
     <t xml:space="preserve">EBITDA du bilan (somme des lignes)</t>
@@ -927,7 +941,7 @@
     <t xml:space="preserve">Après remboursements (bilan)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ligne 0 : aujourd’hui. Récap : moyenne de mars à septembre ; bilan : avril → septembre. Une vente faite avec une remise rapporte moins que la marge directe.</t>
+    <t xml:space="preserve">Ligne 0 : aujourd’hui, moyenne de mars à septembre (le bilan recalculé sur sept mois). Une vente faite avec une remise rapporte moins que la marge directe.</t>
   </si>
 </sst>
 </file>
@@ -1124,7 +1138,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1311,6 +1325,14 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -3520,16 +3542,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3551,10 +3573,10 @@
       <c r="A5" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="B5" s="27" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="B5" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>148</v>
       </c>
     </row>
@@ -3562,10 +3584,10 @@
       <c r="A6" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B6" s="14" t="n">
-        <v>4600</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="B6" s="47" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>150</v>
       </c>
     </row>
@@ -3574,9 +3596,9 @@
         <v>151</v>
       </c>
       <c r="B7" s="27" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D7" s="2" t="s">
+        <v>0.05</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>152</v>
       </c>
     </row>
@@ -3585,887 +3607,1096 @@
         <v>153</v>
       </c>
       <c r="B8" s="27" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>154</v>
-      </c>
+        <v>0.08</v>
+      </c>
+      <c r="C8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="B9" s="14" t="n">
-        <v>500</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>156</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="B9" s="27" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="B10" s="14" t="n">
-        <v>2900</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
+      </c>
+      <c r="B10" s="17" t="n">
+        <v>19500</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="B11" s="27" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B12" s="27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B11" s="15" t="n">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="B13" s="27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B15" s="14" t="n">
+        <v>2900</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B16" s="15" t="n">
         <f aca="false">52/12</f>
         <v>4.33333333333333</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="B14" s="17" t="n">
+    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="B19" s="17" t="n">
         <v>58216</v>
       </c>
-      <c r="C14" s="24" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B14/B$14,0)</f>
+      <c r="C19" s="23" t="n">
+        <f aca="false">B19*$B$5/$B$6</f>
+        <v>49899.4285714286</v>
+      </c>
+      <c r="D19" s="24" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C19/C$19,0)</f>
         <v>1</v>
       </c>
-      <c r="D14" s="23" t="n">
-        <f aca="false">B14*(1+$B$5)</f>
-        <v>61126.8</v>
-      </c>
-      <c r="E14" s="24" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D14/D$14,0)</f>
+      <c r="E19" s="23" t="n">
+        <f aca="false">C19*(1+$B$7)</f>
+        <v>52394.4</v>
+      </c>
+      <c r="F19" s="24" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E19/E$19,0)</f>
         <v>1</v>
       </c>
-      <c r="F14" s="23" t="n">
-        <f aca="false">B14*(1+$B$7)</f>
-        <v>66948.4</v>
-      </c>
-      <c r="G14" s="24" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F14/F$14,0)</f>
+      <c r="G19" s="23" t="n">
+        <f aca="false">C19*(1+$B$12)</f>
+        <v>57384.3428571429</v>
+      </c>
+      <c r="H19" s="24" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G19/G$19,0)</f>
         <v>1</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B15" s="17" t="n">
-        <v>28144</v>
-      </c>
-      <c r="C15" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B15/B$14,0)</f>
-        <v>0.483440978425175</v>
-      </c>
-      <c r="D15" s="8" t="n">
-        <f aca="false">B15-$B$6</f>
-        <v>23544</v>
-      </c>
-      <c r="E15" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D15/D$14,0)</f>
-        <v>0.385166571781935</v>
-      </c>
-      <c r="F15" s="8" t="n">
-        <f aca="false">F14*$B$8</f>
-        <v>26779.36</v>
-      </c>
-      <c r="G15" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F15/F$14,0)</f>
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="B16" s="17" t="n">
-        <v>914</v>
-      </c>
-      <c r="C16" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B16/B$14,0)</f>
-        <v>0.0157001511611928</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <f aca="false">B16</f>
-        <v>914</v>
-      </c>
-      <c r="E16" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D16/D$14,0)</f>
-        <v>0.0149525249154217</v>
-      </c>
-      <c r="F16" s="8" t="n">
-        <f aca="false">IF(B14&gt;0,B16/B14*F14,0)</f>
-        <v>1051.1</v>
-      </c>
-      <c r="G16" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F16/F$14,0)</f>
-        <v>0.0157001511611928</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="B17" s="20" t="n">
-        <f aca="false">B14-B15-B16</f>
-        <v>29158</v>
-      </c>
-      <c r="C17" s="24" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B17/B$14,0)</f>
-        <v>0.500858870413632</v>
-      </c>
-      <c r="D17" s="20" t="n">
-        <f aca="false">D14-D15-D16</f>
-        <v>36668.8</v>
-      </c>
-      <c r="E17" s="24" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D17/D$14,0)</f>
-        <v>0.599880903302643</v>
-      </c>
-      <c r="F17" s="20" t="n">
-        <f aca="false">F14-F15-F16</f>
-        <v>39117.94</v>
-      </c>
-      <c r="G17" s="24" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F17/F$14,0)</f>
-        <v>0.584299848838807</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="B18" s="17" t="n">
-        <v>9364</v>
-      </c>
-      <c r="C18" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B18/B$14,0)</f>
-        <v>0.160849251064999</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <f aca="false">B18</f>
-        <v>9364</v>
-      </c>
-      <c r="E18" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D18/D$14,0)</f>
-        <v>0.153189762919047</v>
-      </c>
-      <c r="F18" s="8" t="n">
-        <f aca="false">B18</f>
-        <v>9364</v>
-      </c>
-      <c r="G18" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F18/F$14,0)</f>
-        <v>0.139868913969565</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="B19" s="17" t="n">
-        <v>4862</v>
-      </c>
-      <c r="C19" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B19/B$14,0)</f>
-        <v>0.0835165590215748</v>
-      </c>
-      <c r="D19" s="8" t="n">
-        <f aca="false">B19</f>
-        <v>4862</v>
-      </c>
-      <c r="E19" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D19/D$14,0)</f>
-        <v>0.0795395800205475</v>
-      </c>
-      <c r="F19" s="8" t="n">
-        <f aca="false">B19</f>
-        <v>4862</v>
-      </c>
-      <c r="G19" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F19/F$14,0)</f>
-        <v>0.0726230948013694</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B20" s="17" t="n">
-        <v>1514</v>
-      </c>
-      <c r="C20" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B20/B$14,0)</f>
-        <v>0.0260065961247767</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <f aca="false">B20</f>
-        <v>1514</v>
-      </c>
-      <c r="E20" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D20/D$14,0)</f>
-        <v>0.0247681867855016</v>
-      </c>
-      <c r="F20" s="8" t="n">
-        <f aca="false">B20</f>
-        <v>1514</v>
-      </c>
-      <c r="G20" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F20/F$14,0)</f>
-        <v>0.0226144314128493</v>
+        <v>28144</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <f aca="false">B20*$B$5/$B$6</f>
+        <v>24123.4285714286</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C20/C$19,0)</f>
+        <v>0.483440978425175</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <f aca="false">C20*(1-$B$8-$B$9)-$B$10/$B$6*$B$11</f>
+        <v>20253.6171428571</v>
+      </c>
+      <c r="F20" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E20/E$19,0)</f>
+        <v>0.386560722956216</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <f aca="false">G19*$B$13</f>
+        <v>22953.7371428571</v>
+      </c>
+      <c r="H20" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G20/G$19,0)</f>
+        <v>0.4</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B21" s="17" t="n">
-        <v>1510</v>
-      </c>
-      <c r="C21" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B21/B$14,0)</f>
-        <v>0.0259378864916861</v>
-      </c>
-      <c r="D21" s="8" t="n">
-        <f aca="false">B21</f>
-        <v>1510</v>
-      </c>
-      <c r="E21" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D21/D$14,0)</f>
-        <v>0.0247027490397011</v>
-      </c>
-      <c r="F21" s="8" t="n">
-        <f aca="false">B21</f>
-        <v>1510</v>
-      </c>
-      <c r="G21" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F21/F$14,0)</f>
-        <v>0.022554683905814</v>
+        <v>914</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <f aca="false">B21*$B$5/$B$6</f>
+        <v>783.428571428571</v>
+      </c>
+      <c r="D21" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C21/C$19,0)</f>
+        <v>0.0157001511611928</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <f aca="false">C21</f>
+        <v>783.428571428571</v>
+      </c>
+      <c r="F21" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E21/E$19,0)</f>
+        <v>0.0149525249154217</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <f aca="false">IF(C19&gt;0,C21/C19*G19,0)</f>
+        <v>900.942857142857</v>
+      </c>
+      <c r="H21" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G21/G$19,0)</f>
+        <v>0.0157001511611928</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="B22" s="17" t="n">
-        <v>1493</v>
-      </c>
-      <c r="C22" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B22/B$14,0)</f>
-        <v>0.0256458705510513</v>
-      </c>
-      <c r="D22" s="8" t="n">
-        <f aca="false">B22</f>
-        <v>1493</v>
-      </c>
-      <c r="E22" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D22/D$14,0)</f>
-        <v>0.0244246386200488</v>
-      </c>
-      <c r="F22" s="8" t="n">
-        <f aca="false">B22</f>
-        <v>1493</v>
-      </c>
-      <c r="G22" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F22/F$14,0)</f>
-        <v>0.0223007570009141</v>
+      <c r="A22" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B22" s="20" t="n">
+        <f aca="false">B19-B20-B21</f>
+        <v>29158</v>
+      </c>
+      <c r="C22" s="20" t="n">
+        <f aca="false">C19-C20-C21</f>
+        <v>24992.5714285714</v>
+      </c>
+      <c r="D22" s="24" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C22/C$19,0)</f>
+        <v>0.500858870413632</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <f aca="false">E19-E20-E21</f>
+        <v>31357.3542857143</v>
+      </c>
+      <c r="F22" s="24" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E22/E$19,0)</f>
+        <v>0.598486752128363</v>
+      </c>
+      <c r="G22" s="20" t="n">
+        <f aca="false">G19-G20-G21</f>
+        <v>33529.6628571429</v>
+      </c>
+      <c r="H22" s="24" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G22/G$19,0)</f>
+        <v>0.584299848838807</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B23" s="17" t="n">
-        <v>1295</v>
-      </c>
-      <c r="C23" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B23/B$14,0)</f>
-        <v>0.0222447437130686</v>
-      </c>
-      <c r="D23" s="8" t="n">
-        <f aca="false">B23</f>
-        <v>1295</v>
-      </c>
-      <c r="E23" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D23/D$14,0)</f>
-        <v>0.0211854702029224</v>
-      </c>
-      <c r="F23" s="8" t="n">
-        <f aca="false">B23</f>
-        <v>1295</v>
-      </c>
-      <c r="G23" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F23/F$14,0)</f>
-        <v>0.0193432554026683</v>
+        <v>9364</v>
+      </c>
+      <c r="C23" s="8" t="n">
+        <f aca="false">B23*$B$5/$B$6</f>
+        <v>8026.28571428572</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C23/C$19,0)</f>
+        <v>0.160849251064999</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <f aca="false">C23</f>
+        <v>8026.28571428572</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E23/E$19,0)</f>
+        <v>0.153189762919047</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <f aca="false">C23</f>
+        <v>8026.28571428572</v>
+      </c>
+      <c r="H23" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G23/G$19,0)</f>
+        <v>0.139868913969565</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B24" s="17" t="n">
-        <v>1104</v>
-      </c>
-      <c r="C24" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B24/B$14,0)</f>
-        <v>0.0189638587329944</v>
-      </c>
-      <c r="D24" s="8" t="n">
+        <v>4862</v>
+      </c>
+      <c r="C24" s="8" t="n">
         <f aca="false">B24</f>
-        <v>1104</v>
-      </c>
-      <c r="E24" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D24/D$14,0)</f>
-        <v>0.018060817840947</v>
-      </c>
-      <c r="F24" s="8" t="n">
-        <f aca="false">B24</f>
-        <v>1104</v>
-      </c>
-      <c r="G24" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F24/F$14,0)</f>
-        <v>0.0164903119417342</v>
+        <v>4862</v>
+      </c>
+      <c r="D24" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C24/C$19,0)</f>
+        <v>0.0974359855251706</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <f aca="false">C24</f>
+        <v>4862</v>
+      </c>
+      <c r="F24" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E24/E$19,0)</f>
+        <v>0.0927961766906387</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <f aca="false">C24</f>
+        <v>4862</v>
+      </c>
+      <c r="H24" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G24/G$19,0)</f>
+        <v>0.084726943934931</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B25" s="17" t="n">
-        <v>1011</v>
-      </c>
-      <c r="C25" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B25/B$14,0)</f>
-        <v>0.0173663597636389</v>
-      </c>
-      <c r="D25" s="8" t="n">
-        <f aca="false">B25</f>
-        <v>1011</v>
-      </c>
-      <c r="E25" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D25/D$14,0)</f>
-        <v>0.0165393902510846</v>
-      </c>
-      <c r="F25" s="8" t="n">
-        <f aca="false">B25</f>
-        <v>1011</v>
-      </c>
-      <c r="G25" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F25/F$14,0)</f>
-        <v>0.0151011824031642</v>
+        <v>1514</v>
+      </c>
+      <c r="C25" s="8" t="n">
+        <f aca="false">B25*$B$5/$B$6</f>
+        <v>1297.71428571429</v>
+      </c>
+      <c r="D25" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C25/C$19,0)</f>
+        <v>0.0260065961247767</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <f aca="false">C25</f>
+        <v>1297.71428571429</v>
+      </c>
+      <c r="F25" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E25/E$19,0)</f>
+        <v>0.0247681867855016</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <f aca="false">C25</f>
+        <v>1297.71428571429</v>
+      </c>
+      <c r="H25" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G25/G$19,0)</f>
+        <v>0.0226144314128493</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B26" s="17" t="n">
-        <v>778</v>
-      </c>
-      <c r="C26" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B26/B$14,0)</f>
-        <v>0.0133640236361138</v>
-      </c>
-      <c r="D26" s="8" t="n">
-        <f aca="false">B26</f>
-        <v>778</v>
-      </c>
-      <c r="E26" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D26/D$14,0)</f>
-        <v>0.0127276415582036</v>
-      </c>
-      <c r="F26" s="8" t="n">
-        <f aca="false">B26</f>
-        <v>778</v>
-      </c>
-      <c r="G26" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F26/F$14,0)</f>
-        <v>0.0116208901183598</v>
+        <v>1510</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <f aca="false">B26*$B$5/$B$6</f>
+        <v>1294.28571428571</v>
+      </c>
+      <c r="D26" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C26/C$19,0)</f>
+        <v>0.0259378864916861</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <f aca="false">C26</f>
+        <v>1294.28571428571</v>
+      </c>
+      <c r="F26" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E26/E$19,0)</f>
+        <v>0.0247027490397011</v>
+      </c>
+      <c r="G26" s="8" t="n">
+        <f aca="false">C26</f>
+        <v>1294.28571428571</v>
+      </c>
+      <c r="H26" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G26/G$19,0)</f>
+        <v>0.022554683905814</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B27" s="17" t="n">
-        <v>738</v>
-      </c>
-      <c r="C27" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B27/B$14,0)</f>
-        <v>0.0126769273052082</v>
-      </c>
-      <c r="D27" s="8" t="n">
+        <v>1493</v>
+      </c>
+      <c r="C27" s="8" t="n">
         <f aca="false">B27</f>
-        <v>738</v>
-      </c>
-      <c r="E27" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D27/D$14,0)</f>
-        <v>0.0120732641001983</v>
-      </c>
-      <c r="F27" s="8" t="n">
-        <f aca="false">B27</f>
-        <v>738</v>
-      </c>
-      <c r="G27" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F27/F$14,0)</f>
-        <v>0.0110234150480071</v>
+        <v>1493</v>
+      </c>
+      <c r="D27" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C27/C$19,0)</f>
+        <v>0.0299201823095598</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <f aca="false">C27</f>
+        <v>1493</v>
+      </c>
+      <c r="F27" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E27/E$19,0)</f>
+        <v>0.0284954117233903</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <f aca="false">C27</f>
+        <v>1493</v>
+      </c>
+      <c r="H27" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G27/G$19,0)</f>
+        <v>0.0260175498343998</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B28" s="17" t="n">
-        <v>685</v>
-      </c>
-      <c r="C28" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B28/B$14,0)</f>
-        <v>0.0117665246667583</v>
-      </c>
-      <c r="D28" s="8" t="n">
-        <f aca="false">B28</f>
-        <v>685</v>
-      </c>
-      <c r="E28" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D28/D$14,0)</f>
-        <v>0.0112062139683412</v>
-      </c>
-      <c r="F28" s="8" t="n">
-        <f aca="false">B28</f>
-        <v>685</v>
-      </c>
-      <c r="G28" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F28/F$14,0)</f>
-        <v>0.0102317605797898</v>
+        <v>1295</v>
+      </c>
+      <c r="C28" s="8" t="n">
+        <f aca="false">B28*$B$5/$B$6</f>
+        <v>1110</v>
+      </c>
+      <c r="D28" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C28/C$19,0)</f>
+        <v>0.0222447437130686</v>
+      </c>
+      <c r="E28" s="8" t="n">
+        <f aca="false">C28</f>
+        <v>1110</v>
+      </c>
+      <c r="F28" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E28/E$19,0)</f>
+        <v>0.0211854702029224</v>
+      </c>
+      <c r="G28" s="8" t="n">
+        <f aca="false">C28</f>
+        <v>1110</v>
+      </c>
+      <c r="H28" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G28/G$19,0)</f>
+        <v>0.0193432554026683</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B29" s="17" t="n">
-        <v>512</v>
-      </c>
-      <c r="C29" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B29/B$14,0)</f>
-        <v>0.00879483303559159</v>
-      </c>
-      <c r="D29" s="8" t="n">
-        <f aca="false">B29</f>
-        <v>512</v>
-      </c>
-      <c r="E29" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D29/D$14,0)</f>
-        <v>0.00837603146246818</v>
-      </c>
-      <c r="F29" s="8" t="n">
-        <f aca="false">B29</f>
-        <v>512</v>
-      </c>
-      <c r="G29" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F29/F$14,0)</f>
-        <v>0.00764768090051443</v>
+        <v>1104</v>
+      </c>
+      <c r="C29" s="8" t="n">
+        <f aca="false">B29*$B$5/$B$6</f>
+        <v>946.285714285714</v>
+      </c>
+      <c r="D29" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C29/C$19,0)</f>
+        <v>0.0189638587329944</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <f aca="false">C29</f>
+        <v>946.285714285714</v>
+      </c>
+      <c r="F29" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E29/E$19,0)</f>
+        <v>0.018060817840947</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <f aca="false">C29</f>
+        <v>946.285714285714</v>
+      </c>
+      <c r="H29" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G29/G$19,0)</f>
+        <v>0.0164903119417342</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="19" t="s">
-        <v>181</v>
-      </c>
-      <c r="B30" s="20" t="n">
-        <f aca="false">B17-SUM(B18:B29)</f>
-        <v>4292</v>
-      </c>
-      <c r="C30" s="24" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B30/B$14,0)</f>
-        <v>0.0737254363061701</v>
-      </c>
-      <c r="D30" s="20" t="n">
-        <f aca="false">D17-SUM(D18:D29)</f>
-        <v>11802.8</v>
-      </c>
-      <c r="E30" s="24" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D30/D$14,0)</f>
-        <v>0.193087156533632</v>
-      </c>
-      <c r="F30" s="20" t="n">
-        <f aca="false">F17-SUM(F18:F29)</f>
-        <v>14251.94</v>
-      </c>
-      <c r="G30" s="24" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F30/F$14,0)</f>
-        <v>0.212879471354058</v>
+      <c r="A30" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="B30" s="17" t="n">
+        <v>1011</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <f aca="false">B30*$B$5/$B$6</f>
+        <v>866.571428571429</v>
+      </c>
+      <c r="D30" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C30/C$19,0)</f>
+        <v>0.0173663597636389</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <f aca="false">C30</f>
+        <v>866.571428571429</v>
+      </c>
+      <c r="F30" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E30/E$19,0)</f>
+        <v>0.0165393902510846</v>
+      </c>
+      <c r="G30" s="8" t="n">
+        <f aca="false">C30</f>
+        <v>866.571428571429</v>
+      </c>
+      <c r="H30" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G30/G$19,0)</f>
+        <v>0.0151011824031642</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="B31" s="8" t="n">
-        <f aca="false">-$B$9*$B$11</f>
-        <v>-2166.66666666667</v>
-      </c>
-      <c r="C31" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B31/B$14,0)</f>
-        <v>-0.037217717924053</v>
-      </c>
-      <c r="D31" s="8" t="n">
-        <f aca="false">-$B$9*$B$11</f>
-        <v>-2166.66666666667</v>
-      </c>
-      <c r="E31" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D31/D$14,0)</f>
-        <v>-0.0354454456419552</v>
-      </c>
-      <c r="F31" s="8" t="n">
-        <f aca="false">-$B$9*$B$11</f>
-        <v>-2166.66666666667</v>
-      </c>
-      <c r="G31" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F31/F$14,0)</f>
-        <v>-0.0323632329774374</v>
+        <v>185</v>
+      </c>
+      <c r="B31" s="17" t="n">
+        <v>778</v>
+      </c>
+      <c r="C31" s="8" t="n">
+        <f aca="false">B31*$B$5/$B$6</f>
+        <v>666.857142857143</v>
+      </c>
+      <c r="D31" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C31/C$19,0)</f>
+        <v>0.0133640236361138</v>
+      </c>
+      <c r="E31" s="8" t="n">
+        <f aca="false">C31</f>
+        <v>666.857142857143</v>
+      </c>
+      <c r="F31" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E31/E$19,0)</f>
+        <v>0.0127276415582036</v>
+      </c>
+      <c r="G31" s="8" t="n">
+        <f aca="false">C31</f>
+        <v>666.857142857143</v>
+      </c>
+      <c r="H31" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G31/G$19,0)</f>
+        <v>0.0116208901183598</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
-        <v>183</v>
-      </c>
-      <c r="B32" s="23" t="n">
-        <f aca="false">B30+B31</f>
-        <v>2125.33333333333</v>
-      </c>
-      <c r="C32" s="24" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B32/B$14,0)</f>
-        <v>0.0365077183821172</v>
-      </c>
-      <c r="D32" s="23" t="n">
-        <f aca="false">D30+D31</f>
-        <v>9636.13333333334</v>
-      </c>
-      <c r="E32" s="24" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D32/D$14,0)</f>
-        <v>0.157641710891677</v>
-      </c>
-      <c r="F32" s="23" t="n">
-        <f aca="false">F30+F31</f>
-        <v>12085.2733333333</v>
-      </c>
-      <c r="G32" s="24" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F32/F$14,0)</f>
-        <v>0.18051623837662</v>
+      <c r="A32" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="B32" s="17" t="n">
+        <v>738</v>
+      </c>
+      <c r="C32" s="8" t="n">
+        <f aca="false">B32*$B$5/$B$6</f>
+        <v>632.571428571429</v>
+      </c>
+      <c r="D32" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C32/C$19,0)</f>
+        <v>0.0126769273052082</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <f aca="false">C32</f>
+        <v>632.571428571429</v>
+      </c>
+      <c r="F32" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E32/E$19,0)</f>
+        <v>0.0120732641001983</v>
+      </c>
+      <c r="G32" s="8" t="n">
+        <f aca="false">C32</f>
+        <v>632.571428571429</v>
+      </c>
+      <c r="H32" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G32/G$19,0)</f>
+        <v>0.0110234150480071</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="B33" s="8" t="n">
-        <f aca="false">-$B$10</f>
+        <v>187</v>
+      </c>
+      <c r="B33" s="17" t="n">
+        <v>685</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <f aca="false">B33*$B$5/$B$6</f>
+        <v>587.142857142857</v>
+      </c>
+      <c r="D33" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C33/C$19,0)</f>
+        <v>0.0117665246667583</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <f aca="false">C33</f>
+        <v>587.142857142857</v>
+      </c>
+      <c r="F33" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E33/E$19,0)</f>
+        <v>0.0112062139683412</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <f aca="false">C33</f>
+        <v>587.142857142857</v>
+      </c>
+      <c r="H33" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G33/G$19,0)</f>
+        <v>0.0102317605797898</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B34" s="17" t="n">
+        <v>512</v>
+      </c>
+      <c r="C34" s="8" t="n">
+        <f aca="false">B34*$B$5/$B$6</f>
+        <v>438.857142857143</v>
+      </c>
+      <c r="D34" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C34/C$19,0)</f>
+        <v>0.00879483303559159</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <f aca="false">C34</f>
+        <v>438.857142857143</v>
+      </c>
+      <c r="F34" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E34/E$19,0)</f>
+        <v>0.00837603146246818</v>
+      </c>
+      <c r="G34" s="8" t="n">
+        <f aca="false">C34</f>
+        <v>438.857142857143</v>
+      </c>
+      <c r="H34" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G34/G$19,0)</f>
+        <v>0.00764768090051443</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="B35" s="20" t="n">
+        <f aca="false">B22-SUM(B23:B34)</f>
+        <v>4292</v>
+      </c>
+      <c r="C35" s="20" t="n">
+        <f aca="false">C22-SUM(C23:C34)</f>
+        <v>2771</v>
+      </c>
+      <c r="D35" s="24" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C35/C$19,0)</f>
+        <v>0.0555316980440658</v>
+      </c>
+      <c r="E35" s="20" t="n">
+        <f aca="false">E22-SUM(E23:E34)</f>
+        <v>9135.78285714286</v>
+      </c>
+      <c r="F35" s="24" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E35/E$19,0)</f>
+        <v>0.174365635585919</v>
+      </c>
+      <c r="G35" s="20" t="n">
+        <f aca="false">G22-SUM(G23:G34)</f>
+        <v>11308.0914285714</v>
+      </c>
+      <c r="H35" s="24" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G35/G$19,0)</f>
+        <v>0.19705882938701</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="B36" s="8" t="n">
+        <f aca="false">-$B$14*$B$16</f>
+        <v>-2166.66666666667</v>
+      </c>
+      <c r="C36" s="8" t="n">
+        <f aca="false">-$B$14*$B$16</f>
+        <v>-2166.66666666667</v>
+      </c>
+      <c r="D36" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C36/C$19,0)</f>
+        <v>-0.0434206709113951</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <f aca="false">-$B$14*$B$16</f>
+        <v>-2166.66666666667</v>
+      </c>
+      <c r="F36" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E36/E$19,0)</f>
+        <v>-0.0413530199156144</v>
+      </c>
+      <c r="G36" s="8" t="n">
+        <f aca="false">-$B$14*$B$16</f>
+        <v>-2166.66666666667</v>
+      </c>
+      <c r="H36" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G36/G$19,0)</f>
+        <v>-0.0377571051403436</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="B37" s="23" t="n">
+        <f aca="false">B35+B36</f>
+        <v>2125.33333333333</v>
+      </c>
+      <c r="C37" s="23" t="n">
+        <f aca="false">C35+C36</f>
+        <v>604.333333333334</v>
+      </c>
+      <c r="D37" s="24" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C37/C$19,0)</f>
+        <v>0.0121110271326707</v>
+      </c>
+      <c r="E37" s="23" t="n">
+        <f aca="false">E35+E36</f>
+        <v>6969.11619047619</v>
+      </c>
+      <c r="F37" s="24" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E37/E$19,0)</f>
+        <v>0.133012615670304</v>
+      </c>
+      <c r="G37" s="23" t="n">
+        <f aca="false">G35+G36</f>
+        <v>9141.42476190476</v>
+      </c>
+      <c r="H37" s="24" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G37/G$19,0)</f>
+        <v>0.159301724246667</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B38" s="8" t="n">
+        <f aca="false">-$B$15</f>
         <v>-2900</v>
       </c>
-      <c r="C33" s="18" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B33/B$14,0)</f>
-        <v>-0.0498144839906555</v>
-      </c>
-      <c r="D33" s="8" t="n">
-        <f aca="false">-$B$10</f>
+      <c r="C38" s="8" t="n">
+        <f aca="false">-$B$15</f>
         <v>-2900</v>
       </c>
-      <c r="E33" s="18" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D33/D$14,0)</f>
-        <v>-0.0474423657053862</v>
-      </c>
-      <c r="F33" s="8" t="n">
-        <f aca="false">-$B$10</f>
+      <c r="D38" s="18" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C38/C$19,0)</f>
+        <v>-0.0581168979890981</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <f aca="false">-$B$15</f>
         <v>-2900</v>
       </c>
-      <c r="G33" s="18" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F33/F$14,0)</f>
-        <v>-0.04331694260057</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="19" t="s">
-        <v>185</v>
-      </c>
-      <c r="B34" s="20" t="n">
-        <f aca="false">B32+B33</f>
+      <c r="F38" s="18" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E38/E$19,0)</f>
+        <v>-0.0553494266562839</v>
+      </c>
+      <c r="G38" s="8" t="n">
+        <f aca="false">-$B$15</f>
+        <v>-2900</v>
+      </c>
+      <c r="H38" s="18" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G38/G$19,0)</f>
+        <v>-0.0505364330339983</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="B39" s="20" t="n">
+        <f aca="false">B37+B38</f>
         <v>-774.666666666667</v>
       </c>
-      <c r="C34" s="24" t="n">
-        <f aca="false">IF(B$14&lt;&gt;0,B34/B$14,0)</f>
-        <v>-0.0133067656085383</v>
-      </c>
-      <c r="D34" s="20" t="n">
-        <f aca="false">D32+D33</f>
-        <v>6736.13333333334</v>
-      </c>
-      <c r="E34" s="24" t="n">
-        <f aca="false">IF(D$14&lt;&gt;0,D34/D$14,0)</f>
-        <v>0.11019934518629</v>
-      </c>
-      <c r="F34" s="20" t="n">
-        <f aca="false">F32+F33</f>
-        <v>9185.27333333333</v>
-      </c>
-      <c r="G34" s="24" t="n">
-        <f aca="false">IF(F$14&lt;&gt;0,F34/F$14,0)</f>
-        <v>0.13719929577605</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="28" t="s">
-        <v>186</v>
-      </c>
-      <c r="B36" s="32" t="n">
-        <f aca="false">IF(B14&gt;0,(SUM(B18:B29)-B31)/(1-(B15+B16)/B14),0)</f>
+      <c r="C39" s="20" t="n">
+        <f aca="false">C37+C38</f>
+        <v>-2295.66666666667</v>
+      </c>
+      <c r="D39" s="24" t="n">
+        <f aca="false">IF(C$19&lt;&gt;0,C39/C$19,0)</f>
+        <v>-0.0460058708564274</v>
+      </c>
+      <c r="E39" s="20" t="n">
+        <f aca="false">E37+E38</f>
+        <v>4069.11619047619</v>
+      </c>
+      <c r="F39" s="24" t="n">
+        <f aca="false">IF(E$19&lt;&gt;0,E39/E$19,0)</f>
+        <v>0.0776631890140204</v>
+      </c>
+      <c r="G39" s="20" t="n">
+        <f aca="false">G37+G38</f>
+        <v>6241.42476190476</v>
+      </c>
+      <c r="H39" s="24" t="n">
+        <f aca="false">IF(G$19&lt;&gt;0,G39/G$19,0)</f>
+        <v>0.108765291212669</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="28" t="s">
+        <v>194</v>
+      </c>
+      <c r="B41" s="32" t="n">
+        <f aca="false">IF(B19&gt;0,(SUM(B23:B34)-B36)/(1-(B20+B21)/B19),0)</f>
         <v>53972.6223563573</v>
       </c>
-      <c r="D36" s="32" t="n">
-        <f aca="false">IF(D14&gt;0,(SUM(D18:D29)-D31)/(1-(D15+D16)/D14),0)</f>
-        <v>45063.3892791692</v>
-      </c>
-      <c r="F36" s="32" t="n">
-        <f aca="false">IF(F14&gt;0,(SUM(F18:F29)-F31)/(1-(F15+F16)/F14),0)</f>
-        <v>46265.0584633717</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="28" t="s">
-        <v>187</v>
-      </c>
-      <c r="B37" s="32" t="n">
-        <f aca="false">IF(B14&gt;0,(SUM(B18:B29)-B31-B33)/(1-(B15+B16)/B14),0)</f>
+      <c r="C41" s="32" t="n">
+        <f aca="false">IF(C19&gt;0,(SUM(C23:C34)-C36)/(1-(C20+C21)/C19),0)</f>
+        <v>48692.8345206249</v>
+      </c>
+      <c r="E41" s="32" t="n">
+        <f aca="false">IF(E19&gt;0,(SUM(E23:E34)-E36)/(1-(E20+E21)/E19),0)</f>
+        <v>40749.8378343508</v>
+      </c>
+      <c r="G41" s="32" t="n">
+        <f aca="false">IF(G19&gt;0,(SUM(G23:G34)-G36)/(1-(G20+G21)/G19),0)</f>
+        <v>41739.2510775168</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="28" t="s">
+        <v>195</v>
+      </c>
+      <c r="B42" s="32" t="n">
+        <f aca="false">IF(B19&gt;0,(SUM(B23:B34)-B36-B38)/(1-(B20+B21)/B19),0)</f>
         <v>59762.6765438873</v>
       </c>
-      <c r="D37" s="32" t="n">
-        <f aca="false">IF(D14&gt;0,(SUM(D18:D29)-D31-D33)/(1-(D15+D16)/D14),0)</f>
-        <v>49897.682193036</v>
-      </c>
-      <c r="F37" s="32" t="n">
-        <f aca="false">IF(F14&gt;0,(SUM(F18:F29)-F31-F33)/(1-(F15+F16)/F14),0)</f>
-        <v>51228.2635810236</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="B41" s="8" t="n">
-        <f aca="false">B14*6</f>
+      <c r="C42" s="32" t="n">
+        <f aca="false">IF(C19&gt;0,(SUM(C23:C34)-C36-C38)/(1-(C20+C21)/C19),0)</f>
+        <v>54482.8887081549</v>
+      </c>
+      <c r="E42" s="32" t="n">
+        <f aca="false">IF(E19&gt;0,(SUM(E23:E34)-E36-E38)/(1-(E20+E21)/E19),0)</f>
+        <v>45595.3920420035</v>
+      </c>
+      <c r="G42" s="32" t="n">
+        <f aca="false">IF(G19&gt;0,(SUM(G23:G34)-G36-G38)/(1-(G20+G21)/G19),0)</f>
+        <v>46702.4561951687</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="B46" s="8" t="n">
+        <f aca="false">B19*$B$5</f>
         <v>349296</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="B42" s="7" t="n">
+      <c r="D46" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B47" s="7" t="n">
+        <f aca="false">SUM('Mois par mois'!C5:C11)</f>
+        <v>361223.56</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="B48" s="8" t="n">
+        <f aca="false">B46-B47</f>
+        <v>-11927.56</v>
+      </c>
+      <c r="C48" s="18" t="n">
+        <f aca="false">IF(B47&gt;0,B48/B47,0)</f>
+        <v>-0.0330198838636107</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B49" s="7" t="n">
         <f aca="false">SUM('Mois par mois'!C6:C11)</f>
         <v>312456.22</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="B43" s="8" t="n">
-        <f aca="false">B41-B42</f>
-        <v>36839.78</v>
-      </c>
-      <c r="C43" s="18" t="n">
-        <f aca="false">IF(B42&gt;0,B43/B42,0)</f>
-        <v>0.117903813852706</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="B44" s="7" t="n">
-        <f aca="false">SUM('Mois par mois'!C5:C11)+6506.85</f>
-        <v>367730.41</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="B47" s="17" t="n">
-        <v>-22600</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="B48" s="17" t="n">
-        <v>-31800</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="B49" s="17" t="n">
-        <v>-6200</v>
-      </c>
-    </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="B50" s="17" t="n">
-        <v>25800</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="B51" s="17" t="n">
-        <v>-13400</v>
+        <v>203</v>
+      </c>
+      <c r="B50" s="8" t="n">
+        <f aca="false">B46-B49</f>
+        <v>36839.78</v>
+      </c>
+      <c r="C50" s="18" t="n">
+        <f aca="false">IF(B49&gt;0,B50/B49,0)</f>
+        <v>0.117903813852706</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="B52" s="17" t="n">
-        <v>-11900</v>
+      <c r="A52" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B52" s="48" t="s">
+        <v>205</v>
+      </c>
+      <c r="C52" s="48" t="s">
+        <v>206</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G52" s="17" t="n">
+        <v>5300</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="19" t="s">
-        <v>203</v>
-      </c>
-      <c r="B53" s="20" t="n">
-        <f aca="false">SUM(B47:B52)</f>
-        <v>-60100</v>
+      <c r="A53" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="B53" s="17" t="n">
+        <v>-22600</v>
+      </c>
+      <c r="C53" s="8" t="n">
+        <f aca="false">B53</f>
+        <v>-22600</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="G53" s="47" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B54" s="17" t="n">
+        <v>-31800</v>
+      </c>
+      <c r="C54" s="8" t="n">
+        <f aca="false">-$G$52*$G$53</f>
+        <v>-26500</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="B55" s="17" t="n">
+        <v>-6200</v>
+      </c>
+      <c r="C55" s="8" t="n">
+        <f aca="false">B55</f>
+        <v>-6200</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="B56" s="17" t="n">
+        <v>25800</v>
+      </c>
+      <c r="C56" s="8" t="n">
+        <f aca="false">C35*$B$6</f>
+        <v>19397</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="B57" s="17" t="n">
+        <v>-13400</v>
+      </c>
+      <c r="C57" s="8" t="n">
+        <f aca="false">B57</f>
+        <v>-13400</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="B58" s="17" t="n">
+        <v>-11900</v>
+      </c>
+      <c r="C58" s="8" t="n">
+        <f aca="false">B58</f>
+        <v>-11900</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="B59" s="20" t="n">
+        <f aca="false">SUM(B53:B58)</f>
+        <v>-60100</v>
+      </c>
+      <c r="C59" s="20" t="n">
+        <f aca="false">SUM(C53:C58)</f>
+        <v>-61203</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="B60" s="17" t="n">
         <v>-59900</v>
       </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="35" t="s">
-        <v>206</v>
-      </c>
-      <c r="B57" s="35"/>
-      <c r="C57" s="35"/>
-      <c r="D57" s="35"/>
-      <c r="E57" s="35"/>
-      <c r="F57" s="35"/>
-      <c r="G57" s="35"/>
-    </row>
-    <row r="58" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="35" t="s">
-        <v>207</v>
-      </c>
-      <c r="B58" s="35"/>
-      <c r="C58" s="35"/>
-      <c r="D58" s="35"/>
-      <c r="E58" s="35"/>
-      <c r="F58" s="35"/>
-      <c r="G58" s="35"/>
-    </row>
-    <row r="59" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="35" t="s">
-        <v>208</v>
-      </c>
-      <c r="B59" s="35"/>
-      <c r="C59" s="35"/>
-      <c r="D59" s="35"/>
-      <c r="E59" s="35"/>
-      <c r="F59" s="35"/>
-      <c r="G59" s="35"/>
-    </row>
-    <row r="60" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="35" t="s">
-        <v>209</v>
-      </c>
-      <c r="B60" s="35"/>
-      <c r="C60" s="35"/>
-      <c r="D60" s="35"/>
-      <c r="E60" s="35"/>
-      <c r="F60" s="35"/>
-      <c r="G60" s="35"/>
-    </row>
-    <row r="61" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="B61" s="35"/>
-      <c r="C61" s="35"/>
-      <c r="D61" s="35"/>
-      <c r="E61" s="35"/>
-      <c r="F61" s="35"/>
-      <c r="G61" s="35"/>
+      <c r="C60" s="8" t="n">
+        <f aca="false">B60</f>
+        <v>-59900</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="3" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="35" t="s">
+        <v>218</v>
+      </c>
+      <c r="B63" s="35"/>
+      <c r="C63" s="35"/>
+      <c r="D63" s="35"/>
+      <c r="E63" s="35"/>
+      <c r="F63" s="35"/>
+      <c r="G63" s="35"/>
+      <c r="H63" s="35"/>
+    </row>
+    <row r="64" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="35" t="s">
+        <v>219</v>
+      </c>
+      <c r="B64" s="35"/>
+      <c r="C64" s="35"/>
+      <c r="D64" s="35"/>
+      <c r="E64" s="35"/>
+      <c r="F64" s="35"/>
+      <c r="G64" s="35"/>
+      <c r="H64" s="35"/>
+    </row>
+    <row r="65" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="35" t="s">
+        <v>220</v>
+      </c>
+      <c r="B65" s="35"/>
+      <c r="C65" s="35"/>
+      <c r="D65" s="35"/>
+      <c r="E65" s="35"/>
+      <c r="F65" s="35"/>
+      <c r="G65" s="35"/>
+      <c r="H65" s="35"/>
+    </row>
+    <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="35" t="s">
+        <v>221</v>
+      </c>
+      <c r="B66" s="35"/>
+      <c r="C66" s="35"/>
+      <c r="D66" s="35"/>
+      <c r="E66" s="35"/>
+      <c r="F66" s="35"/>
+      <c r="G66" s="35"/>
+      <c r="H66" s="35"/>
+    </row>
+    <row r="67" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="35" t="s">
+        <v>222</v>
+      </c>
+      <c r="B67" s="35"/>
+      <c r="C67" s="35"/>
+      <c r="D67" s="35"/>
+      <c r="E67" s="35"/>
+      <c r="F67" s="35"/>
+      <c r="G67" s="35"/>
+      <c r="H67" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A57:G57"/>
-    <mergeCell ref="A58:G58"/>
-    <mergeCell ref="A59:G59"/>
-    <mergeCell ref="A60:G60"/>
-    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A65:H65"/>
+    <mergeCell ref="A66:H66"/>
+    <mergeCell ref="A67:H67"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4474,7 +4705,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4497,12 +4727,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4510,59 +4740,59 @@
         <v>115</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B5" s="7" t="n">
-        <f aca="false">AVERAGE('Mois par mois'!C6:C11)</f>
-        <v>52076.0366666667</v>
+        <f aca="false">AVERAGE('Mois par mois'!C5:C11)</f>
+        <v>51603.3657142857</v>
       </c>
       <c r="D5" s="7" t="n">
-        <f aca="false">'Compte d’exploitation'!B14</f>
-        <v>58216</v>
+        <f aca="false">'Compte d’exploitation'!C19</f>
+        <v>49899.4285714286</v>
       </c>
       <c r="F5" s="23" t="n">
         <f aca="false">D5-B5</f>
-        <v>6139.96333333334</v>
+        <v>-1703.93714285714</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="B6" s="7" t="n">
-        <f aca="false">SUMPRODUCT('Mois par mois'!C6:C11,'Mois par mois'!T6:T11)/6</f>
-        <v>19293.28865</v>
+        <f aca="false">SUMPRODUCT('Mois par mois'!C5:C11,'Mois par mois'!T5:T11)/7</f>
+        <v>19309.8761742857</v>
       </c>
       <c r="C6" s="18" t="n">
         <f aca="false">IF(B$5&gt;0,B6/B$5,0)</f>
-        <v>0.370483045272711</v>
+        <v>0.374197998657673</v>
       </c>
       <c r="D6" s="7" t="n">
-        <f aca="false">'Compte d’exploitation'!B15+'Compte d’exploitation'!B16</f>
-        <v>29058</v>
+        <f aca="false">'Compte d’exploitation'!C20+'Compte d’exploitation'!C21</f>
+        <v>24906.8571428571</v>
       </c>
       <c r="E6" s="18" t="n">
         <f aca="false">IF(D$5&gt;0,D6/D$5,0)</f>
@@ -4570,27 +4800,27 @@
       </c>
       <c r="F6" s="8" t="n">
         <f aca="false">D6-B6</f>
-        <v>9764.71135</v>
+        <v>5596.98096857143</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B5-B6</f>
-        <v>32782.7480166667</v>
+        <v>32293.48954</v>
       </c>
       <c r="C7" s="18" t="n">
         <f aca="false">IF(B$5&gt;0,B7/B$5,0)</f>
-        <v>0.62951695472729</v>
+        <v>0.625802001342327</v>
       </c>
       <c r="D7" s="8" t="n">
         <f aca="false">D5-D6</f>
-        <v>29158</v>
+        <v>24992.5714285714</v>
       </c>
       <c r="E7" s="18" t="n">
         <f aca="false">IF(D$5&gt;0,D7/D$5,0)</f>
@@ -4598,25 +4828,25 @@
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">D7-B7</f>
-        <v>-3624.74801666666</v>
+        <v>-7300.91811142857</v>
       </c>
       <c r="G7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="B8" s="7" t="n">
-        <f aca="false">AVERAGE('Mois par mois'!U6:U11)</f>
-        <v>8394.16666666667</v>
+        <f aca="false">AVERAGE('Mois par mois'!U5:U11)</f>
+        <v>8099.85714285714</v>
       </c>
       <c r="C8" s="18" t="n">
         <f aca="false">IF(B$5&gt;0,B8/B$5,0)</f>
-        <v>0.161190582155798</v>
+        <v>0.156963737359767</v>
       </c>
       <c r="D8" s="7" t="n">
-        <f aca="false">'Compte d’exploitation'!B18</f>
-        <v>9364</v>
+        <f aca="false">'Compte d’exploitation'!C23</f>
+        <v>8026.28571428572</v>
       </c>
       <c r="E8" s="18" t="n">
         <f aca="false">IF(D$5&gt;0,D8/D$5,0)</f>
@@ -4624,10 +4854,10 @@
       </c>
       <c r="F8" s="8" t="n">
         <f aca="false">D8-B8</f>
-        <v>969.833333333334</v>
+        <v>-73.5714285714284</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4635,152 +4865,152 @@
         <v>138</v>
       </c>
       <c r="B9" s="7" t="n">
-        <f aca="false">AVERAGE('Mois par mois'!P6:P11)</f>
-        <v>13154.8633333333</v>
+        <f aca="false">AVERAGE('Mois par mois'!P5:P11)</f>
+        <v>12612.6714285714</v>
       </c>
       <c r="C9" s="18" t="n">
         <f aca="false">IF(B$5&gt;0,B9/B$5,0)</f>
-        <v>0.252608765477608</v>
+        <v>0.244415674326448</v>
       </c>
       <c r="D9" s="7" t="n">
-        <f aca="false">SUM('Compte d’exploitation'!B19:B29)</f>
-        <v>15502</v>
+        <f aca="false">SUM('Compte d’exploitation'!C24:C34)</f>
+        <v>14195.2857142857</v>
       </c>
       <c r="E9" s="18" t="n">
         <f aca="false">IF(D$5&gt;0,D9/D$5,0)</f>
-        <v>0.266284183042463</v>
+        <v>0.284477921304567</v>
       </c>
       <c r="F9" s="8" t="n">
         <f aca="false">D9-B9</f>
-        <v>2347.13666666667</v>
+        <v>1582.61428571429</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">B7-B8-B9</f>
-        <v>11233.7180166667</v>
+        <v>11580.9609685714</v>
       </c>
       <c r="C10" s="18" t="n">
         <f aca="false">IF(B$5&gt;0,B10/B$5,0)</f>
-        <v>0.215717607093883</v>
+        <v>0.224422589656112</v>
       </c>
       <c r="D10" s="8" t="n">
         <f aca="false">D7-D8-D9</f>
-        <v>4292</v>
+        <v>2771</v>
       </c>
       <c r="E10" s="18" t="n">
         <f aca="false">IF(D$5&gt;0,D10/D$5,0)</f>
-        <v>0.0737254363061701</v>
+        <v>0.0555316980440658</v>
       </c>
       <c r="F10" s="23" t="n">
         <f aca="false">D10-B10</f>
-        <v>-6941.71801666667</v>
+        <v>-8809.96096857143</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B5&gt;0,(B8+B9)/(1-B6/B5),0)</f>
-        <v>34231.0557931441</v>
+        <v>33097.5748351728</v>
       </c>
       <c r="D11" s="8" t="n">
         <f aca="false">IF(D5&gt;0,(D8+D9)/(1-D6/D5),0)</f>
-        <v>49646.7198024556</v>
+        <v>44366.9319667232</v>
       </c>
       <c r="F11" s="8" t="n">
         <f aca="false">D11-B11</f>
-        <v>15415.6640093115</v>
+        <v>11269.3571315504</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="B12" s="9" t="n">
-        <f aca="false">AVERAGE('Mois par mois'!F6:F11)</f>
-        <v>4218</v>
+        <f aca="false">AVERAGE('Mois par mois'!F5:F11)</f>
+        <v>4235.57142857143</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">IF(B12&gt;0,B5/B12,0)</f>
-        <v>12.3461443021969</v>
+        <v>12.1833302978178</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B10</f>
-        <v>11233.7180166667</v>
+        <v>11580.9609685714</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">D5-B5</f>
-        <v>6139.96333333334</v>
+        <v>-1703.93714285714</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">-(D6-B6)</f>
-        <v>-9764.71135</v>
+        <v>-5596.98096857143</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-(D8-B8)</f>
-        <v>-969.833333333334</v>
+        <v>73.5714285714284</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">-(D9-B9)</f>
-        <v>-2347.13666666667</v>
+        <v>-1582.61428571429</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="B21" s="20" t="n">
         <f aca="false">SUM(B16:B20)</f>
-        <v>4292.00000000001</v>
+        <v>2771</v>
       </c>
       <c r="C21" s="2" t="str">
         <f aca="false">IF(ABS(B21-D10)&lt;1,"= bilan","écart")</f>
@@ -4815,27 +5045,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="B4" s="47" t="n">
+        <v>250</v>
+      </c>
+      <c r="B4" s="49" t="n">
         <f aca="false">Récap!B13</f>
         <v>30.4166666666667</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="F4" s="31" t="n">
-        <f aca="false">1-('Compte d’exploitation'!B15+'Compte d’exploitation'!B16)/'Compte d’exploitation'!B14</f>
+        <f aca="false">1-('Compte d’exploitation'!C20+'Compte d’exploitation'!C21)/'Compte d’exploitation'!C19</f>
         <v>0.500858870413632</v>
       </c>
     </row>
@@ -4848,11 +5078,11 @@
         <v>12.1833302978178</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="F5" s="7" t="n">
-        <f aca="false">'Compte d’exploitation'!B32</f>
-        <v>2125.33333333333</v>
+        <f aca="false">'Compte d’exploitation'!C37</f>
+        <v>604.333333333334</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4864,16 +5094,16 @@
         <v>139.197183098592</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="F6" s="7" t="n">
-        <f aca="false">'Compte d’exploitation'!B34</f>
-        <v>-774.666666666667</v>
+        <f aca="false">'Compte d’exploitation'!C39</f>
+        <v>-2295.66666666667</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="B7" s="31" t="n">
         <f aca="false">1-Récap!B31</f>
@@ -4882,7 +5112,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">Récap!B25</f>
@@ -4891,34 +5121,34 @@
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4955,11 +5185,11 @@
       </c>
       <c r="I11" s="23" t="n">
         <f aca="false">$F$5+H11</f>
-        <v>2125.33333333333</v>
+        <v>604.333333333334</v>
       </c>
       <c r="J11" s="23" t="n">
         <f aca="false">$F$6+H11</f>
-        <v>-774.666666666667</v>
+        <v>-2295.66666666667</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4996,11 +5226,11 @@
       </c>
       <c r="I12" s="23" t="n">
         <f aca="false">$F$5+H12</f>
-        <v>2887.05619875407</v>
+        <v>1366.05619875407</v>
       </c>
       <c r="J12" s="23" t="n">
         <f aca="false">$F$6+H12</f>
-        <v>-12.9438012459344</v>
+        <v>-1533.94380124593</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5037,11 +5267,11 @@
       </c>
       <c r="I13" s="23" t="n">
         <f aca="false">$F$5+H13</f>
-        <v>3648.7790641748</v>
+        <v>2127.7790641748</v>
       </c>
       <c r="J13" s="23" t="n">
         <f aca="false">$F$6+H13</f>
-        <v>748.779064174798</v>
+        <v>-772.220935825202</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5078,11 +5308,11 @@
       </c>
       <c r="I14" s="23" t="n">
         <f aca="false">$F$5+H14</f>
-        <v>4410.50192959553</v>
+        <v>2889.50192959553</v>
       </c>
       <c r="J14" s="23" t="n">
         <f aca="false">$F$6+H14</f>
-        <v>1510.50192959553</v>
+        <v>-10.4980704044706</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5119,11 +5349,11 @@
       </c>
       <c r="I15" s="23" t="n">
         <f aca="false">$F$5+H15</f>
-        <v>5172.22479501626</v>
+        <v>3651.22479501626</v>
       </c>
       <c r="J15" s="23" t="n">
         <f aca="false">$F$6+H15</f>
-        <v>2272.22479501626</v>
+        <v>751.224795016262</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5160,16 +5390,16 @@
       </c>
       <c r="I16" s="23" t="n">
         <f aca="false">$F$5+H16</f>
-        <v>5933.94766043699</v>
+        <v>4412.94766043699</v>
       </c>
       <c r="J16" s="23" t="n">
         <f aca="false">$F$6+H16</f>
-        <v>3033.94766043699</v>
+        <v>1512.94766043699</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tableau récap Halle : page 3 avec la seule analyse (sept mois d'exploitation) et le CA qu'il faut pour finir le mois à 0, 5 000 et 10 000 € après Nathan et la banque
Achats et emballages suivent le CA, les autres charges restent les mêmes. Dans l'Excel, les trois résultats visés sont des cases jaunes (feuille « Compte d'exploitation », ligne 18) ; les autres feuilles lisent la colonne Analyse.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfhpzegTMHxDopBcc2QwLH
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
+++ b/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="263">
   <si>
     <t xml:space="preserve">Atelier by – Halle · tableau récap</t>
   </si>
@@ -578,22 +578,37 @@
     <t xml:space="preserve">Le compte d’exploitation comptable, mars → septembre 2026 (à valider)</t>
   </si>
   <si>
-    <t xml:space="preserve">Analyse transmise le 13 octobre 2026, à partir de la situation comptable au 30/09/2026 de la fiduciaire (Pardoen), lissée sur 6 mois (ouverture supposée en avril). Recalcul du 13 octobre : le magasin a ouvert en mars, les totaux de la période se divisent par 7 ; loyer, charges locatives, assurance et honoraires, déjà ramenés à leur coût mensuel par l'analyse, restent tels quels. À valider avec la fiduciaire. En bleu : montants de l’analyse ; fond jaune : paramètres ; en noir : calculs.</t>
+    <t xml:space="preserve">Situation au 30/09/2026 de la fiduciaire (Pardoen), ramenée au mois sur les 7 mois d’exploitation (ouverture en mars) ; loyer, charges locatives, assurance et honoraires à leur coût mensuel. En bleu : montants de l’analyse ; fond jaune : paramètres et résultats visés ; en noir : calculs.</t>
   </si>
   <si>
     <t xml:space="preserve">Paramètres</t>
   </si>
   <si>
-    <t xml:space="preserve">Mois de l’analyse (ouverture supposée en avril)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">la division faite par l’analyse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mois d’exploitation réels (ouverture en mars)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">chaque ligne × mois de l’analyse ÷ mois réels, sauf les coûts déjà mensuels</t>
+    <t xml:space="preserve">Rémunération de Nathan, € par semaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">absente des comptes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remboursements crédits et leasing, € par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≈ 211 k€ sur 10 ans et 38 k€ sur 5 ans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semaines par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jours par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ouvert 7 jours sur 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mois d’exploitation (ouverture en mars)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pour ramener au mois les totaux de la période</t>
   </si>
   <si>
     <t xml:space="preserve">Hausse de prix moyenne (plan B1)</t>
@@ -611,7 +626,7 @@
     <t xml:space="preserve">Achats fournitures sur la période</t>
   </si>
   <si>
-    <t xml:space="preserve">total de la période, selon l’analyse</t>
+    <t xml:space="preserve">total de la période</t>
   </si>
   <si>
     <t xml:space="preserve">Audit fournitures (B4), % de la ligne</t>
@@ -629,33 +644,21 @@
     <t xml:space="preserve">la cible du plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Rémunération de Nathan, € par semaine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">absente des comptes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remboursements crédits et leasing, € par mois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈ 211 k€ sur 10 ans et 38 k€ sur 5 ans, selon l’analyse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Semaines par mois</t>
+    <t xml:space="preserve">Résultat visé après Nathan et la banque (€ par mois)</t>
   </si>
   <si>
     <t xml:space="preserve">Poste (€ par mois)</t>
   </si>
   <si>
-    <t xml:space="preserve">Analyse (÷ 6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recalcul (mois réels)</t>
+    <t xml:space="preserve">Analyse</t>
   </si>
   <si>
     <t xml:space="preserve">% CA</t>
   </si>
   <si>
+    <t xml:space="preserve">CA pour le résultat visé</t>
+  </si>
+  <si>
     <t xml:space="preserve">Plan matière (B1 → B4)</t>
   </si>
   <si>
@@ -677,7 +680,7 @@
     <t xml:space="preserve">Personnel (sans rémunération de Nathan)</t>
   </si>
   <si>
-    <t xml:space="preserve">Loyer + charges locatives + assurance incendie (coût mensuel, inchangé)</t>
+    <t xml:space="preserve">Loyer + charges locatives + assurance incendie</t>
   </si>
   <si>
     <t xml:space="preserve">Énergie, eau, location panneaux PV</t>
@@ -686,7 +689,7 @@
     <t xml:space="preserve">Autres charges diverses (probablement les redevances)</t>
   </si>
   <si>
-    <t xml:space="preserve">Honoraires (fiduciaire, secrétariat social, Indeed…) (coût mensuel, inchangé)</t>
+    <t xml:space="preserve">Honoraires (fiduciaire, secrétariat social, Indeed…)</t>
   </si>
   <si>
     <t xml:space="preserve">Location containers</t>
@@ -725,22 +728,25 @@
     <t xml:space="preserve">Après Nathan et la banque</t>
   </si>
   <si>
+    <t xml:space="preserve">CA en plus par mois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA en plus par jour</t>
+  </si>
+  <si>
     <t xml:space="preserve">Point mort, Nathan payé (CA par mois)</t>
   </si>
   <si>
     <t xml:space="preserve">Point mort avec les remboursements (CA par mois)</t>
   </si>
   <si>
-    <t xml:space="preserve">Point mort : charges fixes (Nathan et remboursements compris) ÷ (1 − achats et emballages en % du CA). « Autres charges diverses » (probablement les redevances) comptées en fixe. Plan matière et scénario partent du recalcul.</t>
+    <t xml:space="preserve">Colonnes D à F : le CA qui donne le résultat visé (ligne 18) ; achats et emballages suivent le CA, les autres charges restent les mêmes. Point mort : charges fixes (Nathan et remboursements compris) ÷ (1 − achats et emballages en % du CA).</t>
   </si>
   <si>
     <t xml:space="preserve">Le rapprochement avec la caisse</t>
   </si>
   <si>
-    <t xml:space="preserve">CA comptable de la période (analyse × mois de l’analyse)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le CA comptable colle à la caisse de mars à septembre, pas à celle d’avril à septembre : les comptes couvrent sept mois.</t>
+    <t xml:space="preserve">CA comptable de la période (€ par mois × mois d’exploitation)</t>
   </si>
   <si>
     <t xml:space="preserve">CA de caisse HT, mars → septembre</t>
@@ -749,21 +755,9 @@
     <t xml:space="preserve">Écart comptable − caisse</t>
   </si>
   <si>
-    <t xml:space="preserve">CA de caisse HT, avril → septembre (l’hypothèse de l’analyse)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Écart comptable − caisse d’avril à septembre</t>
-  </si>
-  <si>
     <t xml:space="preserve">D’où vient la perte de la situation au 30/09</t>
   </si>
   <si>
-    <t xml:space="preserve">Analyse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recalcul</t>
-  </si>
-  <si>
     <t xml:space="preserve">Charges courues par mois sans CA</t>
   </si>
   <si>
@@ -773,13 +767,13 @@
     <t xml:space="preserve">Mois sans CA (octobre → février)</t>
   </si>
   <si>
-    <t xml:space="preserve">Charges courues sans CA (analyse : octobre → mars ; recalcul : octobre → février)</t>
+    <t xml:space="preserve">Charges courues sans CA, d’octobre à février</t>
   </si>
   <si>
     <t xml:space="preserve">Erreur de stock</t>
   </si>
   <si>
-    <t xml:space="preserve">Exploitation réelle (analyse : avril → septembre ; recalcul : mars → septembre)</t>
+    <t xml:space="preserve">Exploitation réelle de mars → septembre</t>
   </si>
   <si>
     <t xml:space="preserve">Amortissements</t>
@@ -815,7 +809,7 @@
     <t xml:space="preserve">L’application ou le bilan : mars → septembre 2026, en € par mois</t>
   </si>
   <si>
-    <t xml:space="preserve">Application : la caisse et le P&amp;L du panel (feuille « Mois par mois », main-d’œuvre encodée, food cost mesuré par le panel). Bilan : la situation au 30/09 de la fiduciaire, recalculée sur les mois réels (feuille « Compte d’exploitation », colonne Recalcul, à valider). En vert : liens ; en noir : calculs.</t>
+    <t xml:space="preserve">Application : la caisse et le P&amp;L du panel (feuille « Mois par mois », main-d’œuvre encodée, food cost mesuré par le panel). Bilan : la situation au 30/09 de la fiduciaire, ramenée au mois (feuille « Compte d’exploitation », colonne Analyse, à valider). En vert : liens ; en noir : calculs.</t>
   </si>
   <si>
     <t xml:space="preserve">Application</t>
@@ -830,7 +824,7 @@
     <t xml:space="preserve">Ce qui change d’une source à l’autre</t>
   </si>
   <si>
-    <t xml:space="preserve">caisse HT, contre CA comptable recalculé</t>
+    <t xml:space="preserve">caisse HT, contre CA comptable</t>
   </si>
   <si>
     <t xml:space="preserve">Matière</t>
@@ -893,9 +887,6 @@
     <t xml:space="preserve">À personnel et frais généraux égaux, un euro vendu en plus ne coûte que sa matière. Paliers en bleu (modifiables) ; liens en vert vers « Récap » et « Compte d’exploitation ».</t>
   </si>
   <si>
-    <t xml:space="preserve">Jours par mois</t>
-  </si>
-  <si>
     <t xml:space="preserve">Taux de marge, bilan</t>
   </si>
   <si>
@@ -914,9 +905,6 @@
     <t xml:space="preserve">€ par jour en plus</t>
   </si>
   <si>
-    <t xml:space="preserve">CA en plus par mois</t>
-  </si>
-  <si>
     <t xml:space="preserve">CA en plus par an</t>
   </si>
   <si>
@@ -941,7 +929,7 @@
     <t xml:space="preserve">Après remboursements (bilan)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ligne 0 : aujourd’hui, moyenne de mars à septembre (le bilan recalculé sur sept mois). Une vente faite avec une remise rapporte moins que la marge directe.</t>
+    <t xml:space="preserve">Ligne 0 : aujourd’hui, moyenne de mars à septembre (le bilan de la page 3). Une vente faite avec une remise rapporte moins que la marge directe.</t>
   </si>
 </sst>
 </file>
@@ -1138,7 +1126,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1325,14 +1313,6 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -3542,16 +3522,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3573,8 +3554,8 @@
       <c r="A5" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="B5" s="36" t="n">
-        <v>6</v>
+      <c r="B5" s="14" t="n">
+        <v>500</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>148</v>
@@ -3584,8 +3565,8 @@
       <c r="A6" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B6" s="47" t="n">
-        <v>7</v>
+      <c r="B6" s="14" t="n">
+        <v>2900</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>150</v>
@@ -3595,68 +3576,70 @@
       <c r="A7" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="27" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>152</v>
-      </c>
+      <c r="B7" s="15" t="n">
+        <f aca="false">52/12</f>
+        <v>4.33333333333333</v>
+      </c>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8" s="15" t="n">
+        <f aca="false">365/12</f>
+        <v>30.4166666666667</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B8" s="27" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="C8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="B9" s="27" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="C9" s="2"/>
+      <c r="B9" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="B10" s="17" t="n">
-        <v>19500</v>
+        <v>156</v>
+      </c>
+      <c r="B10" s="27" t="n">
+        <v>0.05</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B11" s="27" t="n">
-        <v>0.35</v>
+        <v>0.08</v>
       </c>
       <c r="C11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B12" s="27" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>159</v>
-      </c>
+        <v>0.04</v>
+      </c>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="B13" s="27" t="n">
-        <v>0.4</v>
+      <c r="B13" s="17" t="n">
+        <v>19500</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>161</v>
@@ -3666,121 +3649,117 @@
       <c r="A14" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="B14" s="14" t="n">
-        <v>500</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>163</v>
-      </c>
+      <c r="B14" s="27" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B15" s="27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="B15" s="14" t="n">
-        <v>2900</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="B16" s="27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B16" s="15" t="n">
-        <f aca="false">52/12</f>
-        <v>4.33333333333333</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="D18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="B19" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="E19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="H19" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="H18" s="4" t="s">
+      <c r="I19" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="J19" s="4" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="B19" s="17" t="n">
-        <v>58216</v>
-      </c>
-      <c r="C19" s="23" t="n">
-        <f aca="false">B19*$B$5/$B$6</f>
-        <v>49899.4285714286</v>
-      </c>
-      <c r="D19" s="24" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C19/C$19,0)</f>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="B20" s="17" t="n">
+        <v>49899.43</v>
+      </c>
+      <c r="C20" s="24" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B20/B$20,0)</f>
         <v>1</v>
       </c>
-      <c r="E19" s="23" t="n">
-        <f aca="false">C19*(1+$B$7)</f>
-        <v>52394.4</v>
-      </c>
-      <c r="F19" s="24" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E19/E$19,0)</f>
+      <c r="D20" s="32" t="n">
+        <f aca="false">(SUM($B$24:$B$35)+$B$5*$B$7+$B$6+D$18)/(1-($B$21+$B$22)/$B$20)</f>
+        <v>54482.910495642</v>
+      </c>
+      <c r="E20" s="32" t="n">
+        <f aca="false">(SUM($B$24:$B$35)+$B$5*$B$7+$B$6+E$18)/(1-($B$21+$B$22)/$B$20)</f>
+        <v>64465.763399525</v>
+      </c>
+      <c r="F20" s="32" t="n">
+        <f aca="false">(SUM($B$24:$B$35)+$B$5*$B$7+$B$6+F$18)/(1-($B$21+$B$22)/$B$20)</f>
+        <v>74448.6163034081</v>
+      </c>
+      <c r="G20" s="23" t="n">
+        <f aca="false">B20*(1+$B$10)</f>
+        <v>52394.4015</v>
+      </c>
+      <c r="H20" s="24" t="n">
+        <f aca="false">IF(G$20&lt;&gt;0,G20/G$20,0)</f>
         <v>1</v>
       </c>
-      <c r="G19" s="23" t="n">
-        <f aca="false">C19*(1+$B$12)</f>
-        <v>57384.3428571429</v>
-      </c>
-      <c r="H19" s="24" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G19/G$19,0)</f>
+      <c r="I20" s="23" t="n">
+        <f aca="false">B20*(1+$B$15)</f>
+        <v>57384.3445</v>
+      </c>
+      <c r="J20" s="24" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I20/I$20,0)</f>
         <v>1</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="B20" s="17" t="n">
-        <v>28144</v>
-      </c>
-      <c r="C20" s="8" t="n">
-        <f aca="false">B20*$B$5/$B$6</f>
-        <v>24123.4285714286</v>
-      </c>
-      <c r="D20" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C20/C$19,0)</f>
-        <v>0.483440978425175</v>
-      </c>
-      <c r="E20" s="8" t="n">
-        <f aca="false">C20*(1-$B$8-$B$9)-$B$10/$B$6*$B$11</f>
-        <v>20253.6171428571</v>
-      </c>
-      <c r="F20" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E20/E$19,0)</f>
-        <v>0.386560722956216</v>
-      </c>
-      <c r="G20" s="8" t="n">
-        <f aca="false">G19*$B$13</f>
-        <v>22953.7371428571</v>
-      </c>
-      <c r="H20" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G20/G$19,0)</f>
-        <v>0.4</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3788,96 +3767,120 @@
         <v>175</v>
       </c>
       <c r="B21" s="17" t="n">
-        <v>914</v>
-      </c>
-      <c r="C21" s="8" t="n">
-        <f aca="false">B21*$B$5/$B$6</f>
-        <v>783.428571428571</v>
-      </c>
-      <c r="D21" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C21/C$19,0)</f>
-        <v>0.0157001511611928</v>
+        <v>24123.43</v>
+      </c>
+      <c r="C21" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B21/B$20,0)</f>
+        <v>0.48344099321375</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <f aca="false">D20*$B$21/$B$20</f>
+        <v>26339.272363189</v>
       </c>
       <c r="E21" s="8" t="n">
-        <f aca="false">C21</f>
-        <v>783.428571428571</v>
-      </c>
-      <c r="F21" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E21/E$19,0)</f>
-        <v>0.0149525249154217</v>
+        <f aca="false">E20*$B$21/$B$20</f>
+        <v>31165.392686149</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <f aca="false">F20*$B$21/$B$20</f>
+        <v>35991.513009109</v>
       </c>
       <c r="G21" s="8" t="n">
-        <f aca="false">IF(C19&gt;0,C21/C19*G19,0)</f>
-        <v>900.942857142857</v>
+        <f aca="false">B21*(1-$B$11-$B$12)-$B$13/$B$9*$B$14</f>
+        <v>20253.6184</v>
       </c>
       <c r="H21" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G21/G$19,0)</f>
-        <v>0.0157001511611928</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G21/G$20,0)</f>
+        <v>0.386560735883203</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <f aca="false">I20*$B$16</f>
+        <v>22953.7378</v>
+      </c>
+      <c r="J21" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I21/I$20,0)</f>
+        <v>0.4</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="B22" s="20" t="n">
-        <f aca="false">B19-B20-B21</f>
-        <v>29158</v>
-      </c>
-      <c r="C22" s="20" t="n">
-        <f aca="false">C19-C20-C21</f>
-        <v>24992.5714285714</v>
-      </c>
-      <c r="D22" s="24" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C22/C$19,0)</f>
-        <v>0.500858870413632</v>
-      </c>
-      <c r="E22" s="20" t="n">
-        <f aca="false">E19-E20-E21</f>
-        <v>31357.3542857143</v>
-      </c>
-      <c r="F22" s="24" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E22/E$19,0)</f>
-        <v>0.598486752128363</v>
-      </c>
-      <c r="G22" s="20" t="n">
-        <f aca="false">G19-G20-G21</f>
-        <v>33529.6628571429</v>
-      </c>
-      <c r="H22" s="24" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G22/G$19,0)</f>
-        <v>0.584299848838807</v>
+      <c r="B22" s="17" t="n">
+        <v>783.43</v>
+      </c>
+      <c r="C22" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B22/B$20,0)</f>
+        <v>0.0157001793407259</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <f aca="false">D20*$B$22/$B$20</f>
+        <v>855.391465786299</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <f aca="false">E20*$B$22/$B$20</f>
+        <v>1012.12404670935</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <f aca="false">F20*$B$22/$B$20</f>
+        <v>1168.8566276324</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <f aca="false">B22</f>
+        <v>783.43</v>
+      </c>
+      <c r="H22" s="18" t="n">
+        <f aca="false">IF(G$20&lt;&gt;0,G22/G$20,0)</f>
+        <v>0.0149525517530723</v>
+      </c>
+      <c r="I22" s="8" t="n">
+        <f aca="false">IF(B20&gt;0,B22/B20*I20,0)</f>
+        <v>900.9445</v>
+      </c>
+      <c r="J22" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I22/I$20,0)</f>
+        <v>0.0157001793407259</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="B23" s="17" t="n">
-        <v>9364</v>
-      </c>
-      <c r="C23" s="8" t="n">
-        <f aca="false">B23*$B$5/$B$6</f>
-        <v>8026.28571428572</v>
-      </c>
-      <c r="D23" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C23/C$19,0)</f>
-        <v>0.160849251064999</v>
-      </c>
-      <c r="E23" s="8" t="n">
-        <f aca="false">C23</f>
-        <v>8026.28571428572</v>
-      </c>
-      <c r="F23" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E23/E$19,0)</f>
-        <v>0.153189762919047</v>
-      </c>
-      <c r="G23" s="8" t="n">
-        <f aca="false">C23</f>
-        <v>8026.28571428572</v>
-      </c>
-      <c r="H23" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G23/G$19,0)</f>
-        <v>0.139868913969565</v>
+      <c r="B23" s="20" t="n">
+        <f aca="false">B20-B21-B22</f>
+        <v>24992.57</v>
+      </c>
+      <c r="C23" s="24" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B23/B$20,0)</f>
+        <v>0.500858827445524</v>
+      </c>
+      <c r="D23" s="20" t="n">
+        <f aca="false">D20-D21-D22</f>
+        <v>27288.2466666667</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <f aca="false">E20-E21-E22</f>
+        <v>32288.2466666667</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <f aca="false">F20-F21-F22</f>
+        <v>37288.2466666667</v>
+      </c>
+      <c r="G23" s="20" t="n">
+        <f aca="false">G20-G21-G22</f>
+        <v>31357.3531</v>
+      </c>
+      <c r="H23" s="24" t="n">
+        <f aca="false">IF(G$20&lt;&gt;0,G23/G$20,0)</f>
+        <v>0.598486712363725</v>
+      </c>
+      <c r="I23" s="20" t="n">
+        <f aca="false">I20-I21-I22</f>
+        <v>33529.6622</v>
+      </c>
+      <c r="J23" s="24" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I23/I$20,0)</f>
+        <v>0.584299820659274</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3885,31 +3888,39 @@
         <v>178</v>
       </c>
       <c r="B24" s="17" t="n">
-        <v>4862</v>
-      </c>
-      <c r="C24" s="8" t="n">
-        <f aca="false">B24</f>
-        <v>4862</v>
-      </c>
-      <c r="D24" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C24/C$19,0)</f>
-        <v>0.0974359855251706</v>
+        <v>8026.29</v>
+      </c>
+      <c r="C24" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B24/B$20,0)</f>
+        <v>0.160849332347083</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <f aca="false">$B24</f>
+        <v>8026.29</v>
       </c>
       <c r="E24" s="8" t="n">
-        <f aca="false">C24</f>
-        <v>4862</v>
-      </c>
-      <c r="F24" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E24/E$19,0)</f>
-        <v>0.0927961766906387</v>
+        <f aca="false">$B24</f>
+        <v>8026.29</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <f aca="false">$B24</f>
+        <v>8026.29</v>
       </c>
       <c r="G24" s="8" t="n">
-        <f aca="false">C24</f>
-        <v>4862</v>
+        <f aca="false">$B24</f>
+        <v>8026.29</v>
       </c>
       <c r="H24" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G24/G$19,0)</f>
-        <v>0.084726943934931</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G24/G$20,0)</f>
+        <v>0.153189840330555</v>
+      </c>
+      <c r="I24" s="8" t="n">
+        <f aca="false">$B24</f>
+        <v>8026.29</v>
+      </c>
+      <c r="J24" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I24/I$20,0)</f>
+        <v>0.139868984649637</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3917,31 +3928,39 @@
         <v>179</v>
       </c>
       <c r="B25" s="17" t="n">
-        <v>1514</v>
-      </c>
-      <c r="C25" s="8" t="n">
-        <f aca="false">B25*$B$5/$B$6</f>
-        <v>1297.71428571429</v>
-      </c>
-      <c r="D25" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C25/C$19,0)</f>
-        <v>0.0260065961247767</v>
+        <v>4862</v>
+      </c>
+      <c r="C25" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B25/B$20,0)</f>
+        <v>0.0974359827356745</v>
+      </c>
+      <c r="D25" s="8" t="n">
+        <f aca="false">$B25</f>
+        <v>4862</v>
       </c>
       <c r="E25" s="8" t="n">
-        <f aca="false">C25</f>
-        <v>1297.71428571429</v>
-      </c>
-      <c r="F25" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E25/E$19,0)</f>
-        <v>0.0247681867855016</v>
+        <f aca="false">$B25</f>
+        <v>4862</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <f aca="false">$B25</f>
+        <v>4862</v>
       </c>
       <c r="G25" s="8" t="n">
-        <f aca="false">C25</f>
-        <v>1297.71428571429</v>
+        <f aca="false">$B25</f>
+        <v>4862</v>
       </c>
       <c r="H25" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G25/G$19,0)</f>
-        <v>0.0226144314128493</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G25/G$20,0)</f>
+        <v>0.0927961740339758</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <f aca="false">$B25</f>
+        <v>4862</v>
+      </c>
+      <c r="J25" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I25/I$20,0)</f>
+        <v>0.0847269415092822</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3949,31 +3968,39 @@
         <v>180</v>
       </c>
       <c r="B26" s="17" t="n">
-        <v>1510</v>
-      </c>
-      <c r="C26" s="8" t="n">
-        <f aca="false">B26*$B$5/$B$6</f>
-        <v>1294.28571428571</v>
-      </c>
-      <c r="D26" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C26/C$19,0)</f>
-        <v>0.0259378864916861</v>
+        <v>1297.71</v>
+      </c>
+      <c r="C26" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B26/B$20,0)</f>
+        <v>0.0260065094931946</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <f aca="false">$B26</f>
+        <v>1297.71</v>
       </c>
       <c r="E26" s="8" t="n">
-        <f aca="false">C26</f>
-        <v>1294.28571428571</v>
-      </c>
-      <c r="F26" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E26/E$19,0)</f>
-        <v>0.0247027490397011</v>
+        <f aca="false">$B26</f>
+        <v>1297.71</v>
+      </c>
+      <c r="F26" s="8" t="n">
+        <f aca="false">$B26</f>
+        <v>1297.71</v>
       </c>
       <c r="G26" s="8" t="n">
-        <f aca="false">C26</f>
-        <v>1294.28571428571</v>
+        <f aca="false">$B26</f>
+        <v>1297.71</v>
       </c>
       <c r="H26" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G26/G$19,0)</f>
-        <v>0.022554683905814</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G26/G$20,0)</f>
+        <v>0.024768104279233</v>
+      </c>
+      <c r="I26" s="8" t="n">
+        <f aca="false">$B26</f>
+        <v>1297.71</v>
+      </c>
+      <c r="J26" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I26/I$20,0)</f>
+        <v>0.0226143560810388</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3981,31 +4008,39 @@
         <v>181</v>
       </c>
       <c r="B27" s="17" t="n">
-        <v>1493</v>
-      </c>
-      <c r="C27" s="8" t="n">
-        <f aca="false">B27</f>
-        <v>1493</v>
-      </c>
-      <c r="D27" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C27/C$19,0)</f>
-        <v>0.0299201823095598</v>
+        <v>1294.29</v>
+      </c>
+      <c r="C27" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B27/B$20,0)</f>
+        <v>0.025937971636149</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <f aca="false">$B27</f>
+        <v>1294.29</v>
       </c>
       <c r="E27" s="8" t="n">
-        <f aca="false">C27</f>
-        <v>1493</v>
-      </c>
-      <c r="F27" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E27/E$19,0)</f>
-        <v>0.0284954117233903</v>
+        <f aca="false">$B27</f>
+        <v>1294.29</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <f aca="false">$B27</f>
+        <v>1294.29</v>
       </c>
       <c r="G27" s="8" t="n">
-        <f aca="false">C27</f>
-        <v>1493</v>
+        <f aca="false">$B27</f>
+        <v>1294.29</v>
       </c>
       <c r="H27" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G27/G$19,0)</f>
-        <v>0.0260175498343998</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G27/G$20,0)</f>
+        <v>0.0247028301296657</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <f aca="false">$B27</f>
+        <v>1294.29</v>
+      </c>
+      <c r="J27" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I27/I$20,0)</f>
+        <v>0.0225547579444774</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4013,31 +4048,39 @@
         <v>182</v>
       </c>
       <c r="B28" s="17" t="n">
-        <v>1295</v>
-      </c>
-      <c r="C28" s="8" t="n">
-        <f aca="false">B28*$B$5/$B$6</f>
-        <v>1110</v>
-      </c>
-      <c r="D28" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C28/C$19,0)</f>
-        <v>0.0222447437130686</v>
+        <v>1493</v>
+      </c>
+      <c r="C28" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B28/B$20,0)</f>
+        <v>0.0299201814529745</v>
+      </c>
+      <c r="D28" s="8" t="n">
+        <f aca="false">$B28</f>
+        <v>1493</v>
       </c>
       <c r="E28" s="8" t="n">
-        <f aca="false">C28</f>
-        <v>1110</v>
-      </c>
-      <c r="F28" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E28/E$19,0)</f>
-        <v>0.0211854702029224</v>
+        <f aca="false">$B28</f>
+        <v>1493</v>
+      </c>
+      <c r="F28" s="8" t="n">
+        <f aca="false">$B28</f>
+        <v>1493</v>
       </c>
       <c r="G28" s="8" t="n">
-        <f aca="false">C28</f>
-        <v>1110</v>
+        <f aca="false">$B28</f>
+        <v>1493</v>
       </c>
       <c r="H28" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G28/G$19,0)</f>
-        <v>0.0193432554026683</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G28/G$20,0)</f>
+        <v>0.0284954109075948</v>
+      </c>
+      <c r="I28" s="8" t="n">
+        <f aca="false">$B28</f>
+        <v>1493</v>
+      </c>
+      <c r="J28" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I28/I$20,0)</f>
+        <v>0.0260175490895431</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4045,31 +4088,39 @@
         <v>183</v>
       </c>
       <c r="B29" s="17" t="n">
-        <v>1104</v>
-      </c>
-      <c r="C29" s="8" t="n">
-        <f aca="false">B29*$B$5/$B$6</f>
-        <v>946.285714285714</v>
-      </c>
-      <c r="D29" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C29/C$19,0)</f>
-        <v>0.0189638587329944</v>
+        <v>1110</v>
+      </c>
+      <c r="C29" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B29/B$20,0)</f>
+        <v>0.0222447430762235</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <f aca="false">$B29</f>
+        <v>1110</v>
       </c>
       <c r="E29" s="8" t="n">
-        <f aca="false">C29</f>
-        <v>946.285714285714</v>
-      </c>
-      <c r="F29" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E29/E$19,0)</f>
-        <v>0.018060817840947</v>
+        <f aca="false">$B29</f>
+        <v>1110</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <f aca="false">$B29</f>
+        <v>1110</v>
       </c>
       <c r="G29" s="8" t="n">
-        <f aca="false">C29</f>
-        <v>946.285714285714</v>
+        <f aca="false">$B29</f>
+        <v>1110</v>
       </c>
       <c r="H29" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G29/G$19,0)</f>
-        <v>0.0164903119417342</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G29/G$20,0)</f>
+        <v>0.0211854695964034</v>
+      </c>
+      <c r="I29" s="8" t="n">
+        <f aca="false">$B29</f>
+        <v>1110</v>
+      </c>
+      <c r="J29" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I29/I$20,0)</f>
+        <v>0.01934325484889</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4077,31 +4128,39 @@
         <v>184</v>
       </c>
       <c r="B30" s="17" t="n">
-        <v>1011</v>
-      </c>
-      <c r="C30" s="8" t="n">
-        <f aca="false">B30*$B$5/$B$6</f>
-        <v>866.571428571429</v>
-      </c>
-      <c r="D30" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C30/C$19,0)</f>
-        <v>0.0173663597636389</v>
+        <v>946.29</v>
+      </c>
+      <c r="C30" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B30/B$20,0)</f>
+        <v>0.0189639440771167</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <f aca="false">$B30</f>
+        <v>946.29</v>
       </c>
       <c r="E30" s="8" t="n">
-        <f aca="false">C30</f>
-        <v>866.571428571429</v>
-      </c>
-      <c r="F30" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E30/E$19,0)</f>
-        <v>0.0165393902510846</v>
+        <f aca="false">$B30</f>
+        <v>946.29</v>
+      </c>
+      <c r="F30" s="8" t="n">
+        <f aca="false">$B30</f>
+        <v>946.29</v>
       </c>
       <c r="G30" s="8" t="n">
-        <f aca="false">C30</f>
-        <v>866.571428571429</v>
+        <f aca="false">$B30</f>
+        <v>946.29</v>
       </c>
       <c r="H30" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G30/G$19,0)</f>
-        <v>0.0151011824031642</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G30/G$20,0)</f>
+        <v>0.0180608991210635</v>
+      </c>
+      <c r="I30" s="8" t="n">
+        <f aca="false">$B30</f>
+        <v>946.29</v>
+      </c>
+      <c r="J30" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I30/I$20,0)</f>
+        <v>0.0164903861540145</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4109,31 +4168,39 @@
         <v>185</v>
       </c>
       <c r="B31" s="17" t="n">
-        <v>778</v>
-      </c>
-      <c r="C31" s="8" t="n">
-        <f aca="false">B31*$B$5/$B$6</f>
-        <v>666.857142857143</v>
-      </c>
-      <c r="D31" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C31/C$19,0)</f>
-        <v>0.0133640236361138</v>
+        <v>866.57</v>
+      </c>
+      <c r="C31" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B31/B$20,0)</f>
+        <v>0.0173663306374442</v>
+      </c>
+      <c r="D31" s="8" t="n">
+        <f aca="false">$B31</f>
+        <v>866.57</v>
       </c>
       <c r="E31" s="8" t="n">
-        <f aca="false">C31</f>
-        <v>666.857142857143</v>
-      </c>
-      <c r="F31" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E31/E$19,0)</f>
-        <v>0.0127276415582036</v>
+        <f aca="false">$B31</f>
+        <v>866.57</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <f aca="false">$B31</f>
+        <v>866.57</v>
       </c>
       <c r="G31" s="8" t="n">
-        <f aca="false">C31</f>
-        <v>666.857142857143</v>
+        <f aca="false">$B31</f>
+        <v>866.57</v>
       </c>
       <c r="H31" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G31/G$19,0)</f>
-        <v>0.0116208901183598</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G31/G$20,0)</f>
+        <v>0.0165393625118516</v>
+      </c>
+      <c r="I31" s="8" t="n">
+        <f aca="false">$B31</f>
+        <v>866.57</v>
+      </c>
+      <c r="J31" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I31/I$20,0)</f>
+        <v>0.0151011570760384</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4141,31 +4208,39 @@
         <v>186</v>
       </c>
       <c r="B32" s="17" t="n">
-        <v>738</v>
-      </c>
-      <c r="C32" s="8" t="n">
-        <f aca="false">B32*$B$5/$B$6</f>
-        <v>632.571428571429</v>
-      </c>
-      <c r="D32" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C32/C$19,0)</f>
-        <v>0.0126769273052082</v>
+        <v>666.86</v>
+      </c>
+      <c r="C32" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B32/B$20,0)</f>
+        <v>0.0133640805115409</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <f aca="false">$B32</f>
+        <v>666.86</v>
       </c>
       <c r="E32" s="8" t="n">
-        <f aca="false">C32</f>
-        <v>632.571428571429</v>
-      </c>
-      <c r="F32" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E32/E$19,0)</f>
-        <v>0.0120732641001983</v>
+        <f aca="false">$B32</f>
+        <v>666.86</v>
+      </c>
+      <c r="F32" s="8" t="n">
+        <f aca="false">$B32</f>
+        <v>666.86</v>
       </c>
       <c r="G32" s="8" t="n">
-        <f aca="false">C32</f>
-        <v>632.571428571429</v>
+        <f aca="false">$B32</f>
+        <v>666.86</v>
       </c>
       <c r="H32" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G32/G$19,0)</f>
-        <v>0.0110234150480071</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G32/G$20,0)</f>
+        <v>0.0127276957252771</v>
+      </c>
+      <c r="I32" s="8" t="n">
+        <f aca="false">$B32</f>
+        <v>666.86</v>
+      </c>
+      <c r="J32" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I32/I$20,0)</f>
+        <v>0.011620939575253</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4173,31 +4248,39 @@
         <v>187</v>
       </c>
       <c r="B33" s="17" t="n">
-        <v>685</v>
-      </c>
-      <c r="C33" s="8" t="n">
-        <f aca="false">B33*$B$5/$B$6</f>
-        <v>587.142857142857</v>
-      </c>
-      <c r="D33" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C33/C$19,0)</f>
-        <v>0.0117665246667583</v>
+        <v>632.57</v>
+      </c>
+      <c r="C33" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B33/B$20,0)</f>
+        <v>0.0126768983132673</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <f aca="false">$B33</f>
+        <v>632.57</v>
       </c>
       <c r="E33" s="8" t="n">
-        <f aca="false">C33</f>
-        <v>587.142857142857</v>
-      </c>
-      <c r="F33" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E33/E$19,0)</f>
-        <v>0.0112062139683412</v>
+        <f aca="false">$B33</f>
+        <v>632.57</v>
+      </c>
+      <c r="F33" s="8" t="n">
+        <f aca="false">$B33</f>
+        <v>632.57</v>
       </c>
       <c r="G33" s="8" t="n">
-        <f aca="false">C33</f>
-        <v>587.142857142857</v>
+        <f aca="false">$B33</f>
+        <v>632.57</v>
       </c>
       <c r="H33" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G33/G$19,0)</f>
-        <v>0.0102317605797898</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G33/G$20,0)</f>
+        <v>0.012073236488826</v>
+      </c>
+      <c r="I33" s="8" t="n">
+        <f aca="false">$B33</f>
+        <v>632.57</v>
+      </c>
+      <c r="J33" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I33/I$20,0)</f>
+        <v>0.0110233898376237</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4205,446 +4288,503 @@
         <v>188</v>
       </c>
       <c r="B34" s="17" t="n">
-        <v>512</v>
-      </c>
-      <c r="C34" s="8" t="n">
-        <f aca="false">B34*$B$5/$B$6</f>
-        <v>438.857142857143</v>
-      </c>
-      <c r="D34" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C34/C$19,0)</f>
-        <v>0.00879483303559159</v>
+        <v>587.14</v>
+      </c>
+      <c r="C34" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B34/B$20,0)</f>
+        <v>0.0117664670718684</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <f aca="false">$B34</f>
+        <v>587.14</v>
       </c>
       <c r="E34" s="8" t="n">
-        <f aca="false">C34</f>
-        <v>438.857142857143</v>
-      </c>
-      <c r="F34" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E34/E$19,0)</f>
-        <v>0.00837603146246818</v>
+        <f aca="false">$B34</f>
+        <v>587.14</v>
+      </c>
+      <c r="F34" s="8" t="n">
+        <f aca="false">$B34</f>
+        <v>587.14</v>
       </c>
       <c r="G34" s="8" t="n">
-        <f aca="false">C34</f>
-        <v>438.857142857143</v>
+        <f aca="false">$B34</f>
+        <v>587.14</v>
       </c>
       <c r="H34" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G34/G$19,0)</f>
-        <v>0.00764768090051443</v>
+        <f aca="false">IF(G$20&lt;&gt;0,G34/G$20,0)</f>
+        <v>0.0112061591160651</v>
+      </c>
+      <c r="I34" s="8" t="n">
+        <f aca="false">$B34</f>
+        <v>587.14</v>
+      </c>
+      <c r="J34" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I34/I$20,0)</f>
+        <v>0.0102317104972768</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="B35" s="20" t="n">
-        <f aca="false">B22-SUM(B23:B34)</f>
-        <v>4292</v>
-      </c>
-      <c r="C35" s="20" t="n">
-        <f aca="false">C22-SUM(C23:C34)</f>
-        <v>2771</v>
-      </c>
-      <c r="D35" s="24" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C35/C$19,0)</f>
-        <v>0.0555316980440658</v>
-      </c>
-      <c r="E35" s="20" t="n">
-        <f aca="false">E22-SUM(E23:E34)</f>
-        <v>9135.78285714286</v>
-      </c>
-      <c r="F35" s="24" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E35/E$19,0)</f>
-        <v>0.174365635585919</v>
-      </c>
-      <c r="G35" s="20" t="n">
-        <f aca="false">G22-SUM(G23:G34)</f>
-        <v>11308.0914285714</v>
-      </c>
-      <c r="H35" s="24" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G35/G$19,0)</f>
-        <v>0.19705882938701</v>
+      <c r="B35" s="17" t="n">
+        <v>438.86</v>
+      </c>
+      <c r="C35" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B35/B$20,0)</f>
+        <v>0.00879489004183014</v>
+      </c>
+      <c r="D35" s="8" t="n">
+        <f aca="false">$B35</f>
+        <v>438.86</v>
+      </c>
+      <c r="E35" s="8" t="n">
+        <f aca="false">$B35</f>
+        <v>438.86</v>
+      </c>
+      <c r="F35" s="8" t="n">
+        <f aca="false">$B35</f>
+        <v>438.86</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <f aca="false">$B35</f>
+        <v>438.86</v>
+      </c>
+      <c r="H35" s="18" t="n">
+        <f aca="false">IF(G$20&lt;&gt;0,G35/G$20,0)</f>
+        <v>0.00837608575412394</v>
+      </c>
+      <c r="I35" s="8" t="n">
+        <f aca="false">$B35</f>
+        <v>438.86</v>
+      </c>
+      <c r="J35" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I35/I$20,0)</f>
+        <v>0.00764773047115664</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
+      <c r="A36" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="B36" s="8" t="n">
-        <f aca="false">-$B$14*$B$16</f>
+      <c r="B36" s="20" t="n">
+        <f aca="false">B23-SUM(B24:B35)</f>
+        <v>2770.99</v>
+      </c>
+      <c r="C36" s="24" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B36/B$20,0)</f>
+        <v>0.0555314960511573</v>
+      </c>
+      <c r="D36" s="20" t="n">
+        <f aca="false">D23-SUM(D24:D35)</f>
+        <v>5066.66666666667</v>
+      </c>
+      <c r="E36" s="20" t="n">
+        <f aca="false">E23-SUM(E24:E35)</f>
+        <v>10066.6666666667</v>
+      </c>
+      <c r="F36" s="20" t="n">
+        <f aca="false">F23-SUM(F24:F35)</f>
+        <v>15066.6666666667</v>
+      </c>
+      <c r="G36" s="20" t="n">
+        <f aca="false">G23-SUM(G24:G35)</f>
+        <v>9135.7731</v>
+      </c>
+      <c r="H36" s="24" t="n">
+        <f aca="false">IF(G$20&lt;&gt;0,G36/G$20,0)</f>
+        <v>0.17436544436909</v>
+      </c>
+      <c r="I36" s="20" t="n">
+        <f aca="false">I23-SUM(I24:I35)</f>
+        <v>11308.0822</v>
+      </c>
+      <c r="J36" s="24" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I36/I$20,0)</f>
+        <v>0.197058662925042</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="B37" s="8" t="n">
+        <f aca="false">-$B$5*$B$7</f>
         <v>-2166.66666666667</v>
       </c>
-      <c r="C36" s="8" t="n">
-        <f aca="false">-$B$14*$B$16</f>
+      <c r="C37" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B37/B$20,0)</f>
+        <v>-0.0434206696683042</v>
+      </c>
+      <c r="D37" s="8" t="n">
+        <f aca="false">-$B$5*$B$7</f>
         <v>-2166.66666666667</v>
       </c>
-      <c r="D36" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C36/C$19,0)</f>
-        <v>-0.0434206709113951</v>
-      </c>
-      <c r="E36" s="8" t="n">
-        <f aca="false">-$B$14*$B$16</f>
+      <c r="E37" s="8" t="n">
+        <f aca="false">-$B$5*$B$7</f>
         <v>-2166.66666666667</v>
       </c>
-      <c r="F36" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E36/E$19,0)</f>
-        <v>-0.0413530199156144</v>
-      </c>
-      <c r="G36" s="8" t="n">
-        <f aca="false">-$B$14*$B$16</f>
+      <c r="F37" s="8" t="n">
+        <f aca="false">-$B$5*$B$7</f>
         <v>-2166.66666666667</v>
       </c>
-      <c r="H36" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G36/G$19,0)</f>
-        <v>-0.0377571051403436</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="B37" s="23" t="n">
-        <f aca="false">B35+B36</f>
-        <v>2125.33333333333</v>
-      </c>
-      <c r="C37" s="23" t="n">
-        <f aca="false">C35+C36</f>
-        <v>604.333333333334</v>
-      </c>
-      <c r="D37" s="24" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C37/C$19,0)</f>
-        <v>0.0121110271326707</v>
-      </c>
-      <c r="E37" s="23" t="n">
-        <f aca="false">E35+E36</f>
-        <v>6969.11619047619</v>
-      </c>
-      <c r="F37" s="24" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E37/E$19,0)</f>
-        <v>0.133012615670304</v>
-      </c>
-      <c r="G37" s="23" t="n">
-        <f aca="false">G35+G36</f>
-        <v>9141.42476190476</v>
-      </c>
-      <c r="H37" s="24" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G37/G$19,0)</f>
-        <v>0.159301724246667</v>
+      <c r="G37" s="8" t="n">
+        <f aca="false">-$B$5*$B$7</f>
+        <v>-2166.66666666667</v>
+      </c>
+      <c r="H37" s="18" t="n">
+        <f aca="false">IF(G$20&lt;&gt;0,G37/G$20,0)</f>
+        <v>-0.0413530187317183</v>
+      </c>
+      <c r="I37" s="8" t="n">
+        <f aca="false">-$B$5*$B$7</f>
+        <v>-2166.66666666667</v>
+      </c>
+      <c r="J37" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I37/I$20,0)</f>
+        <v>-0.0377571040593949</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="22" t="s">
         <v>192</v>
       </c>
-      <c r="B38" s="8" t="n">
-        <f aca="false">-$B$15</f>
+      <c r="B38" s="23" t="n">
+        <f aca="false">B36+B37</f>
+        <v>604.323333333331</v>
+      </c>
+      <c r="C38" s="24" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B38/B$20,0)</f>
+        <v>0.0121108263828531</v>
+      </c>
+      <c r="D38" s="23" t="n">
+        <f aca="false">D36+D37</f>
+        <v>2900.00000000001</v>
+      </c>
+      <c r="E38" s="23" t="n">
+        <f aca="false">E36+E37</f>
+        <v>7900</v>
+      </c>
+      <c r="F38" s="23" t="n">
+        <f aca="false">F36+F37</f>
+        <v>12900</v>
+      </c>
+      <c r="G38" s="23" t="n">
+        <f aca="false">G36+G37</f>
+        <v>6969.10643333333</v>
+      </c>
+      <c r="H38" s="24" t="n">
+        <f aca="false">IF(G$20&lt;&gt;0,G38/G$20,0)</f>
+        <v>0.133012425637371</v>
+      </c>
+      <c r="I38" s="23" t="n">
+        <f aca="false">I36+I37</f>
+        <v>9141.41553333333</v>
+      </c>
+      <c r="J38" s="24" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I38/I$20,0)</f>
+        <v>0.159301558865647</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B39" s="8" t="n">
+        <f aca="false">-$B$6</f>
         <v>-2900</v>
       </c>
-      <c r="C38" s="8" t="n">
-        <f aca="false">-$B$15</f>
+      <c r="C39" s="18" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B39/B$20,0)</f>
+        <v>-0.0581168963252687</v>
+      </c>
+      <c r="D39" s="8" t="n">
+        <f aca="false">-$B$6</f>
         <v>-2900</v>
       </c>
-      <c r="D38" s="18" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C38/C$19,0)</f>
-        <v>-0.0581168979890981</v>
-      </c>
-      <c r="E38" s="8" t="n">
-        <f aca="false">-$B$15</f>
+      <c r="E39" s="8" t="n">
+        <f aca="false">-$B$6</f>
         <v>-2900</v>
       </c>
-      <c r="F38" s="18" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E38/E$19,0)</f>
-        <v>-0.0553494266562839</v>
-      </c>
-      <c r="G38" s="8" t="n">
-        <f aca="false">-$B$15</f>
+      <c r="F39" s="8" t="n">
+        <f aca="false">-$B$6</f>
         <v>-2900</v>
       </c>
-      <c r="H38" s="18" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G38/G$19,0)</f>
-        <v>-0.0505364330339983</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="19" t="s">
-        <v>193</v>
-      </c>
-      <c r="B39" s="20" t="n">
-        <f aca="false">B37+B38</f>
-        <v>-774.666666666667</v>
-      </c>
-      <c r="C39" s="20" t="n">
-        <f aca="false">C37+C38</f>
-        <v>-2295.66666666667</v>
-      </c>
-      <c r="D39" s="24" t="n">
-        <f aca="false">IF(C$19&lt;&gt;0,C39/C$19,0)</f>
-        <v>-0.0460058708564274</v>
-      </c>
-      <c r="E39" s="20" t="n">
-        <f aca="false">E37+E38</f>
-        <v>4069.11619047619</v>
-      </c>
-      <c r="F39" s="24" t="n">
-        <f aca="false">IF(E$19&lt;&gt;0,E39/E$19,0)</f>
-        <v>0.0776631890140204</v>
-      </c>
-      <c r="G39" s="20" t="n">
-        <f aca="false">G37+G38</f>
-        <v>6241.42476190476</v>
-      </c>
-      <c r="H39" s="24" t="n">
-        <f aca="false">IF(G$19&lt;&gt;0,G39/G$19,0)</f>
-        <v>0.108765291212669</v>
+      <c r="G39" s="8" t="n">
+        <f aca="false">-$B$6</f>
+        <v>-2900</v>
+      </c>
+      <c r="H39" s="18" t="n">
+        <f aca="false">IF(G$20&lt;&gt;0,G39/G$20,0)</f>
+        <v>-0.0553494250716844</v>
+      </c>
+      <c r="I39" s="8" t="n">
+        <f aca="false">-$B$6</f>
+        <v>-2900</v>
+      </c>
+      <c r="J39" s="18" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I39/I$20,0)</f>
+        <v>-0.0505364315871901</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="19" t="s">
+        <v>194</v>
+      </c>
+      <c r="B40" s="20" t="n">
+        <f aca="false">B38+B39</f>
+        <v>-2295.67666666667</v>
+      </c>
+      <c r="C40" s="24" t="n">
+        <f aca="false">IF(B$20&lt;&gt;0,B40/B$20,0)</f>
+        <v>-0.0460060699424155</v>
+      </c>
+      <c r="D40" s="20" t="n">
+        <f aca="false">D38+D39</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="20" t="n">
+        <f aca="false">E38+E39</f>
+        <v>5000</v>
+      </c>
+      <c r="F40" s="20" t="n">
+        <f aca="false">F38+F39</f>
+        <v>10000</v>
+      </c>
+      <c r="G40" s="20" t="n">
+        <f aca="false">G38+G39</f>
+        <v>4069.10643333333</v>
+      </c>
+      <c r="H40" s="24" t="n">
+        <f aca="false">IF(G$20&lt;&gt;0,G40/G$20,0)</f>
+        <v>0.077663000565687</v>
+      </c>
+      <c r="I40" s="20" t="n">
+        <f aca="false">I38+I39</f>
+        <v>6241.41553333333</v>
+      </c>
+      <c r="J40" s="24" t="n">
+        <f aca="false">IF(I$20&lt;&gt;0,I40/I$20,0)</f>
+        <v>0.108765127278457</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="28" t="s">
-        <v>194</v>
-      </c>
-      <c r="B41" s="32" t="n">
-        <f aca="false">IF(B19&gt;0,(SUM(B23:B34)-B36)/(1-(B20+B21)/B19),0)</f>
-        <v>53972.6223563573</v>
-      </c>
-      <c r="C41" s="32" t="n">
-        <f aca="false">IF(C19&gt;0,(SUM(C23:C34)-C36)/(1-(C20+C21)/C19),0)</f>
-        <v>48692.8345206249</v>
-      </c>
-      <c r="E41" s="32" t="n">
-        <f aca="false">IF(E19&gt;0,(SUM(E23:E34)-E36)/(1-(E20+E21)/E19),0)</f>
-        <v>40749.8378343508</v>
-      </c>
-      <c r="G41" s="32" t="n">
-        <f aca="false">IF(G19&gt;0,(SUM(G23:G34)-G36)/(1-(G20+G21)/G19),0)</f>
-        <v>41739.2510775168</v>
+      <c r="A41" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D41" s="8" t="n">
+        <f aca="false">D20-$B$20</f>
+        <v>4583.48049564198</v>
+      </c>
+      <c r="E41" s="8" t="n">
+        <f aca="false">E20-$B$20</f>
+        <v>14566.333399525</v>
+      </c>
+      <c r="F41" s="8" t="n">
+        <f aca="false">F20-$B$20</f>
+        <v>24549.1863034081</v>
+      </c>
+      <c r="G41" s="8" t="n">
+        <f aca="false">G20-$B$20</f>
+        <v>2494.9715</v>
+      </c>
+      <c r="I41" s="8" t="n">
+        <f aca="false">I20-$B$20</f>
+        <v>7484.9145</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="28" t="s">
-        <v>195</v>
-      </c>
-      <c r="B42" s="32" t="n">
-        <f aca="false">IF(B19&gt;0,(SUM(B23:B34)-B36-B38)/(1-(B20+B21)/B19),0)</f>
-        <v>59762.6765438873</v>
-      </c>
-      <c r="C42" s="32" t="n">
-        <f aca="false">IF(C19&gt;0,(SUM(C23:C34)-C36-C38)/(1-(C20+C21)/C19),0)</f>
-        <v>54482.8887081549</v>
-      </c>
-      <c r="E42" s="32" t="n">
-        <f aca="false">IF(E19&gt;0,(SUM(E23:E34)-E36-E38)/(1-(E20+E21)/E19),0)</f>
-        <v>45595.3920420035</v>
-      </c>
-      <c r="G42" s="32" t="n">
-        <f aca="false">IF(G19&gt;0,(SUM(G23:G34)-G36-G38)/(1-(G20+G21)/G19),0)</f>
-        <v>46702.4561951687</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2" t="s">
+      <c r="A42" s="6" t="s">
         <v>196</v>
       </c>
+      <c r="D42" s="8" t="n">
+        <f aca="false">D41/$B$8</f>
+        <v>150.689769719736</v>
+      </c>
+      <c r="E42" s="8" t="n">
+        <f aca="false">E41/$B$8</f>
+        <v>478.893152861096</v>
+      </c>
+      <c r="F42" s="8" t="n">
+        <f aca="false">F41/$B$8</f>
+        <v>807.096536002456</v>
+      </c>
+      <c r="G42" s="8" t="n">
+        <f aca="false">G41/$B$8</f>
+        <v>82.0264602739726</v>
+      </c>
+      <c r="I42" s="8" t="n">
+        <f aca="false">I41/$B$8</f>
+        <v>246.079380821918</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="28" t="s">
+        <v>197</v>
+      </c>
+      <c r="B44" s="32" t="n">
+        <f aca="false">IF(B20&gt;0,(SUM(B24:B35)-B37)/(1-(B21+B22)/B20),0)</f>
+        <v>48692.8558113898</v>
+      </c>
+      <c r="G44" s="32" t="n">
+        <f aca="false">IF(G20&gt;0,(SUM(G24:G35)-G37)/(1-(G21+G22)/G20),0)</f>
+        <v>40749.8548636865</v>
+      </c>
+      <c r="I44" s="32" t="n">
+        <f aca="false">IF(I20&gt;0,(SUM(I24:I35)-I37)/(1-(I21+I22)/I20),0)</f>
+        <v>41739.2677600843</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
-        <v>197</v>
+      <c r="A45" s="28" t="s">
+        <v>198</v>
+      </c>
+      <c r="B45" s="32" t="n">
+        <f aca="false">IF(B20&gt;0,(SUM(B24:B35)-B37-B39)/(1-(B21+B22)/B20),0)</f>
+        <v>54482.910495642</v>
+      </c>
+      <c r="G45" s="32" t="n">
+        <f aca="false">IF(G20&gt;0,(SUM(G24:G35)-G37-G39)/(1-(G21+G22)/G20),0)</f>
+        <v>45595.4093932874</v>
+      </c>
+      <c r="I45" s="32" t="n">
+        <f aca="false">IF(I20&gt;0,(SUM(I24:I35)-I37-I39)/(1-(I21+I22)/I20),0)</f>
+        <v>46702.473117101</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="B46" s="8" t="n">
-        <f aca="false">B19*$B$5</f>
-        <v>349296</v>
-      </c>
-      <c r="D46" s="2" t="s">
+      <c r="A46" s="2" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="6" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="B47" s="7" t="n">
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="B49" s="8" t="n">
+        <f aca="false">B20*$B$9</f>
+        <v>349296.01</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B50" s="7" t="n">
         <f aca="false">SUM('Mois par mois'!C5:C11)</f>
         <v>361223.56</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="B48" s="8" t="n">
-        <f aca="false">B46-B47</f>
-        <v>-11927.56</v>
-      </c>
-      <c r="C48" s="18" t="n">
-        <f aca="false">IF(B47&gt;0,B48/B47,0)</f>
-        <v>-0.0330198838636107</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="B49" s="7" t="n">
-        <f aca="false">SUM('Mois par mois'!C6:C11)</f>
-        <v>312456.22</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="6" t="s">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="B50" s="8" t="n">
-        <f aca="false">B46-B49</f>
-        <v>36839.78</v>
-      </c>
-      <c r="C50" s="18" t="n">
-        <f aca="false">IF(B49&gt;0,B50/B49,0)</f>
-        <v>0.117903813852706</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
+      <c r="B51" s="8" t="n">
+        <f aca="false">B49-B50</f>
+        <v>-11927.55</v>
+      </c>
+      <c r="C51" s="18" t="n">
+        <f aca="false">IF(B50&gt;0,B51/B50,0)</f>
+        <v>-0.0330198561799236</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="B52" s="48" t="s">
+      <c r="D53" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="C52" s="48" t="s">
-        <v>206</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="G52" s="17" t="n">
+      <c r="G53" s="17" t="n">
         <v>5300</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="B53" s="17" t="n">
-        <v>-22600</v>
-      </c>
-      <c r="C53" s="8" t="n">
-        <f aca="false">B53</f>
-        <v>-22600</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="G53" s="47" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B54" s="17" t="n">
-        <v>-31800</v>
-      </c>
-      <c r="C54" s="8" t="n">
-        <f aca="false">-$G$52*$G$53</f>
-        <v>-26500</v>
+        <v>-22600</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G54" s="36" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="B55" s="17" t="n">
-        <v>-6200</v>
-      </c>
-      <c r="C55" s="8" t="n">
-        <f aca="false">B55</f>
-        <v>-6200</v>
+        <v>208</v>
+      </c>
+      <c r="B55" s="8" t="n">
+        <f aca="false">-$G$53*$G$54</f>
+        <v>-26500</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B56" s="17" t="n">
-        <v>25800</v>
-      </c>
-      <c r="C56" s="8" t="n">
-        <f aca="false">C35*$B$6</f>
-        <v>19397</v>
+        <v>-6200</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="B57" s="17" t="n">
-        <v>-13400</v>
-      </c>
-      <c r="C57" s="8" t="n">
-        <f aca="false">B57</f>
-        <v>-13400</v>
+        <v>210</v>
+      </c>
+      <c r="B57" s="8" t="n">
+        <f aca="false">B36*$B$9</f>
+        <v>19396.93</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="B58" s="17" t="n">
+        <v>-13400</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="B59" s="17" t="n">
+        <v>-11900</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="B60" s="20" t="n">
+        <f aca="false">SUM(B54:B59)</f>
+        <v>-61203.07</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="B58" s="17" t="n">
-        <v>-11900</v>
-      </c>
-      <c r="C58" s="8" t="n">
-        <f aca="false">B58</f>
-        <v>-11900</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="19" t="s">
+      <c r="B61" s="17" t="n">
+        <v>-59900</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="B59" s="20" t="n">
-        <f aca="false">SUM(B53:B58)</f>
-        <v>-60100</v>
-      </c>
-      <c r="C59" s="20" t="n">
-        <f aca="false">SUM(C53:C58)</f>
-        <v>-61203</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="B60" s="17" t="n">
-        <v>-59900</v>
-      </c>
-      <c r="C60" s="8" t="n">
-        <f aca="false">B60</f>
-        <v>-59900</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="3" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="35" t="s">
-        <v>218</v>
-      </c>
-      <c r="B63" s="35"/>
-      <c r="C63" s="35"/>
-      <c r="D63" s="35"/>
-      <c r="E63" s="35"/>
-      <c r="F63" s="35"/>
-      <c r="G63" s="35"/>
-      <c r="H63" s="35"/>
     </row>
     <row r="64" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="35" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B64" s="35"/>
       <c r="C64" s="35"/>
@@ -4653,10 +4793,12 @@
       <c r="F64" s="35"/>
       <c r="G64" s="35"/>
       <c r="H64" s="35"/>
+      <c r="I64" s="35"/>
+      <c r="J64" s="35"/>
     </row>
     <row r="65" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="35" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B65" s="35"/>
       <c r="C65" s="35"/>
@@ -4665,10 +4807,12 @@
       <c r="F65" s="35"/>
       <c r="G65" s="35"/>
       <c r="H65" s="35"/>
+      <c r="I65" s="35"/>
+      <c r="J65" s="35"/>
     </row>
     <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="35" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B66" s="35"/>
       <c r="C66" s="35"/>
@@ -4677,10 +4821,12 @@
       <c r="F66" s="35"/>
       <c r="G66" s="35"/>
       <c r="H66" s="35"/>
+      <c r="I66" s="35"/>
+      <c r="J66" s="35"/>
     </row>
     <row r="67" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="35" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B67" s="35"/>
       <c r="C67" s="35"/>
@@ -4689,14 +4835,30 @@
       <c r="F67" s="35"/>
       <c r="G67" s="35"/>
       <c r="H67" s="35"/>
+      <c r="I67" s="35"/>
+      <c r="J67" s="35"/>
+    </row>
+    <row r="68" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="35" t="s">
+        <v>220</v>
+      </c>
+      <c r="B68" s="35"/>
+      <c r="C68" s="35"/>
+      <c r="D68" s="35"/>
+      <c r="E68" s="35"/>
+      <c r="F68" s="35"/>
+      <c r="G68" s="35"/>
+      <c r="H68" s="35"/>
+      <c r="I68" s="35"/>
+      <c r="J68" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A63:H63"/>
-    <mergeCell ref="A64:H64"/>
-    <mergeCell ref="A65:H65"/>
-    <mergeCell ref="A66:H66"/>
-    <mergeCell ref="A67:H67"/>
+    <mergeCell ref="A64:J64"/>
+    <mergeCell ref="A65:J65"/>
+    <mergeCell ref="A66:J66"/>
+    <mergeCell ref="A67:J67"/>
+    <mergeCell ref="A68:J68"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4727,12 +4889,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4740,47 +4902,47 @@
         <v>115</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>170</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>170</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B5" s="7" t="n">
         <f aca="false">AVERAGE('Mois par mois'!C5:C11)</f>
         <v>51603.3657142857</v>
       </c>
       <c r="D5" s="7" t="n">
-        <f aca="false">'Compte d’exploitation'!C19</f>
-        <v>49899.4285714286</v>
+        <f aca="false">'Compte d’exploitation'!B20</f>
+        <v>49899.43</v>
       </c>
       <c r="F5" s="23" t="n">
         <f aca="false">D5-B5</f>
-        <v>-1703.93714285714</v>
+        <v>-1703.93571428571</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">SUMPRODUCT('Mois par mois'!C5:C11,'Mois par mois'!T5:T11)/7</f>
@@ -4791,24 +4953,24 @@
         <v>0.374197998657673</v>
       </c>
       <c r="D6" s="7" t="n">
-        <f aca="false">'Compte d’exploitation'!C20+'Compte d’exploitation'!C21</f>
-        <v>24906.8571428571</v>
+        <f aca="false">'Compte d’exploitation'!B21+'Compte d’exploitation'!B22</f>
+        <v>24906.86</v>
       </c>
       <c r="E6" s="18" t="n">
         <f aca="false">IF(D$5&gt;0,D6/D$5,0)</f>
-        <v>0.499141129586368</v>
+        <v>0.499141172554476</v>
       </c>
       <c r="F6" s="8" t="n">
         <f aca="false">D6-B6</f>
-        <v>5596.98096857143</v>
+        <v>5596.98382571429</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B5-B6</f>
@@ -4820,21 +4982,21 @@
       </c>
       <c r="D7" s="8" t="n">
         <f aca="false">D5-D6</f>
-        <v>24992.5714285714</v>
+        <v>24992.57</v>
       </c>
       <c r="E7" s="18" t="n">
         <f aca="false">IF(D$5&gt;0,D7/D$5,0)</f>
-        <v>0.500858870413632</v>
+        <v>0.500858827445524</v>
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">D7-B7</f>
-        <v>-7300.91811142857</v>
+        <v>-7300.91954</v>
       </c>
       <c r="G7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">AVERAGE('Mois par mois'!U5:U11)</f>
@@ -4845,19 +5007,19 @@
         <v>0.156963737359767</v>
       </c>
       <c r="D8" s="7" t="n">
-        <f aca="false">'Compte d’exploitation'!C23</f>
-        <v>8026.28571428572</v>
+        <f aca="false">'Compte d’exploitation'!B24</f>
+        <v>8026.29</v>
       </c>
       <c r="E8" s="18" t="n">
         <f aca="false">IF(D$5&gt;0,D8/D$5,0)</f>
-        <v>0.160849251064999</v>
+        <v>0.160849332347083</v>
       </c>
       <c r="F8" s="8" t="n">
         <f aca="false">D8-B8</f>
-        <v>-73.5714285714284</v>
+        <v>-73.5671428571432</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4873,24 +5035,24 @@
         <v>0.244415674326448</v>
       </c>
       <c r="D9" s="7" t="n">
-        <f aca="false">SUM('Compte d’exploitation'!C24:C34)</f>
-        <v>14195.2857142857</v>
+        <f aca="false">SUM('Compte d’exploitation'!B25:B35)</f>
+        <v>14195.29</v>
       </c>
       <c r="E9" s="18" t="n">
         <f aca="false">IF(D$5&gt;0,D9/D$5,0)</f>
-        <v>0.284477921304567</v>
+        <v>0.284477999047284</v>
       </c>
       <c r="F9" s="8" t="n">
         <f aca="false">D9-B9</f>
-        <v>1582.61428571429</v>
+        <v>1582.61857142857</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">B7-B8-B9</f>
@@ -4902,23 +5064,23 @@
       </c>
       <c r="D10" s="8" t="n">
         <f aca="false">D7-D8-D9</f>
-        <v>2771</v>
+        <v>2770.99</v>
       </c>
       <c r="E10" s="18" t="n">
         <f aca="false">IF(D$5&gt;0,D10/D$5,0)</f>
-        <v>0.0555316980440658</v>
+        <v>0.0555314960511573</v>
       </c>
       <c r="F10" s="23" t="n">
         <f aca="false">D10-B10</f>
-        <v>-8809.96096857143</v>
+        <v>-8809.97096857143</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B5&gt;0,(B8+B9)/(1-B6/B5),0)</f>
@@ -4926,19 +5088,19 @@
       </c>
       <c r="D11" s="8" t="n">
         <f aca="false">IF(D5&gt;0,(D8+D9)/(1-D6/D5),0)</f>
-        <v>44366.9319667232</v>
+        <v>44366.9528863738</v>
       </c>
       <c r="F11" s="8" t="n">
         <f aca="false">D11-B11</f>
-        <v>11269.3571315504</v>
+        <v>11269.378051201</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">AVERAGE('Mois par mois'!F5:F11)</f>
@@ -4947,7 +5109,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">IF(B12&gt;0,B5/B12,0)</f>
@@ -4956,12 +5118,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B10</f>
@@ -4970,47 +5132,47 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">D5-B5</f>
-        <v>-1703.93714285714</v>
+        <v>-1703.93571428571</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">-(D6-B6)</f>
-        <v>-5596.98096857143</v>
+        <v>-5596.98382571429</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-(D8-B8)</f>
-        <v>73.5714285714284</v>
+        <v>73.5671428571432</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">-(D9-B9)</f>
-        <v>-1582.61428571429</v>
+        <v>-1582.61857142857</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B21" s="20" t="n">
         <f aca="false">SUM(B16:B20)</f>
-        <v>2771</v>
+        <v>2770.99</v>
       </c>
       <c r="C21" s="2" t="str">
         <f aca="false">IF(ABS(B21-D10)&lt;1,"= bilan","écart")</f>
@@ -5045,28 +5207,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="B4" s="49" t="n">
+        <v>152</v>
+      </c>
+      <c r="B4" s="47" t="n">
         <f aca="false">Récap!B13</f>
         <v>30.4166666666667</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="F4" s="31" t="n">
-        <f aca="false">1-('Compte d’exploitation'!C20+'Compte d’exploitation'!C21)/'Compte d’exploitation'!C19</f>
-        <v>0.500858870413632</v>
+        <f aca="false">1-('Compte d’exploitation'!B21+'Compte d’exploitation'!B22)/'Compte d’exploitation'!B20</f>
+        <v>0.500858827445524</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5078,11 +5240,11 @@
         <v>12.1833302978178</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F5" s="7" t="n">
-        <f aca="false">'Compte d’exploitation'!C37</f>
-        <v>604.333333333334</v>
+        <f aca="false">'Compte d’exploitation'!B38</f>
+        <v>604.323333333331</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5094,16 +5256,16 @@
         <v>139.197183098592</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F6" s="7" t="n">
-        <f aca="false">'Compte d’exploitation'!C39</f>
-        <v>-2295.66666666667</v>
+        <f aca="false">'Compte d’exploitation'!B40</f>
+        <v>-2295.67666666667</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B7" s="31" t="n">
         <f aca="false">1-Récap!B31</f>
@@ -5112,7 +5274,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">Récap!B25</f>
@@ -5121,34 +5283,34 @@
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="H10" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="I10" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="J10" s="4" t="s">
         <v>261</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5185,11 +5347,11 @@
       </c>
       <c r="I11" s="23" t="n">
         <f aca="false">$F$5+H11</f>
-        <v>604.333333333334</v>
+        <v>604.323333333331</v>
       </c>
       <c r="J11" s="23" t="n">
         <f aca="false">$F$6+H11</f>
-        <v>-2295.66666666667</v>
+        <v>-2295.67666666667</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5222,15 +5384,15 @@
       </c>
       <c r="H12" s="8" t="n">
         <f aca="false">B12*$F$4</f>
-        <v>761.722865420732</v>
+        <v>761.722800073401</v>
       </c>
       <c r="I12" s="23" t="n">
         <f aca="false">$F$5+H12</f>
-        <v>1366.05619875407</v>
+        <v>1366.04613340673</v>
       </c>
       <c r="J12" s="23" t="n">
         <f aca="false">$F$6+H12</f>
-        <v>-1533.94380124593</v>
+        <v>-1533.95386659327</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5263,15 +5425,15 @@
       </c>
       <c r="H13" s="8" t="n">
         <f aca="false">B13*$F$4</f>
-        <v>1523.44573084146</v>
+        <v>1523.4456001468</v>
       </c>
       <c r="I13" s="23" t="n">
         <f aca="false">$F$5+H13</f>
-        <v>2127.7790641748</v>
+        <v>2127.76893348013</v>
       </c>
       <c r="J13" s="23" t="n">
         <f aca="false">$F$6+H13</f>
-        <v>-772.220935825202</v>
+        <v>-772.231066519867</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5304,15 +5466,15 @@
       </c>
       <c r="H14" s="8" t="n">
         <f aca="false">B14*$F$4</f>
-        <v>2285.1685962622</v>
+        <v>2285.1684002202</v>
       </c>
       <c r="I14" s="23" t="n">
         <f aca="false">$F$5+H14</f>
-        <v>2889.50192959553</v>
+        <v>2889.49173355353</v>
       </c>
       <c r="J14" s="23" t="n">
         <f aca="false">$F$6+H14</f>
-        <v>-10.4980704044706</v>
+        <v>-10.5082664464658</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5345,15 +5507,15 @@
       </c>
       <c r="H15" s="8" t="n">
         <f aca="false">B15*$F$4</f>
-        <v>3046.89146168293</v>
+        <v>3046.8912002936</v>
       </c>
       <c r="I15" s="23" t="n">
         <f aca="false">$F$5+H15</f>
-        <v>3651.22479501626</v>
+        <v>3651.21453362694</v>
       </c>
       <c r="J15" s="23" t="n">
         <f aca="false">$F$6+H15</f>
-        <v>751.224795016262</v>
+        <v>751.214533626936</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5386,20 +5548,20 @@
       </c>
       <c r="H16" s="8" t="n">
         <f aca="false">B16*$F$4</f>
-        <v>3808.61432710366</v>
+        <v>3808.61400036701</v>
       </c>
       <c r="I16" s="23" t="n">
         <f aca="false">$F$5+H16</f>
-        <v>4412.94766043699</v>
+        <v>4412.93733370034</v>
       </c>
       <c r="J16" s="23" t="n">
         <f aca="false">$F$6+H16</f>
-        <v>1512.94766043699</v>
+        <v>1512.93733370034</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tableau récap Halle : la section « À faire corriger par Pardoen » retirée (page 3 et feuille « Compte d'exploitation »)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfhpzegTMHxDopBcc2QwLH
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
+++ b/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="257">
   <si>
     <t xml:space="preserve">Atelier by – Halle · tableau récap</t>
   </si>
@@ -786,24 +786,6 @@
   </si>
   <si>
     <t xml:space="preserve">Perte de la situation au 30/09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À faire corriger par Pardoen avant de signer la situation et le PV d’AG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stock négatif (− 6 173 €) : impossible. Chaque millier d'euros de vrai stock en fin de période, c'est un millier d'euros de résultat en plus.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">« Formation pré et post ouverture » à − 31 000 € en actif : une immobilisation négative n'a pas de sens, probablement une note de crédit mal imputée.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mobilier en leasing (60,9 k€) jamais amorti : il manque environ 1 000 € d'amortissement par mois, le résultat réel est donc plus mauvais que celui affiché.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rémunération dirigeant à − 2 000 € (solde débiteur) : à expliquer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lignes à justifier une par une : « autres charges diverses » à 9 k€ (si ce sont bien les redevances, à 2,6 % du CA, les reclasser), containers 7,8 k€, secrétariat social 5,8 k€ (probablement Liantis de Nathan dedans), voiture 6,6 k€.</t>
   </si>
   <si>
     <t xml:space="preserve">L’application ou le bilan : mars → septembre 2026, en € par mois</t>
@@ -3522,7 +3504,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -4777,89 +4759,7 @@
         <v>-59900</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="3" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="35" t="s">
-        <v>216</v>
-      </c>
-      <c r="B64" s="35"/>
-      <c r="C64" s="35"/>
-      <c r="D64" s="35"/>
-      <c r="E64" s="35"/>
-      <c r="F64" s="35"/>
-      <c r="G64" s="35"/>
-      <c r="H64" s="35"/>
-      <c r="I64" s="35"/>
-      <c r="J64" s="35"/>
-    </row>
-    <row r="65" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="35" t="s">
-        <v>217</v>
-      </c>
-      <c r="B65" s="35"/>
-      <c r="C65" s="35"/>
-      <c r="D65" s="35"/>
-      <c r="E65" s="35"/>
-      <c r="F65" s="35"/>
-      <c r="G65" s="35"/>
-      <c r="H65" s="35"/>
-      <c r="I65" s="35"/>
-      <c r="J65" s="35"/>
-    </row>
-    <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="35" t="s">
-        <v>218</v>
-      </c>
-      <c r="B66" s="35"/>
-      <c r="C66" s="35"/>
-      <c r="D66" s="35"/>
-      <c r="E66" s="35"/>
-      <c r="F66" s="35"/>
-      <c r="G66" s="35"/>
-      <c r="H66" s="35"/>
-      <c r="I66" s="35"/>
-      <c r="J66" s="35"/>
-    </row>
-    <row r="67" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="35" t="s">
-        <v>219</v>
-      </c>
-      <c r="B67" s="35"/>
-      <c r="C67" s="35"/>
-      <c r="D67" s="35"/>
-      <c r="E67" s="35"/>
-      <c r="F67" s="35"/>
-      <c r="G67" s="35"/>
-      <c r="H67" s="35"/>
-      <c r="I67" s="35"/>
-      <c r="J67" s="35"/>
-    </row>
-    <row r="68" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="35" t="s">
-        <v>220</v>
-      </c>
-      <c r="B68" s="35"/>
-      <c r="C68" s="35"/>
-      <c r="D68" s="35"/>
-      <c r="E68" s="35"/>
-      <c r="F68" s="35"/>
-      <c r="G68" s="35"/>
-      <c r="H68" s="35"/>
-      <c r="I68" s="35"/>
-      <c r="J68" s="35"/>
-    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A64:J64"/>
-    <mergeCell ref="A65:J65"/>
-    <mergeCell ref="A66:J66"/>
-    <mergeCell ref="A67:J67"/>
-    <mergeCell ref="A68:J68"/>
-  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4889,12 +4789,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4902,22 +4802,22 @@
         <v>115</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>170</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>170</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4937,12 +4837,12 @@
         <v>-1703.93571428571</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">SUMPRODUCT('Mois par mois'!C5:C11,'Mois par mois'!T5:T11)/7</f>
@@ -4965,7 +4865,7 @@
         <v>5596.98382571429</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4996,7 +4896,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">AVERAGE('Mois par mois'!U5:U11)</f>
@@ -5019,7 +4919,7 @@
         <v>-73.5671428571432</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5047,12 +4947,12 @@
         <v>1582.61857142857</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">B7-B8-B9</f>
@@ -5075,12 +4975,12 @@
         <v>-8809.97096857143</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B5&gt;0,(B8+B9)/(1-B6/B5),0)</f>
@@ -5095,12 +4995,12 @@
         <v>11269.378051201</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">AVERAGE('Mois par mois'!F5:F11)</f>
@@ -5109,7 +5009,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">IF(B12&gt;0,B5/B12,0)</f>
@@ -5118,12 +5018,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B10</f>
@@ -5132,7 +5032,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">D5-B5</f>
@@ -5141,7 +5041,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">-(D6-B6)</f>
@@ -5150,7 +5050,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-(D8-B8)</f>
@@ -5159,7 +5059,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">-(D9-B9)</f>
@@ -5168,7 +5068,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="B21" s="20" t="n">
         <f aca="false">SUM(B16:B20)</f>
@@ -5207,12 +5107,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5224,7 +5124,7 @@
         <v>30.4166666666667</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="F4" s="31" t="n">
         <f aca="false">1-('Compte d’exploitation'!B21+'Compte d’exploitation'!B22)/'Compte d’exploitation'!B20</f>
@@ -5240,7 +5140,7 @@
         <v>12.1833302978178</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">'Compte d’exploitation'!B38</f>
@@ -5256,7 +5156,7 @@
         <v>139.197183098592</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">'Compte d’exploitation'!B40</f>
@@ -5265,7 +5165,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="B7" s="31" t="n">
         <f aca="false">1-Récap!B31</f>
@@ -5274,7 +5174,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">Récap!B25</f>
@@ -5283,34 +5183,34 @@
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>195</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="I10" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="J10" s="4" t="s">
         <v>255</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5561,7 +5461,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tableau récap Halle : plan achats réduit à B1 (prix) et B2 (commandes sur les ventes réelles) ; sorties tracées et audit des fournitures retirés
Achats à 42,4 % du CA au lieu de 48,3 %, + 4 420 € de marge par mois. Titre « Réduire les achats » ; l'indicateur du lundi ne cite plus que B2. Dans l'Excel, les paramètres B3 et B4 sortent de la feuille « Compte d'exploitation ».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfhpzegTMHxDopBcc2QwLH
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
+++ b/docs/dossiers/halle-recap-2026-10/Halle-tableau-recap.xlsx
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="253">
   <si>
     <t xml:space="preserve">Atelier by – Halle · tableau récap</t>
   </si>
@@ -620,18 +620,6 @@
     <t xml:space="preserve">Commandes sur ventes réelles (B2), % des achats</t>
   </si>
   <si>
-    <t xml:space="preserve">Sorties tracées (B3), % des achats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Achats fournitures sur la période</t>
-  </si>
-  <si>
-    <t xml:space="preserve">total de la période</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audit fournitures (B4), % de la ligne</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hausse de CA du scénario</t>
   </si>
   <si>
@@ -659,7 +647,7 @@
     <t xml:space="preserve">CA pour le résultat visé</t>
   </si>
   <si>
-    <t xml:space="preserve">Plan matière (B1 → B4)</t>
+    <t xml:space="preserve">Plan achats (B1 + B2)</t>
   </si>
   <si>
     <t xml:space="preserve">+ 15 % de CA, matière 40 %</t>
@@ -3612,55 +3600,26 @@
         <v>159</v>
       </c>
       <c r="B12" s="27" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="C12" s="2"/>
+        <v>0.15</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="B13" s="17" t="n">
-        <v>19500</v>
+        <v>161</v>
+      </c>
+      <c r="B13" s="27" t="n">
+        <v>0.4</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
         <v>162</v>
-      </c>
-      <c r="B14" s="27" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="B15" s="27" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="B16" s="27" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D18" s="14" t="n">
         <v>0</v>
@@ -3674,39 +3633,39 @@
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="H19" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="I19" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>173</v>
-      </c>
       <c r="J19" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B20" s="17" t="n">
         <v>49899.43</v>
@@ -3736,7 +3695,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="23" t="n">
-        <f aca="false">B20*(1+$B$15)</f>
+        <f aca="false">B20*(1+$B$12)</f>
         <v>57384.3445</v>
       </c>
       <c r="J20" s="24" t="n">
@@ -3746,7 +3705,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B21" s="17" t="n">
         <v>24123.43</v>
@@ -3768,15 +3727,15 @@
         <v>35991.513009109</v>
       </c>
       <c r="G21" s="8" t="n">
-        <f aca="false">B21*(1-$B$11-$B$12)-$B$13/$B$9*$B$14</f>
-        <v>20253.6184</v>
+        <f aca="false">B21*(1-$B$11)</f>
+        <v>22193.5556</v>
       </c>
       <c r="H21" s="18" t="n">
         <f aca="false">IF(G$20&lt;&gt;0,G21/G$20,0)</f>
-        <v>0.386560735883203</v>
+        <v>0.423586394053953</v>
       </c>
       <c r="I21" s="8" t="n">
-        <f aca="false">I20*$B$16</f>
+        <f aca="false">I20*$B$13</f>
         <v>22953.7378</v>
       </c>
       <c r="J21" s="18" t="n">
@@ -3786,7 +3745,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B22" s="17" t="n">
         <v>783.43</v>
@@ -3826,7 +3785,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B23" s="20" t="n">
         <f aca="false">B20-B21-B22</f>
@@ -3850,11 +3809,11 @@
       </c>
       <c r="G23" s="20" t="n">
         <f aca="false">G20-G21-G22</f>
-        <v>31357.3531</v>
+        <v>29417.4159</v>
       </c>
       <c r="H23" s="24" t="n">
         <f aca="false">IF(G$20&lt;&gt;0,G23/G$20,0)</f>
-        <v>0.598486712363725</v>
+        <v>0.561461054192975</v>
       </c>
       <c r="I23" s="20" t="n">
         <f aca="false">I20-I21-I22</f>
@@ -3867,7 +3826,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B24" s="17" t="n">
         <v>8026.29</v>
@@ -3907,7 +3866,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B25" s="17" t="n">
         <v>4862</v>
@@ -3947,7 +3906,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B26" s="17" t="n">
         <v>1297.71</v>
@@ -3987,7 +3946,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B27" s="17" t="n">
         <v>1294.29</v>
@@ -4027,7 +3986,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B28" s="17" t="n">
         <v>1493</v>
@@ -4067,7 +4026,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B29" s="17" t="n">
         <v>1110</v>
@@ -4107,7 +4066,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B30" s="17" t="n">
         <v>946.29</v>
@@ -4147,7 +4106,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B31" s="17" t="n">
         <v>866.57</v>
@@ -4187,7 +4146,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B32" s="17" t="n">
         <v>666.86</v>
@@ -4227,7 +4186,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B33" s="17" t="n">
         <v>632.57</v>
@@ -4267,7 +4226,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B34" s="17" t="n">
         <v>587.14</v>
@@ -4307,7 +4266,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B35" s="17" t="n">
         <v>438.86</v>
@@ -4347,7 +4306,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B36" s="20" t="n">
         <f aca="false">B23-SUM(B24:B35)</f>
@@ -4371,11 +4330,11 @@
       </c>
       <c r="G36" s="20" t="n">
         <f aca="false">G23-SUM(G24:G35)</f>
-        <v>9135.7731</v>
+        <v>7195.8359</v>
       </c>
       <c r="H36" s="24" t="n">
         <f aca="false">IF(G$20&lt;&gt;0,G36/G$20,0)</f>
-        <v>0.17436544436909</v>
+        <v>0.13733978619834</v>
       </c>
       <c r="I36" s="20" t="n">
         <f aca="false">I23-SUM(I24:I35)</f>
@@ -4388,7 +4347,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B37" s="8" t="n">
         <f aca="false">-$B$5*$B$7</f>
@@ -4429,7 +4388,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="22" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B38" s="23" t="n">
         <f aca="false">B36+B37</f>
@@ -4453,11 +4412,11 @@
       </c>
       <c r="G38" s="23" t="n">
         <f aca="false">G36+G37</f>
-        <v>6969.10643333333</v>
+        <v>5029.16923333333</v>
       </c>
       <c r="H38" s="24" t="n">
         <f aca="false">IF(G$20&lt;&gt;0,G38/G$20,0)</f>
-        <v>0.133012425637371</v>
+        <v>0.095986767466622</v>
       </c>
       <c r="I38" s="23" t="n">
         <f aca="false">I36+I37</f>
@@ -4470,7 +4429,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B39" s="8" t="n">
         <f aca="false">-$B$6</f>
@@ -4511,7 +4470,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B40" s="20" t="n">
         <f aca="false">B38+B39</f>
@@ -4535,11 +4494,11 @@
       </c>
       <c r="G40" s="20" t="n">
         <f aca="false">G38+G39</f>
-        <v>4069.10643333333</v>
+        <v>2129.16923333333</v>
       </c>
       <c r="H40" s="24" t="n">
         <f aca="false">IF(G$20&lt;&gt;0,G40/G$20,0)</f>
-        <v>0.077663000565687</v>
+        <v>0.0406373423949376</v>
       </c>
       <c r="I40" s="20" t="n">
         <f aca="false">I38+I39</f>
@@ -4552,7 +4511,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="D41" s="8" t="n">
         <f aca="false">D20-$B$20</f>
@@ -4577,7 +4536,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D42" s="8" t="n">
         <f aca="false">D41/$B$8</f>
@@ -4602,7 +4561,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="28" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B44" s="32" t="n">
         <f aca="false">IF(B20&gt;0,(SUM(B24:B35)-B37)/(1-(B21+B22)/B20),0)</f>
@@ -4610,7 +4569,7 @@
       </c>
       <c r="G44" s="32" t="n">
         <f aca="false">IF(G20&gt;0,(SUM(G24:G35)-G37)/(1-(G21+G22)/G20),0)</f>
-        <v>40749.8548636865</v>
+        <v>43437.1119502162</v>
       </c>
       <c r="I44" s="32" t="n">
         <f aca="false">IF(I20&gt;0,(SUM(I24:I35)-I37)/(1-(I21+I22)/I20),0)</f>
@@ -4619,7 +4578,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="28" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B45" s="32" t="n">
         <f aca="false">IF(B20&gt;0,(SUM(B24:B35)-B37-B39)/(1-(B21+B22)/B20),0)</f>
@@ -4627,7 +4586,7 @@
       </c>
       <c r="G45" s="32" t="n">
         <f aca="false">IF(G20&gt;0,(SUM(G24:G35)-G37-G39)/(1-(G21+G22)/G20),0)</f>
-        <v>45595.4093932874</v>
+        <v>48602.2075135556</v>
       </c>
       <c r="I45" s="32" t="n">
         <f aca="false">IF(I20&gt;0,(SUM(I24:I35)-I37-I39)/(1-(I21+I22)/I20),0)</f>
@@ -4636,17 +4595,17 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B49" s="8" t="n">
         <f aca="false">B20*$B$9</f>
@@ -4655,7 +4614,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B50" s="7" t="n">
         <f aca="false">SUM('Mois par mois'!C5:C11)</f>
@@ -4664,7 +4623,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B51" s="8" t="n">
         <f aca="false">B49-B50</f>
@@ -4677,10 +4636,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="G53" s="17" t="n">
         <v>5300</v>
@@ -4688,13 +4647,13 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B54" s="17" t="n">
         <v>-22600</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="G54" s="36" t="n">
         <v>5</v>
@@ -4702,7 +4661,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B55" s="8" t="n">
         <f aca="false">-$G$53*$G$54</f>
@@ -4711,7 +4670,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="B56" s="17" t="n">
         <v>-6200</v>
@@ -4719,7 +4678,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B57" s="8" t="n">
         <f aca="false">B36*$B$9</f>
@@ -4728,7 +4687,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B58" s="17" t="n">
         <v>-13400</v>
@@ -4736,7 +4695,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B59" s="17" t="n">
         <v>-11900</v>
@@ -4744,7 +4703,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="19" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B60" s="20" t="n">
         <f aca="false">SUM(B54:B59)</f>
@@ -4753,7 +4712,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="B61" s="17" t="n">
         <v>-59900</v>
@@ -4789,12 +4748,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4802,27 +4761,27 @@
         <v>115</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B5" s="7" t="n">
         <f aca="false">AVERAGE('Mois par mois'!C5:C11)</f>
@@ -4837,12 +4796,12 @@
         <v>-1703.93571428571</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">SUMPRODUCT('Mois par mois'!C5:C11,'Mois par mois'!T5:T11)/7</f>
@@ -4865,12 +4824,12 @@
         <v>5596.98382571429</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B5-B6</f>
@@ -4896,7 +4855,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">AVERAGE('Mois par mois'!U5:U11)</f>
@@ -4919,7 +4878,7 @@
         <v>-73.5671428571432</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4947,12 +4906,12 @@
         <v>1582.61857142857</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">B7-B8-B9</f>
@@ -4975,12 +4934,12 @@
         <v>-8809.97096857143</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B5&gt;0,(B8+B9)/(1-B6/B5),0)</f>
@@ -4995,12 +4954,12 @@
         <v>11269.378051201</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">AVERAGE('Mois par mois'!F5:F11)</f>
@@ -5009,7 +4968,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">IF(B12&gt;0,B5/B12,0)</f>
@@ -5018,12 +4977,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B10</f>
@@ -5032,7 +4991,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">D5-B5</f>
@@ -5041,7 +5000,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">-(D6-B6)</f>
@@ -5050,7 +5009,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">-(D8-B8)</f>
@@ -5059,7 +5018,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">-(D9-B9)</f>
@@ -5068,7 +5027,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B21" s="20" t="n">
         <f aca="false">SUM(B16:B20)</f>
@@ -5107,12 +5066,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5124,7 +5083,7 @@
         <v>30.4166666666667</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="F4" s="31" t="n">
         <f aca="false">1-('Compte d’exploitation'!B21+'Compte d’exploitation'!B22)/'Compte d’exploitation'!B20</f>
@@ -5140,7 +5099,7 @@
         <v>12.1833302978178</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">'Compte d’exploitation'!B38</f>
@@ -5156,7 +5115,7 @@
         <v>139.197183098592</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">'Compte d’exploitation'!B40</f>
@@ -5165,7 +5124,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="B7" s="31" t="n">
         <f aca="false">1-Récap!B31</f>
@@ -5174,7 +5133,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">Récap!B25</f>
@@ -5183,34 +5142,34 @@
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="H10" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="I10" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="J10" s="4" t="s">
         <v>251</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5461,7 +5420,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>